<commit_message>
feat(sys): add organization data foundation
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Rd09f965c24d64d03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R28130cf33b0441f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R9da22aab04474969"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Rd96187b01b2b4156"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Raa216fbb0c0d4389"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R27fe8f4fb1384399"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R696fb43c99fc4f86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R50903c79698a49d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rfeef86984d0240f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Rabe41bf7717f4e80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Rda7c6f4a20184ffe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Re16b5cd029b34b05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R72c46644c32d4bbd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R453413c11d6c490b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R9282c6cf18324053"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R077f9d7df3654734"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R1941daa04f184713"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R3156f4f4a97941f0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -63,12 +63,12 @@
   <x:cols>
     <x:col min="1" max="1" width="16" customWidth="1"/>
     <x:col min="2" max="2" width="10" customWidth="1"/>
-    <x:col min="3" max="3" width="14" customWidth="1"/>
+    <x:col min="3" max="3" width="23" customWidth="1"/>
     <x:col min="4" max="4" width="10" customWidth="1"/>
-    <x:col min="5" max="5" width="13" customWidth="1"/>
-    <x:col min="6" max="6" width="10" customWidth="1"/>
-    <x:col min="7" max="7" width="21" customWidth="1"/>
-    <x:col min="8" max="8" width="10" customWidth="1"/>
+    <x:col min="5" max="5" width="60" customWidth="1"/>
+    <x:col min="6" max="6" width="11" customWidth="1"/>
+    <x:col min="7" max="7" width="30" customWidth="1"/>
+    <x:col min="8" max="8" width="40" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -110,6 +110,426 @@
       <x:c r="H1" s="1" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Source</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.20.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B2" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C2" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Company Management</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D2" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E2" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to view company details.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F2" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G2" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">僅有組織檢視權的用戶可見其獲授權公司；無權限回 403。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H2" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:13</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.20.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B3" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C3" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Company Management</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D3" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E3" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to create a company.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F3" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G3" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">代碼全系統唯一；代碼與名稱必填；重複代碼回 409。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H3" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:14</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.20.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B4" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C4" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Company Management</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D4" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E4" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to edit a company.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F4" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G4" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">版本不符回 409；審計欄位記錄修改者。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H4" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:15</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.20.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B5" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C5" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Company Management</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D5" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E5" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to deactivate a company.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F5" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G5" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">停用後不能成為新操作的公司上下文；歷史資料保留。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H5" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:16</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.21.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B6" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C6" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Branch Management</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D6" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E6" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to view branches in the selected company.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F6" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G6" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">公司 A 的查詢不返回公司 B 分店；未選公司結果為空。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H6" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:17</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.21.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B7" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C7" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Branch Management</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D7" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E7" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to create a branch.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F7" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G7" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">公司內代碼唯一；所屬公司必須為授權公司。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H7" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:18</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.21.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B8" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C8" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Branch Management</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D8" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E8" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to edit or deactivate a branch.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F8" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G8" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">版本不符回 409；被引用時只可停用，不得刪除。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H8" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:19</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.22.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B9" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C9" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Department Management</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D9" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E9" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to view departments in the selected company.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F9" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G9" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">公司隔離、軟刪除篩選生效。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H9" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:20</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.22.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B10" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C10" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Department Management</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D10" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E10" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to create a department under a branch or parent department.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F10" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G10" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">分店與上級部門必須屬於同一公司；不得循環參照。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H10" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:21</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.22.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B11" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C11" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Department Management</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D11" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E11" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to edit or deactivate a department.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F11" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G11" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">版本不符回 409；被引用時只可停用。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H11" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:22</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1054,10 +1474,10 @@
   <x:cols>
     <x:col min="1" max="1" width="16" customWidth="1"/>
     <x:col min="2" max="2" width="10" customWidth="1"/>
-    <x:col min="3" max="3" width="12" customWidth="1"/>
-    <x:col min="4" max="4" width="13" customWidth="1"/>
-    <x:col min="5" max="5" width="10" customWidth="1"/>
-    <x:col min="6" max="6" width="15" customWidth="1"/>
+    <x:col min="3" max="3" width="16" customWidth="1"/>
+    <x:col min="4" max="4" width="60" customWidth="1"/>
+    <x:col min="5" max="5" width="11" customWidth="1"/>
+    <x:col min="6" max="6" width="60" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -1089,6 +1509,102 @@
       <x:c r="F1" s="1" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Related REQ_F</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.20</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B2" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C2" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">sys_company</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D2" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Company isolation root; globally unique code, audit, version and soft deletion.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E2" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F2" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.20.1, REQ_F4118.20.2, REQ_F4118.20.3, REQ_F4118.20.4</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.22</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B3" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C3" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">sys_department</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D3" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Department master scoped to a company, optionally linked to a branch and parent department.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E3" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F3" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.22.1, REQ_F4118.22.2, REQ_F4118.22.3</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.89</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B4" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C4" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">sys_branch</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D4" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Branch master scoped to a company.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E4" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F4" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.21.1, REQ_F4118.21.2, REQ_F4118.21.3</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1101,15 +1617,15 @@
   <x:cols>
     <x:col min="1" max="1" width="16" customWidth="1"/>
     <x:col min="2" max="2" width="15" customWidth="1"/>
-    <x:col min="3" max="3" width="11" customWidth="1"/>
-    <x:col min="4" max="4" width="10" customWidth="1"/>
+    <x:col min="3" max="3" width="27" customWidth="1"/>
+    <x:col min="4" max="4" width="30" customWidth="1"/>
     <x:col min="5" max="5" width="13" customWidth="1"/>
     <x:col min="6" max="6" width="10" customWidth="1"/>
-    <x:col min="7" max="7" width="10" customWidth="1"/>
+    <x:col min="7" max="7" width="15" customWidth="1"/>
     <x:col min="8" max="8" width="13" customWidth="1"/>
     <x:col min="9" max="9" width="13" customWidth="1"/>
     <x:col min="10" max="10" width="10" customWidth="1"/>
-    <x:col min="11" max="11" width="10" customWidth="1"/>
+    <x:col min="11" max="11" width="11" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -1166,6 +1682,291 @@
       <x:c r="K1" s="1" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Author</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.58.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B2" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.58</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C2" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Company View Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D2" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Company Code (Input)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E2" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">公司代碼</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F2" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">唯一識別公司</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G2" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">VARCHAR(30)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H2" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1–30 字元</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I2" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J2" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K2" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.58.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B3" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.58</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C3" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Company View Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D3" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Company Name (Input)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E3" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">公司名稱</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F3" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">顯示公司</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G3" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">NVARCHAR(200)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H3" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1–200 字元</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I3" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J3" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K3" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.59.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B4" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.59</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C4" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Branch View Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D4" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Branch Code (Input)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E4" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">分店代碼</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F4" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">公司內唯一</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G4" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">VARCHAR(30)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H4" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1–30 字元</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I4" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J4" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K4" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.60.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B5" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.60</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C5" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Department View Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D5" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Department Code (Input)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E5" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">部門代碼</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F5" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">公司內唯一</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G5" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">VARCHAR(30)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H5" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1–30 字元</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I5" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J5" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K5" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.60.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B6" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.60</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C6" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Department View Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D6" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Parent Department (Dropdown)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E6" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">上級部門</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F6" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">建立層級</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G6" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">bigint ID</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H6" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">同公司啟用部門</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I6" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J6" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K6" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1176,12 +1977,12 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:cols>
-    <x:col min="1" max="1" width="10" customWidth="1"/>
-    <x:col min="2" max="2" width="13" customWidth="1"/>
-    <x:col min="3" max="3" width="10" customWidth="1"/>
+    <x:col min="1" max="1" width="16" customWidth="1"/>
+    <x:col min="2" max="2" width="60" customWidth="1"/>
+    <x:col min="3" max="3" width="13" customWidth="1"/>
     <x:col min="4" max="4" width="12" customWidth="1"/>
-    <x:col min="5" max="5" width="10" customWidth="1"/>
-    <x:col min="6" max="6" width="12" customWidth="1"/>
+    <x:col min="5" max="5" width="32" customWidth="1"/>
+    <x:col min="6" max="6" width="26" customWidth="1"/>
     <x:col min="7" max="7" width="10" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -1219,6 +2020,376 @@
       <x:c r="G1" s="1" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Coverage</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.20.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B2" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to view company details.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C2" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.20</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D2" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.58</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E2" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F2" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-ORG-004</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G2" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.20.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B3" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to create a company.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C3" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.20</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D3" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.58</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E3" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.58.1, REQ_IO_A8.58.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F3" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-ORG-001</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G3" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.20.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B4" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to edit a company.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C4" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.20</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D4" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.58</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E4" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F4" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-ORG-005</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G4" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.20.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B5" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to deactivate a company.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C5" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.20</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D5" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.58</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E5" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F5" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-ORG-006</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G5" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.21.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B6" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to view branches in the selected company.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C6" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.89</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D6" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.59</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E6" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F6" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-ORG-002, SYS-ORG-004</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G6" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.21.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B7" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to create a branch.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C7" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.89</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D7" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.59</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E7" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.59.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F7" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-ORG-001</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G7" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.21.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B8" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to edit or deactivate a branch.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C8" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.89</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D8" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.59</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E8" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F8" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-ORG-005</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G8" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.22.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B9" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to view departments in the selected company.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C9" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.22</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D9" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.60</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E9" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F9" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-ORG-002, SYS-ORG-004</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G9" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.22.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B10" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to create a department under a branch or parent department.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C10" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.22</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D10" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.60</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E10" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.60.1, REQ_IO_A8.60.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F10" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-ORG-001, SYS-ORG-003</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G10" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.22.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B11" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to edit or deactivate a department.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C11" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.22</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D11" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.60</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E11" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F11" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-ORG-005</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G11" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -13809,7 +14980,7 @@
       </x:c>
       <x:c r="F393" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">未開始</x:t>
+          <x:t xml:space="preserve">進行中</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -13873,7 +15044,7 @@
       </x:c>
       <x:c r="F395" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">未開始</x:t>
+          <x:t xml:space="preserve">進行中</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
feat(sys): add internal organization validation service
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Rabe41bf7717f4e80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Rda7c6f4a20184ffe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Re16b5cd029b34b05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R72c46644c32d4bbd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R453413c11d6c490b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R9282c6cf18324053"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R077f9d7df3654734"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R1941daa04f184713"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R3156f4f4a97941f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Rdd614df01d7d4a44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Re9c235f08b0c4022"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R6d55872db3594456"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Rf8e9e8ce6f984042"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R6c9ba592a7fd4426"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="Rf75afa7538134e01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R751f0b4a99a24030"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R4145721c8f8542ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rbf5dd080ea04421f"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
feat(sys): extend organization services and validation
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Rdd614df01d7d4a44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Re9c235f08b0c4022"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R6d55872db3594456"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Rf8e9e8ce6f984042"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R6c9ba592a7fd4426"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="Rf75afa7538134e01"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R751f0b4a99a24030"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R4145721c8f8542ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rbf5dd080ea04421f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Rad2996fbb9bd4b97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R2ab50b8a7b04476e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R4df1fc8b47744252"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R1e6cb695ed564486"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Ra918025d32194f1a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R4d38344d879b407f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Rfebf2755ab0b44ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="Rdb7cabb89e384a72"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R319c32e0245a4886"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -67,7 +67,7 @@
     <x:col min="4" max="4" width="10" customWidth="1"/>
     <x:col min="5" max="5" width="60" customWidth="1"/>
     <x:col min="6" max="6" width="11" customWidth="1"/>
-    <x:col min="7" max="7" width="30" customWidth="1"/>
+    <x:col min="7" max="7" width="60" customWidth="1"/>
     <x:col min="8" max="8" width="40" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -173,7 +173,7 @@
       </x:c>
       <x:c r="D3" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">1.0</x:t>
+          <x:t xml:space="preserve">1.1</x:t>
         </x:is>
       </x:c>
       <x:c r="E3" s="2" t="inlineStr">
@@ -188,7 +188,7 @@
       </x:c>
       <x:c r="G3" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">代碼全系統唯一；代碼與名稱必填；重複代碼回 409。</x:t>
+          <x:t xml:space="preserve">代碼全系統唯一；代碼與名稱必填；代碼限 1–30 字元的 ASCII 英文、數字、-、_，保存為大寫；重複代碼回 409。</x:t>
         </x:is>
       </x:c>
       <x:c r="H3" s="2" t="inlineStr">
@@ -1622,7 +1622,7 @@
     <x:col min="5" max="5" width="13" customWidth="1"/>
     <x:col min="6" max="6" width="10" customWidth="1"/>
     <x:col min="7" max="7" width="15" customWidth="1"/>
-    <x:col min="8" max="8" width="13" customWidth="1"/>
+    <x:col min="8" max="8" width="25" customWidth="1"/>
     <x:col min="9" max="9" width="13" customWidth="1"/>
     <x:col min="10" max="10" width="10" customWidth="1"/>
     <x:col min="11" max="11" width="11" customWidth="1"/>
@@ -1723,7 +1723,7 @@
       </x:c>
       <x:c r="H2" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">1–30 字元</x:t>
+          <x:t xml:space="preserve">1–30 字元；ASCII 英文、數字、-、_</x:t>
         </x:is>
       </x:c>
       <x:c r="I2" s="2" t="inlineStr">
@@ -1837,7 +1837,7 @@
       </x:c>
       <x:c r="H4" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">1–30 字元</x:t>
+          <x:t xml:space="preserve">1–30 字元；ASCII 英文、數字、-、_</x:t>
         </x:is>
       </x:c>
       <x:c r="I4" s="2" t="inlineStr">
@@ -1894,7 +1894,7 @@
       </x:c>
       <x:c r="H5" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">1–30 字元</x:t>
+          <x:t xml:space="preserve">1–30 字元；ASCII 英文、數字、-、_</x:t>
         </x:is>
       </x:c>
       <x:c r="I5" s="2" t="inlineStr">
@@ -2088,7 +2088,7 @@
       </x:c>
       <x:c r="F3" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-ORG-001</x:t>
+          <x:t xml:space="preserve">SYS-ORG-001, SYS-ORG-008</x:t>
         </x:is>
       </x:c>
       <x:c r="G3" s="2" t="inlineStr">
@@ -2384,7 +2384,7 @@
       </x:c>
       <x:c r="F11" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-ORG-005</x:t>
+          <x:t xml:space="preserve">SYS-ORG-005, SYS-ORG-007</x:t>
         </x:is>
       </x:c>
       <x:c r="G11" s="2" t="inlineStr">

</xml_diff>

<commit_message>
test(sys): cover organization constraints and concurrency
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Rad2996fbb9bd4b97"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R2ab50b8a7b04476e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R4df1fc8b47744252"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R1e6cb695ed564486"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Ra918025d32194f1a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R4d38344d879b407f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Rfebf2755ab0b44ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="Rdb7cabb89e384a72"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R319c32e0245a4886"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R4b87c127ccb54bf2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R98f00317b5264425"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Rd991c3fa4a9546a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Rac418e4833f54dea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R1f0272cbc1b94f8a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="Rf1123e791a1f41c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R50e16f7e0cee4e65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R1f4569a1d65b4ed0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rf35e4ffe47cb4d27"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1982,7 +1982,7 @@
     <x:col min="3" max="3" width="13" customWidth="1"/>
     <x:col min="4" max="4" width="12" customWidth="1"/>
     <x:col min="5" max="5" width="32" customWidth="1"/>
-    <x:col min="6" max="6" width="26" customWidth="1"/>
+    <x:col min="6" max="6" width="39" customWidth="1"/>
     <x:col min="7" max="7" width="10" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -2125,7 +2125,7 @@
       </x:c>
       <x:c r="F4" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-ORG-005</x:t>
+          <x:t xml:space="preserve">SYS-ORG-005, SYS-ORG-009</x:t>
         </x:is>
       </x:c>
       <x:c r="G4" s="2" t="inlineStr">
@@ -2384,7 +2384,7 @@
       </x:c>
       <x:c r="F11" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-ORG-005, SYS-ORG-007</x:t>
+          <x:t xml:space="preserve">SYS-ORG-005, SYS-ORG-007, SYS-ORG-009</x:t>
         </x:is>
       </x:c>
       <x:c r="G11" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat(sys): add scoped organization list queries
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R4b87c127ccb54bf2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R98f00317b5264425"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Rd991c3fa4a9546a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Rac418e4833f54dea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R1f0272cbc1b94f8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="Rf1123e791a1f41c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R50e16f7e0cee4e65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R1f4569a1d65b4ed0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rf35e4ffe47cb4d27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R82bc1c13e09f4220"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R74bd908d2ee04eeb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Rfdcc198f541a4440"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Ra7619d5ac1d545dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Ra65783d7eaf64abf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R19e42c6601e84ac3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R5645b1bfd4364302"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="Rfc6a47f45613498c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rffb445f68d244ffc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2199,7 +2199,7 @@
       </x:c>
       <x:c r="F6" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-ORG-002, SYS-ORG-004</x:t>
+          <x:t xml:space="preserve">SYS-ORG-002, SYS-ORG-004, SYS-ORG-010</x:t>
         </x:is>
       </x:c>
       <x:c r="G6" s="2" t="inlineStr">
@@ -2310,7 +2310,7 @@
       </x:c>
       <x:c r="F9" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-ORG-002, SYS-ORG-004</x:t>
+          <x:t xml:space="preserve">SYS-ORG-002, SYS-ORG-004, SYS-ORG-010</x:t>
         </x:is>
       </x:c>
       <x:c r="G9" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat(sys): scope internal company list to authorized IDs
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R82bc1c13e09f4220"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R74bd908d2ee04eeb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Rfdcc198f541a4440"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Ra7619d5ac1d545dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Ra65783d7eaf64abf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R19e42c6601e84ac3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R5645b1bfd4364302"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="Rfc6a47f45613498c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rffb445f68d244ffc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Ra51adb1daf904a50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R0cddb00515a44043"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Rf2859e0b88d04c87"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Rf23a59a7ccb64ea2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Rf3cfc594c28a456b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="Rb565557bcd424ac9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R67e9d84ffbdd4858"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="Ra4fe6b12631647be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rcdd6c3b925ac4be5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -131,7 +131,7 @@
       </x:c>
       <x:c r="D2" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">1.0</x:t>
+          <x:t xml:space="preserve">1.1</x:t>
         </x:is>
       </x:c>
       <x:c r="E2" s="2" t="inlineStr">
@@ -146,7 +146,7 @@
       </x:c>
       <x:c r="G2" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">僅有組織檢視權的用戶可見其獲授權公司；無權限回 403。</x:t>
+          <x:t xml:space="preserve">僅有組織檢視權的用戶可見其獲授權且啟用、未刪除的公司；列表支援分頁、關鍵字及代碼／名稱排序；無權限回 403。</x:t>
         </x:is>
       </x:c>
       <x:c r="H2" s="2" t="inlineStr">
@@ -2051,7 +2051,7 @@
       </x:c>
       <x:c r="F2" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-ORG-004</x:t>
+          <x:t xml:space="preserve">SYS-ORG-004, SYS-ORG-011</x:t>
         </x:is>
       </x:c>
       <x:c r="G2" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat(sys): add roles, permission codes, company access check and data scope
- sys_role, sys_role_permission, sys_user_company, sys_user_role (System_Authorization)
- [RequirePermission] dynamic policies, CompanyAccessMiddleware, 403 error codes
- role CRUD, permission catalog, user-company assignment, current authorization API
- DataScopeFilter for application queries; architecture test for action permissions
- frontend PermissionService, *erpHasPermission, permissionGuard, menu filtering
- ADR-014; fix docgen errors in SYS ui-spec and test-plan

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Ra51adb1daf904a50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R0cddb00515a44043"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Rf2859e0b88d04c87"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Rf23a59a7ccb64ea2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Rf3cfc594c28a456b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="Rb565557bcd424ac9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R67e9d84ffbdd4858"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="Ra4fe6b12631647be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rcdd6c3b925ac4be5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R68f985d6ab084dc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R9b21d50f44664792"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R9bed53bdb2054ef4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Rf77c3ba0cad442f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Rf3b9eca1f5ca490c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="Rdc29fceb741e4333"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R27f3c71e4ba84941"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="Rdfb6975c28c64c16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R9f8187bea4f34786"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -63,7 +63,7 @@
   <x:cols>
     <x:col min="1" max="1" width="16" customWidth="1"/>
     <x:col min="2" max="2" width="10" customWidth="1"/>
-    <x:col min="3" max="3" width="23" customWidth="1"/>
+    <x:col min="3" max="3" width="37" customWidth="1"/>
     <x:col min="4" max="4" width="10" customWidth="1"/>
     <x:col min="5" max="5" width="60" customWidth="1"/>
     <x:col min="6" max="6" width="11" customWidth="1"/>
@@ -530,6 +530,678 @@
       <x:c r="H11" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:22</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.23.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B12" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C12" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">User Identity and Password Security</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D12" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E12" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to create a unique user identity.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F12" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G12" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">帳號不分大小寫唯一，停用及軟刪除後仍不可重用；僅保存雜湊，不保存明文密碼。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H12" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:38</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.23.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B13" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C13" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">User Identity and Password Security</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D13" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E13" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enforce a configurable password policy.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F13" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G13" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">預設 12–128 字元且含大小寫、數字及符號；長度、複雜度與到期天數可由設定調整，不合法設定拒絕啟動。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H13" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:39</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.23.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">User Identity and Password Security</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should lock an account after five consecutive failed password attempts.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">第 5 次連續失敗鎖定 15 分鐘；鎖定期間正確密碼亦不得通過；鎖定到期後開啟新失敗計數窗口，成功後清除計數。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:40</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.23.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B15" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C15" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">User Identity and Password Security</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D15" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E15" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should determine whether a user's password has expired.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F15" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G15" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">依設定天數及 password_changed_at 判斷；0 代表不設到期。登入簽發 Token 前必須檢查。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H15" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:41</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.24.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B16" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C16" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Login, Token and Captcha</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D16" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E16" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow a user to log in with username, password and a numeric captcha.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F16" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G16" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">帳號不分大小寫；Captcha 4–6 位數字，答案只存伺服器端，驗證一次即作廢（不論對錯）；帳密錯誤、帳號不存在、停用或鎖定一律回 401 SYS.AUTH.INVALID_CREDENTIALS；密碼到期回 403 SYS.AUTH.PASSWORD_EXPIRED 且不發 Token。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H16" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:53</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.24.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B17" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C17" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Login, Token and Captcha</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D17" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E17" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should issue a 15-minute access token and a 7-day rotating refresh token.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F17" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G17" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Access Token 為 HS256 JWT，sub 為用戶 Id；Refresh Token 只以 SHA-256 雜湊存 Redis，使用一次即輪替，並發重放只有一個成功。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H17" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:54</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.24.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B18" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C18" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Login, Token and Captcha</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D18" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E18" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow a logged-in user to log out and invalidate the refresh token.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F18" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G18" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">登出須帶有效 Access Token；只撤銷屬於本人的 Refresh Token，撤銷後刷新回 401。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H18" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:55</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.24.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B19" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C19" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Login, Token and Captcha</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D19" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E19" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should provide a development-only captcha master code with startup protection.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F19" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G19" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Captcha:MasterCode 只在 Development 生效且須為 4–6 位數字；其他環境有設定即寫 Error 並拒絕啟動；每次使用寫 Warning（帳號、IP），稽核日誌於 WU-SYS-007 補上。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H19" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:56</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.24.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B20" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C20" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Login, Token and Captcha</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D20" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E20" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should provide a trilingual login page that keeps the session and refreshes tokens automatically.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F20" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G20" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">未登入進入主框架導向 /login?returnUrl=…，登入後只回到站內路徑；Captcha 元件只收 4–6 位數字，失敗後換新圖並清空密碼；錯誤依 errorCode 三語顯示；API 請求帶 Bearer，401 時只刷新一次並重送，並發 401 共用同一 refresh；刷新失敗清除 Session 回登入頁；登出撤銷 Refresh Token，伺服器失敗也清除本機 Session。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H20" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:57</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.25.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B21" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C21" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Role, Permission and Data Scope</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D21" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E21" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to view roles and the permission catalog.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F21" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G21" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">需 SYS.ROLE.VIEW；角色列表支援分頁、關鍵字（代碼／名稱）、code／name 排序；權限目錄列出各模組宣告的全部代碼；已軟刪除角色不顯示，查詢回 404。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H21" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:69</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.25.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B22" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C22" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Role, Permission and Data Scope</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D22" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E22" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to create a role with permissions and a data scope.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F22" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G22" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">需 SYS.ROLE.CREATE；代碼 1–50 字元 ASCII 英文、數字、-、_，保存為大寫，全系統唯一（含已刪除），重複回 409 SYS.ROLE.DUPLICATE_CODE；權限代碼不分大小寫輸入，必須在權限目錄內，否則 400；資料範圍為 Self／Department／Branch／Company。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H22" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:70</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.25.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B23" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C23" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Role, Permission and Data Scope</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D23" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E23" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to edit or deactivate a role.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F23" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G23" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">需 SYS.ROLE.EDIT；帶 version，不符回 409，且權限集合不變（同一交易）；停用角色立即不再授予權限。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H23" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:71</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.25.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B24" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C24" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Role, Permission and Data Scope</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D24" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E24" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to delete an unused role.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F24" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G24" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">需 SYS.ROLE.DELETE；仍有用戶使用回 422 SYS.ROLE.IN_USE；軟刪除，代碼不可重用。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H24" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:72</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.25.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B25" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C25" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Role, Permission and Data Scope</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D25" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E25" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enforce permission codes on every API with the backend as the authority.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F25" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G25" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">每個 API 動作標註 模組.資源.動作 權限（ArchitectureTests 檢查）；未登入 401；缺權限或沒有公司上下文 403 COMMON.PERMISSION.DENIED；已登入請求的 X-Company-Id 不可存取（未授權、用戶公司關聯停用、公司停用）一律 403 COMMON.COMPANY.ACCESS_DENIED。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H25" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:73</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.25.6</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B26" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C26" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Role, Permission and Data Scope</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D26" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E26" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to grant a user access to a company with roles, organization and default company.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F26" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G26" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">需 SYS.USER.EDIT；公司必須啟用；分店／部門必須屬於該公司且啟用；角色必須存在且啟用；角色整組取代；每位用戶最多一間預設公司（設定新預設會取消舊預設）。用戶不存在回 404。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H26" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:74</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.25.7</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Role, Permission and Data Scope</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should resolve the user's effective permissions and data scope per company and hide unauthorized UI.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">同一權限取各啟用角色最寬的資料範圍；全權角色視為全部權限、全公司範圍；分店／部門範圍但用戶無對應歸屬時退回本人。GET /api/v1/sys/auth/authorization 回傳可存取公司（預設在前）與目前公司權限；前端 *erpHasPermission、permissionGuard 與選單依此隱藏，切換公司重新載入；本機記住的公司不可存取時改用預設公司。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:75</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1474,7 +2146,7 @@
   <x:cols>
     <x:col min="1" max="1" width="16" customWidth="1"/>
     <x:col min="2" max="2" width="10" customWidth="1"/>
-    <x:col min="3" max="3" width="16" customWidth="1"/>
+    <x:col min="3" max="3" width="21" customWidth="1"/>
     <x:col min="4" max="4" width="60" customWidth="1"/>
     <x:col min="5" max="5" width="11" customWidth="1"/>
     <x:col min="6" max="6" width="60" customWidth="1"/>
@@ -1579,32 +2251,192 @@
     <x:row r="4">
       <x:c r="A4" s="2" t="inlineStr">
         <x:is>
+          <x:t xml:space="preserve">REQ_DS43.82</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B4" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C4" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">sys_user</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D4" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Global login identities with password hash, failure count, lockout and audit fields.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E4" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F4" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.23.1, REQ_F4118.23.2, REQ_F4118.23.3, REQ_F4118.23.4</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="2" t="inlineStr">
+        <x:is>
           <x:t xml:space="preserve">REQ_DS43.89</x:t>
         </x:is>
       </x:c>
-      <x:c r="B4" s="2" t="inlineStr">
+      <x:c r="B5" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">1.0</x:t>
         </x:is>
       </x:c>
-      <x:c r="C4" s="2" t="inlineStr">
+      <x:c r="C5" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">sys_branch</x:t>
         </x:is>
       </x:c>
-      <x:c r="D4" s="2" t="inlineStr">
+      <x:c r="D5" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Branch master scoped to a company.</x:t>
         </x:is>
       </x:c>
-      <x:c r="E4" s="2" t="inlineStr">
+      <x:c r="E5" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Developer</x:t>
         </x:is>
       </x:c>
-      <x:c r="F4" s="2" t="inlineStr">
+      <x:c r="F5" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">REQ_F4118.21.1, REQ_F4118.21.2, REQ_F4118.21.3</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.90</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B6" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C6" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">sys_role</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D6" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System-wide role definitions with data scope, full-access flag, audit, version and soft deletion.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E6" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F6" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.25.1, REQ_F4118.25.2, REQ_F4118.25.3, REQ_F4118.25.4</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.91</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B7" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C7" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">sys_role_permission</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D7" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Permission codes granted by each role.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E7" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F7" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.25.2, REQ_F4118.25.3, REQ_F4118.25.7</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.92</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B8" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C8" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">sys_user_company</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D8" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Companies a user may access, with branch and department placement and the default company.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E8" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F8" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.25.5, REQ_F4118.25.6, REQ_F4118.25.7</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.93</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B9" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C9" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">sys_user_role</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D9" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Roles assigned to a user within a company.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E9" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F9" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.25.6, REQ_F4118.25.7</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1617,13 +2449,13 @@
   <x:cols>
     <x:col min="1" max="1" width="16" customWidth="1"/>
     <x:col min="2" max="2" width="15" customWidth="1"/>
-    <x:col min="3" max="3" width="27" customWidth="1"/>
+    <x:col min="3" max="3" width="32" customWidth="1"/>
     <x:col min="4" max="4" width="30" customWidth="1"/>
     <x:col min="5" max="5" width="13" customWidth="1"/>
-    <x:col min="6" max="6" width="10" customWidth="1"/>
-    <x:col min="7" max="7" width="15" customWidth="1"/>
-    <x:col min="8" max="8" width="25" customWidth="1"/>
-    <x:col min="9" max="9" width="13" customWidth="1"/>
+    <x:col min="6" max="6" width="23" customWidth="1"/>
+    <x:col min="7" max="7" width="40" customWidth="1"/>
+    <x:col min="8" max="8" width="60" customWidth="1"/>
+    <x:col min="9" max="9" width="16" customWidth="1"/>
     <x:col min="10" max="10" width="10" customWidth="1"/>
     <x:col min="11" max="11" width="11" customWidth="1"/>
   </x:cols>
@@ -1965,6 +2797,462 @@
         </x:is>
       </x:c>
       <x:c r="K6" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.61.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B7" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.61</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C7" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">User Identity Create Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D7" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Username (Input)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E7" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">帳號</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F7" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">建立登入身分</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G7" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">ASCII text</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H7" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">3–100 字元，字母／數字／點／底線／連字號</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I7" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J7" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K7" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.61.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B8" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.61</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C8" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">User Identity Create Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D8" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Password (Input)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E8" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">初始密碼</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F8" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">依目前政策驗證，提交後清空</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G8" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Password text</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H8" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">預設 12–128 字元</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I8" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J8" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K8" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.62.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B9" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.62</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C9" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Login Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D9" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Username (Input)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E9" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">帳號</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F9" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">登入身分</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G9" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Text，autocomplete=username</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H9" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">必填、非空白，最多 100 字元；送出前去除前後空白</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I9" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J9" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K9" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.62.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B10" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.62</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C10" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Login Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D10" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Password (Input)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E10" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">密碼</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F10" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">驗證身分</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G10" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Password，autocomplete=current-password</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H10" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">必填，最多 128 字元；失敗後清空</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I10" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J10" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K10" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.62.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B11" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.62</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C11" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Login Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D11" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Captcha Code (Input)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E11" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">驗證碼</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F11" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">防自動化登入</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G11" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">數字，inputmode=numeric</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H11" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4–6 位數字（非數字自動移除）</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I11" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.62.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J11" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K11" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.62.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B12" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.62</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C12" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Login Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D12" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Captcha Image (Button)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E12" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">驗證碼圖片</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F12" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">顯示題目，點擊換圖</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G12" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SVG data URI</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H12" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">每次送出失敗後自動換新</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I12" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J12" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K12" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.62.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B13" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.62</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C13" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Login Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D13" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Sign In (Button)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E13" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">登入</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F13" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">送出</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G13" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Button</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H13" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">送出中顯示載入狀態，不可重複送出</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I13" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J13" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K13" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.62.6</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.62</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Login Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Error Message (Alert)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">錯誤訊息</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">顯示 errors.&lt;errorCode&gt;</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Text</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">INVALID_CREDENTIALS／CAPTCHA_INVALID／PASSWORD_EXPIRED／VALIDATION_FAILED／網路／未知</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K14" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Developer</x:t>
         </x:is>
@@ -1979,10 +3267,10 @@
   <x:cols>
     <x:col min="1" max="1" width="16" customWidth="1"/>
     <x:col min="2" max="2" width="60" customWidth="1"/>
-    <x:col min="3" max="3" width="13" customWidth="1"/>
+    <x:col min="3" max="3" width="39" customWidth="1"/>
     <x:col min="4" max="4" width="12" customWidth="1"/>
-    <x:col min="5" max="5" width="32" customWidth="1"/>
-    <x:col min="6" max="6" width="39" customWidth="1"/>
+    <x:col min="5" max="5" width="60" customWidth="1"/>
+    <x:col min="6" max="6" width="60" customWidth="1"/>
     <x:col min="7" max="7" width="10" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -2051,7 +3339,7 @@
       </x:c>
       <x:c r="F2" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-ORG-004, SYS-ORG-011</x:t>
+          <x:t xml:space="preserve">SYS-ORG-004, SYS-ORG-011, SYS-ORG-012</x:t>
         </x:is>
       </x:c>
       <x:c r="G2" s="2" t="inlineStr">
@@ -2088,7 +3376,7 @@
       </x:c>
       <x:c r="F3" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-ORG-001, SYS-ORG-008</x:t>
+          <x:t xml:space="preserve">SYS-ORG-001, SYS-ORG-008, SYS-ORG-013</x:t>
         </x:is>
       </x:c>
       <x:c r="G3" s="2" t="inlineStr">
@@ -2199,7 +3487,7 @@
       </x:c>
       <x:c r="F6" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-ORG-002, SYS-ORG-004, SYS-ORG-010</x:t>
+          <x:t xml:space="preserve">SYS-ORG-002, SYS-ORG-004, SYS-ORG-010, SYS-ORG-012</x:t>
         </x:is>
       </x:c>
       <x:c r="G6" s="2" t="inlineStr">
@@ -2236,7 +3524,7 @@
       </x:c>
       <x:c r="F7" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-ORG-001</x:t>
+          <x:t xml:space="preserve">SYS-ORG-001, SYS-ORG-013</x:t>
         </x:is>
       </x:c>
       <x:c r="G7" s="2" t="inlineStr">
@@ -2310,7 +3598,7 @@
       </x:c>
       <x:c r="F9" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-ORG-002, SYS-ORG-004, SYS-ORG-010</x:t>
+          <x:t xml:space="preserve">SYS-ORG-002, SYS-ORG-004, SYS-ORG-010, SYS-ORG-012</x:t>
         </x:is>
       </x:c>
       <x:c r="G9" s="2" t="inlineStr">
@@ -2347,7 +3635,7 @@
       </x:c>
       <x:c r="F10" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-ORG-001, SYS-ORG-003</x:t>
+          <x:t xml:space="preserve">SYS-ORG-001, SYS-ORG-003, SYS-ORG-013</x:t>
         </x:is>
       </x:c>
       <x:c r="G10" s="2" t="inlineStr">
@@ -2390,6 +3678,598 @@
       <x:c r="G11" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.23.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B12" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to create a unique user identity.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C12" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.82</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D12" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.61</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E12" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.61.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F12" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-USER-001, SYS-USER-004, SYS-USER-006</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G12" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.23.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B13" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enforce a configurable password policy.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C13" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.82</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D13" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.61</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E13" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.61.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F13" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-USER-001, SYS-USER-007, SYS-USER-006</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G13" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.23.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should lock an account after five consecutive failed password attempts.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.82</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-USER-002, SYS-USER-003, SYS-USER-005, SYS-USER-006</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.23.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B15" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should determine whether a user's password has expired.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C15" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.82</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D15" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E15" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F15" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-USER-003, SYS-USER-006</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G15" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.24.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B16" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow a user to log in with username, password and a numeric captcha.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C16" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="D16" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.62</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E16" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.62.1, REQ_IO_A8.62.2, REQ_IO_A8.62.3, REQ_IO_A8.62.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F16" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-AUTH-001, SYS-AUTH-002, SYS-AUTH-005, SYS-AUTH-006, SYS-AUTH-009, SYS-AUTH-014, SYS-AUTH-015, SYS-AUTH-016, SYS-AUTH-017</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G16" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.24.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B17" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should issue a 15-minute access token and a 7-day rotating refresh token.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C17" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="D17" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E17" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F17" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-AUTH-001, SYS-AUTH-004, SYS-AUTH-007, SYS-AUTH-009, SYS-AUTH-010, SYS-AUTH-016, SYS-AUTH-017</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G17" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.24.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B18" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow a logged-in user to log out and invalidate the refresh token.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C18" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="D18" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E18" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F18" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-AUTH-008, SYS-AUTH-016, SYS-AUTH-017</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G18" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.24.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B19" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should provide a development-only captcha master code with startup protection.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C19" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="D19" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E19" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F19" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-AUTH-003, SYS-AUTH-004, SYS-AUTH-016, SYS-AUTH-017</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G19" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.24.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B20" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should provide a trilingual login page that keeps the session and refreshes tokens automatically.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C20" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="D20" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.62</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E20" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.62.5, REQ_IO_A8.62.6</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F20" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-AUTH-011, SYS-AUTH-012, SYS-AUTH-013, SYS-AUTH-015, SYS-AUTH-016, SYS-AUTH-017</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G20" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.25.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B21" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to view roles and the permission catalog.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C21" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.90</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D21" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E21" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F21" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-PERM-004, SYS-PERM-011, SYS-PERM-024</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G21" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.25.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B22" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to create a role with permissions and a data scope.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C22" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.90, REQ_DS43.91</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D22" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E22" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F22" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-PERM-011, SYS-PERM-024</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G22" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.25.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B23" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to edit or deactivate a role.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C23" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.90, REQ_DS43.91</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D23" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E23" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F23" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-PERM-011, SYS-PERM-024</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G23" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.25.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B24" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to delete an unused role.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C24" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.90</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D24" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E24" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F24" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-PERM-012, SYS-PERM-024</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G24" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.25.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B25" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enforce permission codes on every API with the backend as the authority.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C25" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.92</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D25" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E25" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F25" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-PERM-001, SYS-PERM-005, SYS-PERM-006, SYS-PERM-010</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G25" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.25.6</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B26" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to grant a user access to a company with roles, organization and default company.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C26" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.92, REQ_DS43.93</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D26" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E26" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F26" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-PERM-015, SYS-PERM-016, SYS-PERM-024</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G26" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.25.7</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should resolve the user's effective permissions and data scope per company and hide unauthorized UI.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.91, REQ_DS43.92, REQ_DS43.93</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-PERM-002, SYS-PERM-003, SYS-PERM-013, SYS-PERM-014, SYS-PERM-020, SYS-PERM-021, SYS-PERM-022, SYS-PERM-023</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -16964,7 +18844,7 @@
       </x:c>
       <x:c r="F455" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">未開始</x:t>
+          <x:t xml:space="preserve">進行中</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
feat(sys): complete WU-SYS-001 organization work unit
Extract PagedResultMapping, add ADR-015 (organization API scope and
creator grant), update SYS requirements/api/ui/test-plan docs and
regenerate SRS/SDS. Backend 414/414, frontend 285/285, E2E 28/28.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R68f985d6ab084dc8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R9b21d50f44664792"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R9bed53bdb2054ef4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Rf77c3ba0cad442f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Rf3b9eca1f5ca490c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="Rdc29fceb741e4333"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R27f3c71e4ba84941"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="Rdfb6975c28c64c16"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R9f8187bea4f34786"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R2563ce78a73b4d8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Ra52784bd7a284867"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R26d4540427c148b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R94a762b990774f90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Rbea054a32ced4542"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R4a2eba0f67f94d2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R0653581235d14cea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R3f2eab2c30a84330"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R3940f2ef141e41bb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -131,7 +131,7 @@
       </x:c>
       <x:c r="D2" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">1.1</x:t>
+          <x:t xml:space="preserve">1.2</x:t>
         </x:is>
       </x:c>
       <x:c r="E2" s="2" t="inlineStr">
@@ -146,7 +146,7 @@
       </x:c>
       <x:c r="G2" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">僅有組織檢視權的用戶可見其獲授權且啟用、未刪除的公司；列表支援分頁、關鍵字及代碼／名稱排序；無權限回 403。</x:t>
+          <x:t xml:space="preserve">僅有組織檢視權的用戶可見其獲授權且未刪除的公司；預設只列啟用公司，勾選「顯示已停用」時一併列出停用公司；列表支援分頁、關鍵字及代碼／名稱排序；無權限回 403。</x:t>
         </x:is>
       </x:c>
       <x:c r="H2" s="2" t="inlineStr">
@@ -173,7 +173,7 @@
       </x:c>
       <x:c r="D3" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">1.1</x:t>
+          <x:t xml:space="preserve">1.2</x:t>
         </x:is>
       </x:c>
       <x:c r="E3" s="2" t="inlineStr">
@@ -188,7 +188,7 @@
       </x:c>
       <x:c r="G3" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">代碼全系統唯一；代碼與名稱必填；代碼限 1–30 字元的 ASCII 英文、數字、-、_，保存為大寫；重複代碼回 409。</x:t>
+          <x:t xml:space="preserve">代碼全系統唯一；代碼與名稱必填；代碼限 1–30 字元的 ASCII 英文、數字、-、_，保存為大寫；重複代碼回 409；建立者在同一交易內獲授權新公司，角色沿用其在目前公司的角色（ADR-015）。</x:t>
         </x:is>
       </x:c>
       <x:c r="H3" s="2" t="inlineStr">
@@ -215,7 +215,7 @@
       </x:c>
       <x:c r="D4" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">1.0</x:t>
+          <x:t xml:space="preserve">1.1</x:t>
         </x:is>
       </x:c>
       <x:c r="E4" s="2" t="inlineStr">
@@ -230,7 +230,7 @@
       </x:c>
       <x:c r="G4" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">版本不符回 409；審計欄位記錄修改者。</x:t>
+          <x:t xml:space="preserve">版本不符回 409；審計欄位記錄修改者；目標公司不是用戶獲授權的公司時回 404。</x:t>
         </x:is>
       </x:c>
       <x:c r="H4" s="2" t="inlineStr">
@@ -571,7 +571,7 @@
       </x:c>
       <x:c r="H12" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:38</x:t>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:40</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -613,7 +613,7 @@
       </x:c>
       <x:c r="H13" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:39</x:t>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:41</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -655,7 +655,7 @@
       </x:c>
       <x:c r="H14" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:40</x:t>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:42</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -697,7 +697,7 @@
       </x:c>
       <x:c r="H15" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:41</x:t>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:43</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -739,7 +739,7 @@
       </x:c>
       <x:c r="H16" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:53</x:t>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:55</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -781,7 +781,7 @@
       </x:c>
       <x:c r="H17" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:54</x:t>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:56</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -823,7 +823,7 @@
       </x:c>
       <x:c r="H18" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:55</x:t>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:57</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -865,7 +865,7 @@
       </x:c>
       <x:c r="H19" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:56</x:t>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:58</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -907,7 +907,7 @@
       </x:c>
       <x:c r="H20" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:57</x:t>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:59</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -949,7 +949,7 @@
       </x:c>
       <x:c r="H21" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:69</x:t>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:71</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -991,7 +991,7 @@
       </x:c>
       <x:c r="H22" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:70</x:t>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:72</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1033,7 +1033,7 @@
       </x:c>
       <x:c r="H23" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:71</x:t>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:73</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1075,7 +1075,7 @@
       </x:c>
       <x:c r="H24" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:72</x:t>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:74</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1117,7 +1117,7 @@
       </x:c>
       <x:c r="H25" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:73</x:t>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:75</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1159,7 +1159,7 @@
       </x:c>
       <x:c r="H26" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:74</x:t>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:76</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1201,7 +1201,7 @@
       </x:c>
       <x:c r="H27" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:75</x:t>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:77</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -3339,7 +3339,7 @@
       </x:c>
       <x:c r="F2" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-ORG-004, SYS-ORG-011, SYS-ORG-012</x:t>
+          <x:t xml:space="preserve">SYS-ORG-004, SYS-ORG-011, SYS-ORG-012, SYS-ORG-020, SYS-ORG-026</x:t>
         </x:is>
       </x:c>
       <x:c r="G2" s="2" t="inlineStr">
@@ -3376,7 +3376,7 @@
       </x:c>
       <x:c r="F3" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-ORG-001, SYS-ORG-008, SYS-ORG-013</x:t>
+          <x:t xml:space="preserve">SYS-ORG-001, SYS-ORG-008, SYS-ORG-013, SYS-ORG-021</x:t>
         </x:is>
       </x:c>
       <x:c r="G3" s="2" t="inlineStr">
@@ -3413,7 +3413,7 @@
       </x:c>
       <x:c r="F4" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-ORG-005, SYS-ORG-009</x:t>
+          <x:t xml:space="preserve">SYS-ORG-005, SYS-ORG-009, SYS-ORG-013, SYS-ORG-021</x:t>
         </x:is>
       </x:c>
       <x:c r="G4" s="2" t="inlineStr">
@@ -3450,7 +3450,7 @@
       </x:c>
       <x:c r="F5" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-ORG-006</x:t>
+          <x:t xml:space="preserve">SYS-ORG-006, SYS-ORG-021</x:t>
         </x:is>
       </x:c>
       <x:c r="G5" s="2" t="inlineStr">
@@ -3487,7 +3487,7 @@
       </x:c>
       <x:c r="F6" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-ORG-002, SYS-ORG-004, SYS-ORG-010, SYS-ORG-012</x:t>
+          <x:t xml:space="preserve">SYS-ORG-002, SYS-ORG-004, SYS-ORG-010, SYS-ORG-012, SYS-ORG-020, SYS-ORG-022, SYS-ORG-024, SYS-ORG-025</x:t>
         </x:is>
       </x:c>
       <x:c r="G6" s="2" t="inlineStr">
@@ -3524,7 +3524,7 @@
       </x:c>
       <x:c r="F7" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-ORG-001, SYS-ORG-013</x:t>
+          <x:t xml:space="preserve">SYS-ORG-001, SYS-ORG-013, SYS-ORG-020, SYS-ORG-022, SYS-ORG-024</x:t>
         </x:is>
       </x:c>
       <x:c r="G7" s="2" t="inlineStr">
@@ -3561,7 +3561,7 @@
       </x:c>
       <x:c r="F8" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-ORG-005</x:t>
+          <x:t xml:space="preserve">SYS-ORG-005, SYS-ORG-022</x:t>
         </x:is>
       </x:c>
       <x:c r="G8" s="2" t="inlineStr">
@@ -3598,7 +3598,7 @@
       </x:c>
       <x:c r="F9" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-ORG-002, SYS-ORG-004, SYS-ORG-010, SYS-ORG-012</x:t>
+          <x:t xml:space="preserve">SYS-ORG-002, SYS-ORG-004, SYS-ORG-010, SYS-ORG-012, SYS-ORG-020, SYS-ORG-023, SYS-ORG-026</x:t>
         </x:is>
       </x:c>
       <x:c r="G9" s="2" t="inlineStr">
@@ -3635,7 +3635,7 @@
       </x:c>
       <x:c r="F10" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-ORG-001, SYS-ORG-003, SYS-ORG-013</x:t>
+          <x:t xml:space="preserve">SYS-ORG-001, SYS-ORG-003, SYS-ORG-013, SYS-ORG-023</x:t>
         </x:is>
       </x:c>
       <x:c r="G10" s="2" t="inlineStr">
@@ -3672,7 +3672,7 @@
       </x:c>
       <x:c r="F11" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-ORG-005, SYS-ORG-007, SYS-ORG-009</x:t>
+          <x:t xml:space="preserve">SYS-ORG-005, SYS-ORG-007, SYS-ORG-009, SYS-ORG-023, SYS-ORG-026</x:t>
         </x:is>
       </x:c>
       <x:c r="G11" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat(sys): add trilingual user maintenance page
Complete WU-SYS-002 with the /sys/users page (interfaces 8.61, 8.63):
server-side paging, username search and sort, status/lock/expiry tags,
create and reset-password dialog with confirmation, activate/deactivate
and unlock, all gated by SYS.USER.* permissions with trilingual errors.
Adds 10 frontend unit tests and 5 Playwright specs, and fills the
REQ_F4118.23.5-8 data-structure trace gap.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R2563ce78a73b4d8c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Ra52784bd7a284867"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R26d4540427c148b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R94a762b990774f90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Rbea054a32ced4542"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R4a2eba0f67f94d2f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R0653581235d14cea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R3f2eab2c30a84330"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R3940f2ef141e41bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R23b7dea85ff1444a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R54dee6920b864470"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R6389d2a2b1af49b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Ra10c7500e3ab4d9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R0d010cc04a25480c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="Reb09fd7f186f4200"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R31275a1f3f7f48a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R22dc2e391ce54910"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rdeff01a5e27d4fc9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -704,7 +704,7 @@
     <x:row r="16">
       <x:c r="A16" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.24.1</x:t>
+          <x:t xml:space="preserve">REQ_F4118.23.5</x:t>
         </x:is>
       </x:c>
       <x:c r="B16" s="2" t="inlineStr">
@@ -714,7 +714,7 @@
       </x:c>
       <x:c r="C16" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Login, Token and Captcha</x:t>
+          <x:t xml:space="preserve">User Identity and Password Security</x:t>
         </x:is>
       </x:c>
       <x:c r="D16" s="2" t="inlineStr">
@@ -724,7 +724,7 @@
       </x:c>
       <x:c r="E16" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">System should allow a user to log in with username, password and a numeric captcha.</x:t>
+          <x:t xml:space="preserve">System should list the users of the current company with paging, keyword and sorting.</x:t>
         </x:is>
       </x:c>
       <x:c r="F16" s="2" t="inlineStr">
@@ -734,19 +734,19 @@
       </x:c>
       <x:c r="G16" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">帳號不分大小寫；Captcha 4–6 位數字，答案只存伺服器端，驗證一次即作廢（不論對錯）；帳密錯誤、帳號不存在、停用或鎖定一律回 401 SYS.AUTH.INVALID_CREDENTIALS；密碼到期回 403 SYS.AUTH.PASSWORD_EXPIRED 且不發 Token。</x:t>
+          <x:t xml:space="preserve">只列在目前公司有用戶公司關聯的用戶（含停用）；關鍵字不分大小寫比對帳號；排序 username／-username，其他欄位 400；回應不含雜湊、失敗次數及鎖定期限，只回 isLocked、isPasswordExpired（ADR-016）。</x:t>
         </x:is>
       </x:c>
       <x:c r="H16" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:55</x:t>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:44</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.24.2</x:t>
+          <x:t xml:space="preserve">REQ_F4118.23.6</x:t>
         </x:is>
       </x:c>
       <x:c r="B17" s="2" t="inlineStr">
@@ -756,7 +756,7 @@
       </x:c>
       <x:c r="C17" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Login, Token and Captcha</x:t>
+          <x:t xml:space="preserve">User Identity and Password Security</x:t>
         </x:is>
       </x:c>
       <x:c r="D17" s="2" t="inlineStr">
@@ -766,7 +766,7 @@
       </x:c>
       <x:c r="E17" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">System should issue a 15-minute access token and a 7-day rotating refresh token.</x:t>
+          <x:t xml:space="preserve">System should allow authorized users to create a user in the current company.</x:t>
         </x:is>
       </x:c>
       <x:c r="F17" s="2" t="inlineStr">
@@ -776,19 +776,19 @@
       </x:c>
       <x:c r="G17" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Access Token 為 HS256 JWT，sub 為用戶 Id；Refresh Token 只以 SHA-256 雜湊存 Redis，使用一次即輪替，並發重放只有一個成功。</x:t>
+          <x:t xml:space="preserve">需 SYS.USER.CREATE；同一交易建立身分及目前公司的預設關聯（無角色）；重複帳號（不分大小寫、含他公司）409 SYS.USER.DUPLICATE；弱密碼或帳號格式錯誤 400；建立後可登入。</x:t>
         </x:is>
       </x:c>
       <x:c r="H17" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:56</x:t>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:45</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.24.3</x:t>
+          <x:t xml:space="preserve">REQ_F4118.23.7</x:t>
         </x:is>
       </x:c>
       <x:c r="B18" s="2" t="inlineStr">
@@ -798,7 +798,7 @@
       </x:c>
       <x:c r="C18" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Login, Token and Captcha</x:t>
+          <x:t xml:space="preserve">User Identity and Password Security</x:t>
         </x:is>
       </x:c>
       <x:c r="D18" s="2" t="inlineStr">
@@ -808,7 +808,7 @@
       </x:c>
       <x:c r="E18" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">System should allow a logged-in user to log out and invalidate the refresh token.</x:t>
+          <x:t xml:space="preserve">System should allow authorized users to activate or deactivate a user.</x:t>
         </x:is>
       </x:c>
       <x:c r="F18" s="2" t="inlineStr">
@@ -818,19 +818,19 @@
       </x:c>
       <x:c r="G18" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">登出須帶有效 Access Token；只撤銷屬於本人的 Refresh Token，撤銷後刷新回 401。</x:t>
+          <x:t xml:space="preserve">需 SYS.USER.EDIT 並帶 version（過期 409）；停用後不可登入與刷新，重新啟用後可登入；不可停用自己 422 SYS.USER.SELF_DEACTIVATION；他公司用戶 404。</x:t>
         </x:is>
       </x:c>
       <x:c r="H18" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:57</x:t>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:46</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.24.4</x:t>
+          <x:t xml:space="preserve">REQ_F4118.23.8</x:t>
         </x:is>
       </x:c>
       <x:c r="B19" s="2" t="inlineStr">
@@ -840,7 +840,7 @@
       </x:c>
       <x:c r="C19" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Login, Token and Captcha</x:t>
+          <x:t xml:space="preserve">User Identity and Password Security</x:t>
         </x:is>
       </x:c>
       <x:c r="D19" s="2" t="inlineStr">
@@ -850,7 +850,7 @@
       </x:c>
       <x:c r="E19" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">System should provide a development-only captcha master code with startup protection.</x:t>
+          <x:t xml:space="preserve">System should allow authorized users to reset a password and unlock a locked user.</x:t>
         </x:is>
       </x:c>
       <x:c r="F19" s="2" t="inlineStr">
@@ -860,19 +860,19 @@
       </x:c>
       <x:c r="G19" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Captcha:MasterCode 只在 Development 生效且須為 4–6 位數字；其他環境有設定即寫 Error 並拒絕啟動；每次使用寫 Warning（帳號、IP），稽核日誌於 WU-SYS-007 補上。</x:t>
+          <x:t xml:space="preserve">重設密碼需 SYS.USER.RESET_PASSWORD，依密碼政策驗證，重新起算到期並清除鎖定，舊密碼即失效；解鎖需 SYS.USER.EDIT，清除失敗計數與鎖定，未鎖定時亦回 204；他公司用戶 404。</x:t>
         </x:is>
       </x:c>
       <x:c r="H19" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:58</x:t>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:47</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.24.5</x:t>
+          <x:t xml:space="preserve">REQ_F4118.24.1</x:t>
         </x:is>
       </x:c>
       <x:c r="B20" s="2" t="inlineStr">
@@ -892,7 +892,7 @@
       </x:c>
       <x:c r="E20" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">System should provide a trilingual login page that keeps the session and refreshes tokens automatically.</x:t>
+          <x:t xml:space="preserve">System should allow a user to log in with username, password and a numeric captcha.</x:t>
         </x:is>
       </x:c>
       <x:c r="F20" s="2" t="inlineStr">
@@ -902,7 +902,7 @@
       </x:c>
       <x:c r="G20" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">未登入進入主框架導向 /login?returnUrl=…，登入後只回到站內路徑；Captcha 元件只收 4–6 位數字，失敗後換新圖並清空密碼；錯誤依 errorCode 三語顯示；API 請求帶 Bearer，401 時只刷新一次並重送，並發 401 共用同一 refresh；刷新失敗清除 Session 回登入頁；登出撤銷 Refresh Token，伺服器失敗也清除本機 Session。</x:t>
+          <x:t xml:space="preserve">帳號不分大小寫；Captcha 4–6 位數字，答案只存伺服器端，驗證一次即作廢（不論對錯）；帳密錯誤、帳號不存在、停用或鎖定一律回 401 SYS.AUTH.INVALID_CREDENTIALS；密碼到期回 403 SYS.AUTH.PASSWORD_EXPIRED 且不發 Token。</x:t>
         </x:is>
       </x:c>
       <x:c r="H20" s="2" t="inlineStr">
@@ -914,7 +914,7 @@
     <x:row r="21">
       <x:c r="A21" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.25.1</x:t>
+          <x:t xml:space="preserve">REQ_F4118.24.2</x:t>
         </x:is>
       </x:c>
       <x:c r="B21" s="2" t="inlineStr">
@@ -924,7 +924,7 @@
       </x:c>
       <x:c r="C21" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Role, Permission and Data Scope</x:t>
+          <x:t xml:space="preserve">Login, Token and Captcha</x:t>
         </x:is>
       </x:c>
       <x:c r="D21" s="2" t="inlineStr">
@@ -934,7 +934,7 @@
       </x:c>
       <x:c r="E21" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">System should allow authorized users to view roles and the permission catalog.</x:t>
+          <x:t xml:space="preserve">System should issue a 15-minute access token and a 7-day rotating refresh token.</x:t>
         </x:is>
       </x:c>
       <x:c r="F21" s="2" t="inlineStr">
@@ -944,19 +944,19 @@
       </x:c>
       <x:c r="G21" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">需 SYS.ROLE.VIEW；角色列表支援分頁、關鍵字（代碼／名稱）、code／name 排序；權限目錄列出各模組宣告的全部代碼；已軟刪除角色不顯示，查詢回 404。</x:t>
+          <x:t xml:space="preserve">Access Token 為 HS256 JWT，sub 為用戶 Id；Refresh Token 只以 SHA-256 雜湊存 Redis，使用一次即輪替，並發重放只有一個成功。</x:t>
         </x:is>
       </x:c>
       <x:c r="H21" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:71</x:t>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:60</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.25.2</x:t>
+          <x:t xml:space="preserve">REQ_F4118.24.3</x:t>
         </x:is>
       </x:c>
       <x:c r="B22" s="2" t="inlineStr">
@@ -966,7 +966,7 @@
       </x:c>
       <x:c r="C22" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Role, Permission and Data Scope</x:t>
+          <x:t xml:space="preserve">Login, Token and Captcha</x:t>
         </x:is>
       </x:c>
       <x:c r="D22" s="2" t="inlineStr">
@@ -976,7 +976,7 @@
       </x:c>
       <x:c r="E22" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">System should allow authorized users to create a role with permissions and a data scope.</x:t>
+          <x:t xml:space="preserve">System should allow a logged-in user to log out and invalidate the refresh token.</x:t>
         </x:is>
       </x:c>
       <x:c r="F22" s="2" t="inlineStr">
@@ -986,19 +986,19 @@
       </x:c>
       <x:c r="G22" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">需 SYS.ROLE.CREATE；代碼 1–50 字元 ASCII 英文、數字、-、_，保存為大寫，全系統唯一（含已刪除），重複回 409 SYS.ROLE.DUPLICATE_CODE；權限代碼不分大小寫輸入，必須在權限目錄內，否則 400；資料範圍為 Self／Department／Branch／Company。</x:t>
+          <x:t xml:space="preserve">登出須帶有效 Access Token；只撤銷屬於本人的 Refresh Token，撤銷後刷新回 401。</x:t>
         </x:is>
       </x:c>
       <x:c r="H22" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:72</x:t>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:61</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.25.3</x:t>
+          <x:t xml:space="preserve">REQ_F4118.24.4</x:t>
         </x:is>
       </x:c>
       <x:c r="B23" s="2" t="inlineStr">
@@ -1008,7 +1008,7 @@
       </x:c>
       <x:c r="C23" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Role, Permission and Data Scope</x:t>
+          <x:t xml:space="preserve">Login, Token and Captcha</x:t>
         </x:is>
       </x:c>
       <x:c r="D23" s="2" t="inlineStr">
@@ -1018,7 +1018,7 @@
       </x:c>
       <x:c r="E23" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">System should allow authorized users to edit or deactivate a role.</x:t>
+          <x:t xml:space="preserve">System should provide a development-only captcha master code with startup protection.</x:t>
         </x:is>
       </x:c>
       <x:c r="F23" s="2" t="inlineStr">
@@ -1028,19 +1028,19 @@
       </x:c>
       <x:c r="G23" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">需 SYS.ROLE.EDIT；帶 version，不符回 409，且權限集合不變（同一交易）；停用角色立即不再授予權限。</x:t>
+          <x:t xml:space="preserve">Captcha:MasterCode 只在 Development 生效且須為 4–6 位數字；其他環境有設定即寫 Error 並拒絕啟動；每次使用寫 Warning（帳號、IP），稽核日誌於 WU-SYS-007 補上。</x:t>
         </x:is>
       </x:c>
       <x:c r="H23" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:73</x:t>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:62</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.25.4</x:t>
+          <x:t xml:space="preserve">REQ_F4118.24.5</x:t>
         </x:is>
       </x:c>
       <x:c r="B24" s="2" t="inlineStr">
@@ -1050,7 +1050,7 @@
       </x:c>
       <x:c r="C24" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Role, Permission and Data Scope</x:t>
+          <x:t xml:space="preserve">Login, Token and Captcha</x:t>
         </x:is>
       </x:c>
       <x:c r="D24" s="2" t="inlineStr">
@@ -1060,7 +1060,7 @@
       </x:c>
       <x:c r="E24" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">System should allow authorized users to delete an unused role.</x:t>
+          <x:t xml:space="preserve">System should provide a trilingual login page that keeps the session and refreshes tokens automatically.</x:t>
         </x:is>
       </x:c>
       <x:c r="F24" s="2" t="inlineStr">
@@ -1070,19 +1070,19 @@
       </x:c>
       <x:c r="G24" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">需 SYS.ROLE.DELETE；仍有用戶使用回 422 SYS.ROLE.IN_USE；軟刪除，代碼不可重用。</x:t>
+          <x:t xml:space="preserve">未登入進入主框架導向 /login?returnUrl=…，登入後只回到站內路徑；Captcha 元件只收 4–6 位數字，失敗後換新圖並清空密碼；錯誤依 errorCode 三語顯示；API 請求帶 Bearer，401 時只刷新一次並重送，並發 401 共用同一 refresh；刷新失敗清除 Session 回登入頁；登出撤銷 Refresh Token，伺服器失敗也清除本機 Session。</x:t>
         </x:is>
       </x:c>
       <x:c r="H24" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:74</x:t>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:63</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.25.5</x:t>
+          <x:t xml:space="preserve">REQ_F4118.25.1</x:t>
         </x:is>
       </x:c>
       <x:c r="B25" s="2" t="inlineStr">
@@ -1102,7 +1102,7 @@
       </x:c>
       <x:c r="E25" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">System should enforce permission codes on every API with the backend as the authority.</x:t>
+          <x:t xml:space="preserve">System should allow authorized users to view roles and the permission catalog.</x:t>
         </x:is>
       </x:c>
       <x:c r="F25" s="2" t="inlineStr">
@@ -1112,7 +1112,7 @@
       </x:c>
       <x:c r="G25" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">每個 API 動作標註 模組.資源.動作 權限（ArchitectureTests 檢查）；未登入 401；缺權限或沒有公司上下文 403 COMMON.PERMISSION.DENIED；已登入請求的 X-Company-Id 不可存取（未授權、用戶公司關聯停用、公司停用）一律 403 COMMON.COMPANY.ACCESS_DENIED。</x:t>
+          <x:t xml:space="preserve">需 SYS.ROLE.VIEW；角色列表支援分頁、關鍵字（代碼／名稱）、code／name 排序；權限目錄列出各模組宣告的全部代碼；已軟刪除角色不顯示，查詢回 404。</x:t>
         </x:is>
       </x:c>
       <x:c r="H25" s="2" t="inlineStr">
@@ -1124,7 +1124,7 @@
     <x:row r="26">
       <x:c r="A26" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.25.6</x:t>
+          <x:t xml:space="preserve">REQ_F4118.25.2</x:t>
         </x:is>
       </x:c>
       <x:c r="B26" s="2" t="inlineStr">
@@ -1144,7 +1144,7 @@
       </x:c>
       <x:c r="E26" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">System should allow authorized users to grant a user access to a company with roles, organization and default company.</x:t>
+          <x:t xml:space="preserve">System should allow authorized users to create a role with permissions and a data scope.</x:t>
         </x:is>
       </x:c>
       <x:c r="F26" s="2" t="inlineStr">
@@ -1154,7 +1154,7 @@
       </x:c>
       <x:c r="G26" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">需 SYS.USER.EDIT；公司必須啟用；分店／部門必須屬於該公司且啟用；角色必須存在且啟用；角色整組取代；每位用戶最多一間預設公司（設定新預設會取消舊預設）。用戶不存在回 404。</x:t>
+          <x:t xml:space="preserve">需 SYS.ROLE.CREATE；代碼 1–50 字元 ASCII 英文、數字、-、_，保存為大寫，全系統唯一（含已刪除），重複回 409 SYS.ROLE.DUPLICATE_CODE；權限代碼不分大小寫輸入，必須在權限目錄內，否則 400；資料範圍為 Self／Department／Branch／Company。</x:t>
         </x:is>
       </x:c>
       <x:c r="H26" s="2" t="inlineStr">
@@ -1166,42 +1166,210 @@
     <x:row r="27">
       <x:c r="A27" s="2" t="inlineStr">
         <x:is>
+          <x:t xml:space="preserve">REQ_F4118.25.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Role, Permission and Data Scope</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to edit or deactivate a role.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">需 SYS.ROLE.EDIT；帶 version，不符回 409，且權限集合不變（同一交易）；停用角色立即不再授予權限。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:77</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.25.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B28" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C28" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Role, Permission and Data Scope</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D28" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E28" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to delete an unused role.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F28" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G28" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">需 SYS.ROLE.DELETE；仍有用戶使用回 422 SYS.ROLE.IN_USE；軟刪除，代碼不可重用。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H28" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:78</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.25.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B29" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C29" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Role, Permission and Data Scope</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D29" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E29" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enforce permission codes on every API with the backend as the authority.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F29" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G29" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">每個 API 動作標註 模組.資源.動作 權限（ArchitectureTests 檢查）；未登入 401；缺權限或沒有公司上下文 403 COMMON.PERMISSION.DENIED；已登入請求的 X-Company-Id 不可存取（未授權、用戶公司關聯停用、公司停用）一律 403 COMMON.COMPANY.ACCESS_DENIED。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H29" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:79</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.25.6</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B30" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C30" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Role, Permission and Data Scope</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D30" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E30" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to grant a user access to a company with roles, organization and default company.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F30" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G30" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">需 SYS.USER.EDIT；公司必須啟用；分店／部門必須屬於該公司且啟用；角色必須存在且啟用；角色整組取代；每位用戶最多一間預設公司（設定新預設會取消舊預設）。用戶不存在回 404。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H30" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:80</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="2" t="inlineStr">
+        <x:is>
           <x:t xml:space="preserve">REQ_F4118.25.7</x:t>
         </x:is>
       </x:c>
-      <x:c r="B27" s="2" t="inlineStr">
+      <x:c r="B31" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Settings</x:t>
         </x:is>
       </x:c>
-      <x:c r="C27" s="2" t="inlineStr">
+      <x:c r="C31" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Role, Permission and Data Scope</x:t>
         </x:is>
       </x:c>
-      <x:c r="D27" s="2" t="inlineStr">
+      <x:c r="D31" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">1.0</x:t>
         </x:is>
       </x:c>
-      <x:c r="E27" s="2" t="inlineStr">
+      <x:c r="E31" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">System should resolve the user's effective permissions and data scope per company and hide unauthorized UI.</x:t>
         </x:is>
       </x:c>
-      <x:c r="F27" s="2" t="inlineStr">
+      <x:c r="F31" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Developer</x:t>
         </x:is>
       </x:c>
-      <x:c r="G27" s="2" t="inlineStr">
+      <x:c r="G31" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">同一權限取各啟用角色最寬的資料範圍；全權角色視為全部權限、全公司範圍；分店／部門範圍但用戶無對應歸屬時退回本人。GET /api/v1/sys/auth/authorization 回傳可存取公司（預設在前）與目前公司權限；前端 *erpHasPermission、permissionGuard 與選單依此隱藏，切換公司重新載入；本機記住的公司不可存取時改用預設公司。</x:t>
         </x:is>
       </x:c>
-      <x:c r="H27" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:77</x:t>
+      <x:c r="H31" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:81</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -2276,7 +2444,7 @@
       </x:c>
       <x:c r="F4" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.23.1, REQ_F4118.23.2, REQ_F4118.23.3, REQ_F4118.23.4</x:t>
+          <x:t xml:space="preserve">REQ_F4118.23.1, REQ_F4118.23.2, REQ_F4118.23.3, REQ_F4118.23.4, REQ_F4118.23.5, REQ_F4118.23.6, REQ_F4118.23.7, REQ_F4118.23.8</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -2404,7 +2572,7 @@
       </x:c>
       <x:c r="F8" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.25.5, REQ_F4118.25.6, REQ_F4118.25.7</x:t>
+          <x:t xml:space="preserve">REQ_F4118.23.5, REQ_F4118.23.6, REQ_F4118.25.5, REQ_F4118.25.6, REQ_F4118.25.7</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -2450,7 +2618,7 @@
     <x:col min="1" max="1" width="16" customWidth="1"/>
     <x:col min="2" max="2" width="15" customWidth="1"/>
     <x:col min="3" max="3" width="32" customWidth="1"/>
-    <x:col min="4" max="4" width="30" customWidth="1"/>
+    <x:col min="4" max="4" width="32" customWidth="1"/>
     <x:col min="5" max="5" width="13" customWidth="1"/>
     <x:col min="6" max="6" width="23" customWidth="1"/>
     <x:col min="7" max="7" width="40" customWidth="1"/>
@@ -2840,7 +3008,7 @@
       </x:c>
       <x:c r="H7" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">3–100 字元，字母／數字／點／底線／連字號</x:t>
+          <x:t xml:space="preserve">去除前後空白後 3–100 字元，字母／數字／點／底線／連字號；不分大小寫唯一</x:t>
         </x:is>
       </x:c>
       <x:c r="I7" s="2" t="inlineStr">
@@ -2892,17 +3060,17 @@
       </x:c>
       <x:c r="G8" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Password text</x:t>
+          <x:t xml:space="preserve">Password，autocomplete=new-password</x:t>
         </x:is>
       </x:c>
       <x:c r="H8" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">預設 12–128 字元</x:t>
+          <x:t xml:space="preserve">必填，最多 128 字元；其餘依政策（預設 12 字元以上，含大小寫、數字、符號），不符時顯示政策說明</x:t>
         </x:is>
       </x:c>
       <x:c r="I8" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">None</x:t>
+          <x:t xml:space="preserve">REQ_IO_A8.61.3</x:t>
         </x:is>
       </x:c>
       <x:c r="J8" s="2" t="inlineStr">
@@ -2919,47 +3087,47 @@
     <x:row r="9">
       <x:c r="A9" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A8.62.1</x:t>
+          <x:t xml:space="preserve">REQ_IO_A8.61.3</x:t>
         </x:is>
       </x:c>
       <x:c r="B9" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.8.62</x:t>
+          <x:t xml:space="preserve">4.4.1.8.61</x:t>
         </x:is>
       </x:c>
       <x:c r="C9" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Login Interface</x:t>
+          <x:t xml:space="preserve">User Identity Create Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D9" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Username (Input)</x:t>
+          <x:t xml:space="preserve">Confirm Password (Input)</x:t>
         </x:is>
       </x:c>
       <x:c r="E9" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">帳號</x:t>
+          <x:t xml:space="preserve">確認密碼</x:t>
         </x:is>
       </x:c>
       <x:c r="F9" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">登入身分</x:t>
+          <x:t xml:space="preserve">防止輸入錯誤</x:t>
         </x:is>
       </x:c>
       <x:c r="G9" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Text，autocomplete=username</x:t>
+          <x:t xml:space="preserve">Password</x:t>
         </x:is>
       </x:c>
       <x:c r="H9" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">必填、非空白，最多 100 字元；送出前去除前後空白</x:t>
+          <x:t xml:space="preserve">須與密碼相同</x:t>
         </x:is>
       </x:c>
       <x:c r="I9" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">None</x:t>
+          <x:t xml:space="preserve">REQ_IO_A8.61.2</x:t>
         </x:is>
       </x:c>
       <x:c r="J9" s="2" t="inlineStr">
@@ -2976,7 +3144,7 @@
     <x:row r="10">
       <x:c r="A10" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A8.62.2</x:t>
+          <x:t xml:space="preserve">REQ_IO_A8.62.1</x:t>
         </x:is>
       </x:c>
       <x:c r="B10" s="2" t="inlineStr">
@@ -2991,27 +3159,27 @@
       </x:c>
       <x:c r="D10" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Password (Input)</x:t>
+          <x:t xml:space="preserve">Username (Input)</x:t>
         </x:is>
       </x:c>
       <x:c r="E10" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">密碼</x:t>
+          <x:t xml:space="preserve">帳號</x:t>
         </x:is>
       </x:c>
       <x:c r="F10" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">驗證身分</x:t>
+          <x:t xml:space="preserve">登入身分</x:t>
         </x:is>
       </x:c>
       <x:c r="G10" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Password，autocomplete=current-password</x:t>
+          <x:t xml:space="preserve">Text，autocomplete=username</x:t>
         </x:is>
       </x:c>
       <x:c r="H10" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">必填，最多 128 字元；失敗後清空</x:t>
+          <x:t xml:space="preserve">必填、非空白，最多 100 字元；送出前去除前後空白</x:t>
         </x:is>
       </x:c>
       <x:c r="I10" s="2" t="inlineStr">
@@ -3033,7 +3201,7 @@
     <x:row r="11">
       <x:c r="A11" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A8.62.3</x:t>
+          <x:t xml:space="preserve">REQ_IO_A8.62.2</x:t>
         </x:is>
       </x:c>
       <x:c r="B11" s="2" t="inlineStr">
@@ -3048,32 +3216,32 @@
       </x:c>
       <x:c r="D11" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Captcha Code (Input)</x:t>
+          <x:t xml:space="preserve">Password (Input)</x:t>
         </x:is>
       </x:c>
       <x:c r="E11" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">驗證碼</x:t>
+          <x:t xml:space="preserve">密碼</x:t>
         </x:is>
       </x:c>
       <x:c r="F11" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">防自動化登入</x:t>
+          <x:t xml:space="preserve">驗證身分</x:t>
         </x:is>
       </x:c>
       <x:c r="G11" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">數字，inputmode=numeric</x:t>
+          <x:t xml:space="preserve">Password，autocomplete=current-password</x:t>
         </x:is>
       </x:c>
       <x:c r="H11" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4–6 位數字（非數字自動移除）</x:t>
+          <x:t xml:space="preserve">必填，最多 128 字元；失敗後清空</x:t>
         </x:is>
       </x:c>
       <x:c r="I11" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A8.62.4</x:t>
+          <x:t xml:space="preserve">None</x:t>
         </x:is>
       </x:c>
       <x:c r="J11" s="2" t="inlineStr">
@@ -3090,47 +3258,47 @@
     <x:row r="12">
       <x:c r="A12" s="2" t="inlineStr">
         <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.62.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B12" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.62</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C12" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Login Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D12" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Captcha Code (Input)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E12" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">驗證碼</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F12" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">防自動化登入</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G12" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">數字，inputmode=numeric</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H12" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4–6 位數字（非數字自動移除）</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I12" s="2" t="inlineStr">
+        <x:is>
           <x:t xml:space="preserve">REQ_IO_A8.62.4</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B12" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">4.4.1.8.62</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C12" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Login Interface</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D12" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Captcha Image (Button)</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E12" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">驗證碼圖片</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F12" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">顯示題目，點擊換圖</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G12" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">SVG data URI</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H12" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">每次送出失敗後自動換新</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I12" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">None</x:t>
         </x:is>
       </x:c>
       <x:c r="J12" s="2" t="inlineStr">
@@ -3147,7 +3315,7 @@
     <x:row r="13">
       <x:c r="A13" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A8.62.5</x:t>
+          <x:t xml:space="preserve">REQ_IO_A8.62.4</x:t>
         </x:is>
       </x:c>
       <x:c r="B13" s="2" t="inlineStr">
@@ -3162,27 +3330,27 @@
       </x:c>
       <x:c r="D13" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Sign In (Button)</x:t>
+          <x:t xml:space="preserve">Captcha Image (Button)</x:t>
         </x:is>
       </x:c>
       <x:c r="E13" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">登入</x:t>
+          <x:t xml:space="preserve">驗證碼圖片</x:t>
         </x:is>
       </x:c>
       <x:c r="F13" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">送出</x:t>
+          <x:t xml:space="preserve">顯示題目，點擊換圖</x:t>
         </x:is>
       </x:c>
       <x:c r="G13" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Button</x:t>
+          <x:t xml:space="preserve">SVG data URI</x:t>
         </x:is>
       </x:c>
       <x:c r="H13" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">送出中顯示載入狀態，不可重複送出</x:t>
+          <x:t xml:space="preserve">每次送出失敗後自動換新</x:t>
         </x:is>
       </x:c>
       <x:c r="I13" s="2" t="inlineStr">
@@ -3204,55 +3372,397 @@
     <x:row r="14">
       <x:c r="A14" s="2" t="inlineStr">
         <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.62.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.62</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Login Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Sign In (Button)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">登入</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">送出</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Button</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">送出中顯示載入狀態，不可重複送出</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="2" t="inlineStr">
+        <x:is>
           <x:t xml:space="preserve">REQ_IO_A8.62.6</x:t>
         </x:is>
       </x:c>
-      <x:c r="B14" s="2" t="inlineStr">
+      <x:c r="B15" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">4.4.1.8.62</x:t>
         </x:is>
       </x:c>
-      <x:c r="C14" s="2" t="inlineStr">
+      <x:c r="C15" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Login Interface</x:t>
         </x:is>
       </x:c>
-      <x:c r="D14" s="2" t="inlineStr">
+      <x:c r="D15" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Error Message (Alert)</x:t>
         </x:is>
       </x:c>
-      <x:c r="E14" s="2" t="inlineStr">
+      <x:c r="E15" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">錯誤訊息</x:t>
         </x:is>
       </x:c>
-      <x:c r="F14" s="2" t="inlineStr">
+      <x:c r="F15" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">顯示 errors.&lt;errorCode&gt;</x:t>
         </x:is>
       </x:c>
-      <x:c r="G14" s="2" t="inlineStr">
+      <x:c r="G15" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Text</x:t>
         </x:is>
       </x:c>
-      <x:c r="H14" s="2" t="inlineStr">
+      <x:c r="H15" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">INVALID_CREDENTIALS／CAPTCHA_INVALID／PASSWORD_EXPIRED／VALIDATION_FAILED／網路／未知</x:t>
         </x:is>
       </x:c>
-      <x:c r="I14" s="2" t="inlineStr">
+      <x:c r="I15" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">None</x:t>
         </x:is>
       </x:c>
-      <x:c r="J14" s="2" t="inlineStr">
+      <x:c r="J15" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">1.0</x:t>
         </x:is>
       </x:c>
-      <x:c r="K14" s="2" t="inlineStr">
+      <x:c r="K15" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.63.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B16" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.63</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C16" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">User Maintenance Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D16" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Keyword (Input)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E16" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">搜尋帳號</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F16" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">篩選列表</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G16" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Text</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H16" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">去除前後空白，不分大小寫</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I16" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J16" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K16" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.63.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B17" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.63</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C17" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">User Maintenance Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D17" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Status (Tag)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E17" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">狀態</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F17" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">顯示啟用、鎖定、密碼過期</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G17" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Tag</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H17" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">啟用／停用；已鎖定；密碼已過期</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I17" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J17" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K17" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.63.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B18" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.63</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C18" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">User Maintenance Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D18" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Activate / Deactivate (Button)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E18" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">啟用／停用</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F18" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">切換帳號狀態</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G18" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Button</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H18" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">帶讀取時的 version；不可停用自己</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I18" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J18" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K18" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.63.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B19" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.63</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C19" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">User Maintenance Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D19" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Unlock (Button)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E19" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">解鎖</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F19" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">清除鎖定</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G19" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Button</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H19" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">只在已鎖定時顯示</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I19" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J19" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K19" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.63.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B20" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.63</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C20" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">User Maintenance Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D20" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Reset Password (Button)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E20" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">重設密碼</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F20" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">開啟重設對話框</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G20" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Button</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H20" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">新密碼依政策驗證，成功後清除鎖定並重新起算到期</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I20" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.61.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J20" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K20" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Developer</x:t>
         </x:is>
@@ -3709,7 +4219,7 @@
       </x:c>
       <x:c r="F12" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-USER-001, SYS-USER-004, SYS-USER-006</x:t>
+          <x:t xml:space="preserve">SYS-USER-001, SYS-USER-004, SYS-USER-012</x:t>
         </x:is>
       </x:c>
       <x:c r="G12" s="2" t="inlineStr">
@@ -3741,12 +4251,12 @@
       </x:c>
       <x:c r="E13" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A8.61.2</x:t>
+          <x:t xml:space="preserve">REQ_IO_A8.61.2, REQ_IO_A8.61.3</x:t>
         </x:is>
       </x:c>
       <x:c r="F13" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-USER-001, SYS-USER-007, SYS-USER-006</x:t>
+          <x:t xml:space="preserve">SYS-USER-001, SYS-USER-007, SYS-USER-012</x:t>
         </x:is>
       </x:c>
       <x:c r="G13" s="2" t="inlineStr">
@@ -3783,7 +4293,7 @@
       </x:c>
       <x:c r="F14" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-USER-002, SYS-USER-003, SYS-USER-005, SYS-USER-006</x:t>
+          <x:t xml:space="preserve">SYS-USER-002, SYS-USER-003, SYS-USER-005, SYS-USER-014</x:t>
         </x:is>
       </x:c>
       <x:c r="G14" s="2" t="inlineStr">
@@ -3820,7 +4330,7 @@
       </x:c>
       <x:c r="F15" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-USER-003, SYS-USER-006</x:t>
+          <x:t xml:space="preserve">SYS-USER-003</x:t>
         </x:is>
       </x:c>
       <x:c r="G15" s="2" t="inlineStr">
@@ -3832,160 +4342,160 @@
     <x:row r="16">
       <x:c r="A16" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.24.1</x:t>
+          <x:t xml:space="preserve">REQ_F4118.23.5</x:t>
         </x:is>
       </x:c>
       <x:c r="B16" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">System should allow a user to log in with username, password and a numeric captcha.</x:t>
+          <x:t xml:space="preserve">System should list the users of the current company with paging, keyword and sorting.</x:t>
         </x:is>
       </x:c>
       <x:c r="C16" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">REQ_DS43.82, REQ_DS43.92</x:t>
         </x:is>
       </x:c>
       <x:c r="D16" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.8.62</x:t>
+          <x:t xml:space="preserve">4.4.1.8.63</x:t>
         </x:is>
       </x:c>
       <x:c r="E16" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A8.62.1, REQ_IO_A8.62.2, REQ_IO_A8.62.3, REQ_IO_A8.62.4</x:t>
+          <x:t xml:space="preserve">REQ_IO_A8.63.1, REQ_IO_A8.63.2</x:t>
         </x:is>
       </x:c>
       <x:c r="F16" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-AUTH-001, SYS-AUTH-002, SYS-AUTH-005, SYS-AUTH-006, SYS-AUTH-009, SYS-AUTH-014, SYS-AUTH-015, SYS-AUTH-016, SYS-AUTH-017</x:t>
+          <x:t xml:space="preserve">SYS-USER-006, SYS-USER-010, SYS-USER-011, SYS-USER-015</x:t>
         </x:is>
       </x:c>
       <x:c r="G16" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Partial</x:t>
+          <x:t xml:space="preserve">Covered</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.24.2</x:t>
+          <x:t xml:space="preserve">REQ_F4118.23.6</x:t>
         </x:is>
       </x:c>
       <x:c r="B17" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">System should issue a 15-minute access token and a 7-day rotating refresh token.</x:t>
+          <x:t xml:space="preserve">System should allow authorized users to create a user in the current company.</x:t>
         </x:is>
       </x:c>
       <x:c r="C17" s="2" t="inlineStr">
         <x:is>
+          <x:t xml:space="preserve">REQ_DS43.82, REQ_DS43.92</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D17" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.61</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E17" s="2" t="inlineStr">
+        <x:is>
           <x:t xml:space="preserve"/>
         </x:is>
       </x:c>
-      <x:c r="D17" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
-      <x:c r="E17" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
       <x:c r="F17" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-AUTH-001, SYS-AUTH-004, SYS-AUTH-007, SYS-AUTH-009, SYS-AUTH-010, SYS-AUTH-016, SYS-AUTH-017</x:t>
+          <x:t xml:space="preserve">SYS-USER-006, SYS-USER-010, SYS-USER-011, SYS-USER-012</x:t>
         </x:is>
       </x:c>
       <x:c r="G17" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Partial</x:t>
+          <x:t xml:space="preserve">Covered</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.24.3</x:t>
+          <x:t xml:space="preserve">REQ_F4118.23.7</x:t>
         </x:is>
       </x:c>
       <x:c r="B18" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">System should allow a logged-in user to log out and invalidate the refresh token.</x:t>
+          <x:t xml:space="preserve">System should allow authorized users to activate or deactivate a user.</x:t>
         </x:is>
       </x:c>
       <x:c r="C18" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">REQ_DS43.82</x:t>
         </x:is>
       </x:c>
       <x:c r="D18" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">4.4.1.8.63</x:t>
         </x:is>
       </x:c>
       <x:c r="E18" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">REQ_IO_A8.63.3</x:t>
         </x:is>
       </x:c>
       <x:c r="F18" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-AUTH-008, SYS-AUTH-016, SYS-AUTH-017</x:t>
+          <x:t xml:space="preserve">SYS-USER-006, SYS-USER-010, SYS-USER-013, SYS-USER-015</x:t>
         </x:is>
       </x:c>
       <x:c r="G18" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Partial</x:t>
+          <x:t xml:space="preserve">Covered</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.24.4</x:t>
+          <x:t xml:space="preserve">REQ_F4118.23.8</x:t>
         </x:is>
       </x:c>
       <x:c r="B19" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">System should provide a development-only captcha master code with startup protection.</x:t>
+          <x:t xml:space="preserve">System should allow authorized users to reset a password and unlock a locked user.</x:t>
         </x:is>
       </x:c>
       <x:c r="C19" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">REQ_DS43.82</x:t>
         </x:is>
       </x:c>
       <x:c r="D19" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">4.4.1.8.63</x:t>
         </x:is>
       </x:c>
       <x:c r="E19" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">REQ_IO_A8.63.4, REQ_IO_A8.63.5</x:t>
         </x:is>
       </x:c>
       <x:c r="F19" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-AUTH-003, SYS-AUTH-004, SYS-AUTH-016, SYS-AUTH-017</x:t>
+          <x:t xml:space="preserve">SYS-USER-006, SYS-USER-010, SYS-USER-014</x:t>
         </x:is>
       </x:c>
       <x:c r="G19" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Partial</x:t>
+          <x:t xml:space="preserve">Covered</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.24.5</x:t>
+          <x:t xml:space="preserve">REQ_F4118.24.1</x:t>
         </x:is>
       </x:c>
       <x:c r="B20" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">System should provide a trilingual login page that keeps the session and refreshes tokens automatically.</x:t>
+          <x:t xml:space="preserve">System should allow a user to log in with username, password and a numeric captcha.</x:t>
         </x:is>
       </x:c>
       <x:c r="C20" s="2" t="inlineStr">
@@ -4000,12 +4510,12 @@
       </x:c>
       <x:c r="E20" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A8.62.5, REQ_IO_A8.62.6</x:t>
+          <x:t xml:space="preserve">REQ_IO_A8.62.1, REQ_IO_A8.62.2, REQ_IO_A8.62.3, REQ_IO_A8.62.4</x:t>
         </x:is>
       </x:c>
       <x:c r="F20" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-AUTH-011, SYS-AUTH-012, SYS-AUTH-013, SYS-AUTH-015, SYS-AUTH-016, SYS-AUTH-017</x:t>
+          <x:t xml:space="preserve">SYS-AUTH-001, SYS-AUTH-002, SYS-AUTH-005, SYS-AUTH-006, SYS-AUTH-009, SYS-AUTH-014, SYS-AUTH-015, SYS-AUTH-016, SYS-AUTH-017</x:t>
         </x:is>
       </x:c>
       <x:c r="G20" s="2" t="inlineStr">
@@ -4017,17 +4527,17 @@
     <x:row r="21">
       <x:c r="A21" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.25.1</x:t>
+          <x:t xml:space="preserve">REQ_F4118.24.2</x:t>
         </x:is>
       </x:c>
       <x:c r="B21" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">System should allow authorized users to view roles and the permission catalog.</x:t>
+          <x:t xml:space="preserve">System should issue a 15-minute access token and a 7-day rotating refresh token.</x:t>
         </x:is>
       </x:c>
       <x:c r="C21" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_DS43.90</x:t>
+          <x:t xml:space="preserve"/>
         </x:is>
       </x:c>
       <x:c r="D21" s="2" t="inlineStr">
@@ -4042,7 +4552,7 @@
       </x:c>
       <x:c r="F21" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-PERM-004, SYS-PERM-011, SYS-PERM-024</x:t>
+          <x:t xml:space="preserve">SYS-AUTH-001, SYS-AUTH-004, SYS-AUTH-007, SYS-AUTH-009, SYS-AUTH-010, SYS-AUTH-016, SYS-AUTH-017</x:t>
         </x:is>
       </x:c>
       <x:c r="G21" s="2" t="inlineStr">
@@ -4054,17 +4564,17 @@
     <x:row r="22">
       <x:c r="A22" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.25.2</x:t>
+          <x:t xml:space="preserve">REQ_F4118.24.3</x:t>
         </x:is>
       </x:c>
       <x:c r="B22" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">System should allow authorized users to create a role with permissions and a data scope.</x:t>
+          <x:t xml:space="preserve">System should allow a logged-in user to log out and invalidate the refresh token.</x:t>
         </x:is>
       </x:c>
       <x:c r="C22" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_DS43.90, REQ_DS43.91</x:t>
+          <x:t xml:space="preserve"/>
         </x:is>
       </x:c>
       <x:c r="D22" s="2" t="inlineStr">
@@ -4079,7 +4589,7 @@
       </x:c>
       <x:c r="F22" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-PERM-011, SYS-PERM-024</x:t>
+          <x:t xml:space="preserve">SYS-AUTH-008, SYS-AUTH-016, SYS-AUTH-017</x:t>
         </x:is>
       </x:c>
       <x:c r="G22" s="2" t="inlineStr">
@@ -4091,17 +4601,17 @@
     <x:row r="23">
       <x:c r="A23" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.25.3</x:t>
+          <x:t xml:space="preserve">REQ_F4118.24.4</x:t>
         </x:is>
       </x:c>
       <x:c r="B23" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">System should allow authorized users to edit or deactivate a role.</x:t>
+          <x:t xml:space="preserve">System should provide a development-only captcha master code with startup protection.</x:t>
         </x:is>
       </x:c>
       <x:c r="C23" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_DS43.90, REQ_DS43.91</x:t>
+          <x:t xml:space="preserve"/>
         </x:is>
       </x:c>
       <x:c r="D23" s="2" t="inlineStr">
@@ -4116,7 +4626,7 @@
       </x:c>
       <x:c r="F23" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-PERM-011, SYS-PERM-024</x:t>
+          <x:t xml:space="preserve">SYS-AUTH-003, SYS-AUTH-004, SYS-AUTH-016, SYS-AUTH-017</x:t>
         </x:is>
       </x:c>
       <x:c r="G23" s="2" t="inlineStr">
@@ -4128,32 +4638,32 @@
     <x:row r="24">
       <x:c r="A24" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.25.4</x:t>
+          <x:t xml:space="preserve">REQ_F4118.24.5</x:t>
         </x:is>
       </x:c>
       <x:c r="B24" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">System should allow authorized users to delete an unused role.</x:t>
+          <x:t xml:space="preserve">System should provide a trilingual login page that keeps the session and refreshes tokens automatically.</x:t>
         </x:is>
       </x:c>
       <x:c r="C24" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_DS43.90</x:t>
+          <x:t xml:space="preserve"/>
         </x:is>
       </x:c>
       <x:c r="D24" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">4.4.1.8.62</x:t>
         </x:is>
       </x:c>
       <x:c r="E24" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">REQ_IO_A8.62.5, REQ_IO_A8.62.6</x:t>
         </x:is>
       </x:c>
       <x:c r="F24" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-PERM-012, SYS-PERM-024</x:t>
+          <x:t xml:space="preserve">SYS-AUTH-011, SYS-AUTH-012, SYS-AUTH-013, SYS-AUTH-015, SYS-AUTH-016, SYS-AUTH-017</x:t>
         </x:is>
       </x:c>
       <x:c r="G24" s="2" t="inlineStr">
@@ -4165,17 +4675,17 @@
     <x:row r="25">
       <x:c r="A25" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.25.5</x:t>
+          <x:t xml:space="preserve">REQ_F4118.25.1</x:t>
         </x:is>
       </x:c>
       <x:c r="B25" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">System should enforce permission codes on every API with the backend as the authority.</x:t>
+          <x:t xml:space="preserve">System should allow authorized users to view roles and the permission catalog.</x:t>
         </x:is>
       </x:c>
       <x:c r="C25" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_DS43.92</x:t>
+          <x:t xml:space="preserve">REQ_DS43.90</x:t>
         </x:is>
       </x:c>
       <x:c r="D25" s="2" t="inlineStr">
@@ -4190,7 +4700,7 @@
       </x:c>
       <x:c r="F25" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-PERM-001, SYS-PERM-005, SYS-PERM-006, SYS-PERM-010</x:t>
+          <x:t xml:space="preserve">SYS-PERM-004, SYS-PERM-011, SYS-PERM-024</x:t>
         </x:is>
       </x:c>
       <x:c r="G25" s="2" t="inlineStr">
@@ -4202,17 +4712,17 @@
     <x:row r="26">
       <x:c r="A26" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.25.6</x:t>
+          <x:t xml:space="preserve">REQ_F4118.25.2</x:t>
         </x:is>
       </x:c>
       <x:c r="B26" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">System should allow authorized users to grant a user access to a company with roles, organization and default company.</x:t>
+          <x:t xml:space="preserve">System should allow authorized users to create a role with permissions and a data scope.</x:t>
         </x:is>
       </x:c>
       <x:c r="C26" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_DS43.92, REQ_DS43.93</x:t>
+          <x:t xml:space="preserve">REQ_DS43.90, REQ_DS43.91</x:t>
         </x:is>
       </x:c>
       <x:c r="D26" s="2" t="inlineStr">
@@ -4227,7 +4737,7 @@
       </x:c>
       <x:c r="F26" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-PERM-015, SYS-PERM-016, SYS-PERM-024</x:t>
+          <x:t xml:space="preserve">SYS-PERM-011, SYS-PERM-024</x:t>
         </x:is>
       </x:c>
       <x:c r="G26" s="2" t="inlineStr">
@@ -4239,35 +4749,183 @@
     <x:row r="27">
       <x:c r="A27" s="2" t="inlineStr">
         <x:is>
+          <x:t xml:space="preserve">REQ_F4118.25.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to edit or deactivate a role.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.90, REQ_DS43.91</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-PERM-011, SYS-PERM-024</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.25.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B28" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to delete an unused role.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C28" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.90</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D28" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E28" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F28" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-PERM-012, SYS-PERM-024</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G28" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.25.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B29" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enforce permission codes on every API with the backend as the authority.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C29" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.92</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D29" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E29" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F29" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-PERM-001, SYS-PERM-005, SYS-PERM-006, SYS-PERM-010</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G29" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.25.6</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B30" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to grant a user access to a company with roles, organization and default company.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C30" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.92, REQ_DS43.93</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D30" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E30" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F30" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-PERM-015, SYS-PERM-016, SYS-PERM-024</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G30" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="2" t="inlineStr">
+        <x:is>
           <x:t xml:space="preserve">REQ_F4118.25.7</x:t>
         </x:is>
       </x:c>
-      <x:c r="B27" s="2" t="inlineStr">
+      <x:c r="B31" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">System should resolve the user's effective permissions and data scope per company and hide unauthorized UI.</x:t>
         </x:is>
       </x:c>
-      <x:c r="C27" s="2" t="inlineStr">
+      <x:c r="C31" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">REQ_DS43.91, REQ_DS43.92, REQ_DS43.93</x:t>
         </x:is>
       </x:c>
-      <x:c r="D27" s="2" t="inlineStr">
+      <x:c r="D31" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve"/>
         </x:is>
       </x:c>
-      <x:c r="E27" s="2" t="inlineStr">
+      <x:c r="E31" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve"/>
         </x:is>
       </x:c>
-      <x:c r="F27" s="2" t="inlineStr">
+      <x:c r="F31" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">SYS-PERM-002, SYS-PERM-003, SYS-PERM-013, SYS-PERM-014, SYS-PERM-020, SYS-PERM-021, SYS-PERM-022, SYS-PERM-023</x:t>
         </x:is>
       </x:c>
-      <x:c r="G27" s="2" t="inlineStr">
+      <x:c r="G31" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Partial</x:t>
         </x:is>

</xml_diff>

<commit_message>
docs(sys): document security middleware and complete WU-SYS-005
Adds ADR-018, architecture/security.md, REQ_F4118.26.x, SYS-SEC test plan,
cross-origin rate-limit test, and updates state and progress.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R23b7dea85ff1444a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R54dee6920b864470"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R6389d2a2b1af49b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Ra10c7500e3ab4d9e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R0d010cc04a25480c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="Reb09fd7f186f4200"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R31275a1f3f7f48a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R22dc2e391ce54910"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rdeff01a5e27d4fc9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R3d774857c42f45a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Rc7f5663132064e7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R309afbf6b838471e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R57122998222b4ce0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R2e150bdb38594b7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R370a3df8acf24061"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Ra29eb8a22c69427f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="Rcfe04b2e8a5f4caf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Redfc728c80a040fa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -68,7 +68,7 @@
     <x:col min="5" max="5" width="60" customWidth="1"/>
     <x:col min="6" max="6" width="11" customWidth="1"/>
     <x:col min="7" max="7" width="60" customWidth="1"/>
-    <x:col min="8" max="8" width="40" customWidth="1"/>
+    <x:col min="8" max="8" width="41" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -1322,7 +1322,7 @@
       </x:c>
       <x:c r="G30" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">需 SYS.USER.EDIT；公司必須啟用；分店／部門必須屬於該公司且啟用；角色必須存在且啟用；角色整組取代；每位用戶最多一間預設公司（設定新預設會取消舊預設）。用戶不存在回 404。</x:t>
+          <x:t xml:space="preserve">需 SYS.USER.EDIT；公司必須啟用；分店／部門必須屬於該公司且啟用；角色必須存在且啟用；角色整組取代；每位用戶最多一間預設公司（設定新預設會取消舊預設）。用戶不存在或不屬於目前公司回 404 SYS.USER.NOT_FOUND；目標公司不是操作者獲授權的公司回 404 SYS.COMPANY.NOT_FOUND；不可停用自己的公司授權（422 SYS.USER.SELF_DEACTIVATION）（ADR-017）。</x:t>
         </x:is>
       </x:c>
       <x:c r="H30" s="2" t="inlineStr">
@@ -1370,6 +1370,342 @@
       <x:c r="H31" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:81</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.25.8</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B32" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C32" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Role, Permission and Data Scope</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D32" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E32" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to view a user's company access, organization and roles.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F32" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G32" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">需 SYS.USER.VIEW；用戶須屬於目前公司，否則 404；只列出操作者獲授權公司的指派（公司代碼／名稱、分店、部門、預設、啟用、角色 ID），依公司代碼排序（ADR-017）。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H32" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:82</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.26.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B33" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C33" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Web Security Middleware</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D33" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E33" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enforce HTTPS with HSTS outside the development environment.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F33" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G33" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">非 Development：HTTP 請求 307 轉 HTTPS；HTTPS 回應帶 Strict-Transport-Security: max-age=31536000; includeSubDomains（天數可設定）。Development 不轉址、不送 HSTS。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H33" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:96</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.26.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B34" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C34" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Web Security Middleware</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D34" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E34" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow cross-origin requests only from configured frontend origins.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F34" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G34" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">來源清單在 Security:Cors:AllowedOrigins，預設空（不允許跨來源）；只接受 scheme://host[:port]，萬用字元、含路徑或非 http(s) 拒絕啟動；不允許 Credentials；允許標頭 Authorization、Content-Type、Accept、Accept-Language、X-Company-Id；公開 Retry-After、Content-Disposition；未列明的來源預檢回應不含 Access-Control-Allow-Origin。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H34" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:97</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.26.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B35" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C35" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Web Security Middleware</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D35" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E35" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should rate-limit login, token refresh and captcha requests per client IP.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F35" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G35" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">登入、Token 刷新每 IP 每端點每分鐘 5 次；Captcha 每 IP 每分鐘 10 次（ADR-018）；超過回 429 ProblemDetails，errorCode 為 COMMON.REQUEST.RATE_LIMITED，標題依 Accept-Language 三語，帶 Retry-After；寫 Warning 日誌（方法、路徑、IP）。CORS 預檢不計入。每個匿名端點必須套用按 IP 的限流政策（ArchitectureTests 檢查）。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H35" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:98</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.26.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B36" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C36" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Web Security Middleware</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D36" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E36" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should rate-limit authenticated API requests per user.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F36" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G36" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">已登入請求每用戶每分鐘 300 次（可設定），不同用戶分開計數；匯出報表政策每用戶每分鐘 10 次，供日後匯出端點套用。白名單內的 IP 仍受限流。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H36" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:99</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.26.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B37" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C37" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Web Security Middleware</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D37" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E37" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should add security headers to every API response.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F37" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G37" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">所有回應（含 404、429、500）帶 X-Content-Type-Options: nosniff、X-Frame-Options: DENY、Referrer-Policy: no-referrer、Content-Security-Policy: default-src 'none'; frame-ancestors 'none'; base-uri 'none'; form-action 'none'。前端站台的 CSP 見 architecture/security.md，E2E 在該 CSP 下執行。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H37" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:100</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.26.6</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B38" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C38" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Web Security Middleware</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D38" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E38" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should honour X-Forwarded-For only from configured proxies.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F38" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G38" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Security:ForwardedHeaders:KnownProxies（IP）與 KnownNetworks（CIDR）皆空時不處理 X-Forwarded-*；有設定時只信任列明來源，其他來源偽造的 X-Forwarded-For 被忽略，限流與日誌使用連線 IP；格式錯誤拒絕啟動。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H38" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:101</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.26.7</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B39" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C39" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Web Security Middleware</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D39" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E39" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should show a trilingual "too many requests" message when an API call is rate-limited.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F39" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G39" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">前端收到 429 一律顯示 errors.COMMON.REQUEST.RATE_LIMITED（三語），登入頁、組織、用戶、角色頁共用 apiErrorKey。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H39" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:102</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1437,7 +1773,7 @@
       </x:c>
       <x:c r="E2" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/01-architecture/architecture.md:184</x:t>
+          <x:t xml:space="preserve">docs/01-architecture/architecture.md:186</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1464,7 +1800,7 @@
       </x:c>
       <x:c r="E3" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/01-architecture/architecture.md:185</x:t>
+          <x:t xml:space="preserve">docs/01-architecture/architecture.md:187</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1491,7 +1827,7 @@
       </x:c>
       <x:c r="E4" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/01-architecture/architecture.md:186</x:t>
+          <x:t xml:space="preserve">docs/01-architecture/architecture.md:188</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1518,7 +1854,7 @@
       </x:c>
       <x:c r="E5" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/01-architecture/architecture.md:187</x:t>
+          <x:t xml:space="preserve">docs/01-architecture/architecture.md:189</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1545,7 +1881,7 @@
       </x:c>
       <x:c r="E6" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/01-architecture/architecture.md:188</x:t>
+          <x:t xml:space="preserve">docs/01-architecture/architecture.md:190</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1572,7 +1908,7 @@
       </x:c>
       <x:c r="E7" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/01-architecture/architecture.md:189</x:t>
+          <x:t xml:space="preserve">docs/01-architecture/architecture.md:191</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1599,7 +1935,7 @@
       </x:c>
       <x:c r="E8" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/01-architecture/architecture.md:190</x:t>
+          <x:t xml:space="preserve">docs/01-architecture/architecture.md:192</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1626,7 +1962,7 @@
       </x:c>
       <x:c r="E9" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/01-architecture/architecture.md:196</x:t>
+          <x:t xml:space="preserve">docs/01-architecture/architecture.md:198</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1653,7 +1989,7 @@
       </x:c>
       <x:c r="E10" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/01-architecture/architecture.md:197</x:t>
+          <x:t xml:space="preserve">docs/01-architecture/architecture.md:199</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1680,7 +2016,7 @@
       </x:c>
       <x:c r="E11" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/01-architecture/architecture.md:198</x:t>
+          <x:t xml:space="preserve">docs/01-architecture/architecture.md:200</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1707,7 +2043,7 @@
       </x:c>
       <x:c r="E12" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/01-architecture/architecture.md:199</x:t>
+          <x:t xml:space="preserve">docs/01-architecture/architecture.md:201</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1734,7 +2070,7 @@
       </x:c>
       <x:c r="E13" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/01-architecture/architecture.md:200</x:t>
+          <x:t xml:space="preserve">docs/01-architecture/architecture.md:202</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1761,7 +2097,7 @@
       </x:c>
       <x:c r="E14" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/01-architecture/architecture.md:201</x:t>
+          <x:t xml:space="preserve">docs/01-architecture/architecture.md:203</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1788,7 +2124,7 @@
       </x:c>
       <x:c r="E15" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/01-architecture/architecture.md:202</x:t>
+          <x:t xml:space="preserve">docs/01-architecture/architecture.md:204</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1815,7 +2151,7 @@
       </x:c>
       <x:c r="E16" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/01-architecture/architecture.md:203</x:t>
+          <x:t xml:space="preserve">docs/01-architecture/architecture.md:205</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1842,7 +2178,7 @@
       </x:c>
       <x:c r="E17" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/01-architecture/architecture.md:204</x:t>
+          <x:t xml:space="preserve">docs/01-architecture/architecture.md:206</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1869,7 +2205,7 @@
       </x:c>
       <x:c r="E18" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/01-architecture/architecture.md:210</x:t>
+          <x:t xml:space="preserve">docs/01-architecture/architecture.md:212</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1896,7 +2232,7 @@
       </x:c>
       <x:c r="E19" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/01-architecture/architecture.md:211</x:t>
+          <x:t xml:space="preserve">docs/01-architecture/architecture.md:213</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1923,7 +2259,7 @@
       </x:c>
       <x:c r="E20" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/01-architecture/architecture.md:212</x:t>
+          <x:t xml:space="preserve">docs/01-architecture/architecture.md:214</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1950,7 +2286,7 @@
       </x:c>
       <x:c r="E21" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/01-architecture/architecture.md:213</x:t>
+          <x:t xml:space="preserve">docs/01-architecture/architecture.md:215</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1977,7 +2313,7 @@
       </x:c>
       <x:c r="E22" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/01-architecture/architecture.md:214</x:t>
+          <x:t xml:space="preserve">docs/01-architecture/architecture.md:216</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -2004,7 +2340,7 @@
       </x:c>
       <x:c r="E23" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/01-architecture/architecture.md:215</x:t>
+          <x:t xml:space="preserve">docs/01-architecture/architecture.md:217</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -2031,7 +2367,7 @@
       </x:c>
       <x:c r="E24" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/01-architecture/architecture.md:221</x:t>
+          <x:t xml:space="preserve">docs/01-architecture/architecture.md:223</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -2058,7 +2394,7 @@
       </x:c>
       <x:c r="E25" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/01-architecture/architecture.md:222</x:t>
+          <x:t xml:space="preserve">docs/01-architecture/architecture.md:224</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -2085,7 +2421,7 @@
       </x:c>
       <x:c r="E26" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/01-architecture/architecture.md:223</x:t>
+          <x:t xml:space="preserve">docs/01-architecture/architecture.md:225</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -2112,7 +2448,7 @@
       </x:c>
       <x:c r="E27" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/01-architecture/architecture.md:224</x:t>
+          <x:t xml:space="preserve">docs/01-architecture/architecture.md:226</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -2139,7 +2475,7 @@
       </x:c>
       <x:c r="E28" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/01-architecture/architecture.md:225</x:t>
+          <x:t xml:space="preserve">docs/01-architecture/architecture.md:227</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -2166,7 +2502,7 @@
       </x:c>
       <x:c r="E29" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/01-architecture/architecture.md:231</x:t>
+          <x:t xml:space="preserve">docs/01-architecture/architecture.md:233</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -2193,7 +2529,7 @@
       </x:c>
       <x:c r="E30" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/01-architecture/architecture.md:232</x:t>
+          <x:t xml:space="preserve">docs/01-architecture/architecture.md:234</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -2220,7 +2556,7 @@
       </x:c>
       <x:c r="E31" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/01-architecture/architecture.md:233</x:t>
+          <x:t xml:space="preserve">docs/01-architecture/architecture.md:235</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -2247,7 +2583,7 @@
       </x:c>
       <x:c r="E32" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/01-architecture/architecture.md:234</x:t>
+          <x:t xml:space="preserve">docs/01-architecture/architecture.md:236</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -2274,7 +2610,7 @@
       </x:c>
       <x:c r="E33" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/01-architecture/architecture.md:235</x:t>
+          <x:t xml:space="preserve">docs/01-architecture/architecture.md:237</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -2301,7 +2637,7 @@
       </x:c>
       <x:c r="E34" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/01-architecture/architecture.md:236</x:t>
+          <x:t xml:space="preserve">docs/01-architecture/architecture.md:238</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -2572,7 +2908,7 @@
       </x:c>
       <x:c r="F8" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.23.5, REQ_F4118.23.6, REQ_F4118.25.5, REQ_F4118.25.6, REQ_F4118.25.7</x:t>
+          <x:t xml:space="preserve">REQ_F4118.23.5, REQ_F4118.23.6, REQ_F4118.25.5, REQ_F4118.25.6, REQ_F4118.25.7, REQ_F4118.25.8</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -2604,7 +2940,7 @@
       </x:c>
       <x:c r="F9" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.25.6, REQ_F4118.25.7</x:t>
+          <x:t xml:space="preserve">REQ_F4118.25.6, REQ_F4118.25.7, REQ_F4118.25.8</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -2617,7 +2953,7 @@
   <x:cols>
     <x:col min="1" max="1" width="16" customWidth="1"/>
     <x:col min="2" max="2" width="15" customWidth="1"/>
-    <x:col min="3" max="3" width="32" customWidth="1"/>
+    <x:col min="3" max="3" width="54" customWidth="1"/>
     <x:col min="4" max="4" width="32" customWidth="1"/>
     <x:col min="5" max="5" width="13" customWidth="1"/>
     <x:col min="6" max="6" width="23" customWidth="1"/>
@@ -3763,6 +4099,633 @@
         </x:is>
       </x:c>
       <x:c r="K20" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.64.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B21" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.64</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C21" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Role Maintenance Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D21" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Role Code (Input)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E21" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">角色代碼</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F21" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">全系統唯一識別角色</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G21" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">VARCHAR(50)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H21" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1–50 字元；ASCII 英文、數字、-、_；保存為大寫；建立後不可修改</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I21" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J21" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K21" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.64.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B22" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.64</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C22" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Role Maintenance Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D22" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Role Name (Input)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E22" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">角色名稱</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F22" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">顯示角色</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G22" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">NVARCHAR(200)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H22" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">去除空白後 1–200 字元</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I22" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J22" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K22" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.64.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B23" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.64</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C23" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Role Maintenance Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D23" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Data Scope (Dropdown)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E23" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">資料範圍</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F23" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">決定可見單據範圍</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G23" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Self／Department／Branch／Company</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H23" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">必選，預設本人</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I23" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J23" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K23" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.64.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B24" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.64</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C24" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Role Maintenance Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D24" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Full Access (Checkbox)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E24" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">全權</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F24" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">擁有全部權限</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G24" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Boolean</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H24" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">勾選時權限清單停用</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I24" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.64.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J24" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K24" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.64.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B25" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.64</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C25" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Role Maintenance Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D25" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Permissions (Checkbox group)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E25" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">權限</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F25" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">依模組勾選權限代碼</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G25" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">模組.資源.動作</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H25" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">只可選權限目錄內的代碼；模組可全選</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I25" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.64.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J25" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K25" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.64.6</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B26" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.64</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C26" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Role Maintenance Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D26" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Delete (Button)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E26" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">刪除</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F26" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">軟刪除未使用的角色</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G26" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Button + popconfirm</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H26" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">帶 version；使用中回 SYS.ROLE.IN_USE</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I26" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J26" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K26" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.65.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.65</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">User Permission Edit Interface（BlueWhale 4.4.1.8.26）</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Company (Dropdown)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">公司</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">選擇要設定的公司</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">bigint ID</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">操作者可切換的公司</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.65.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K27" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.65.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B28" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.65</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C28" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">User Permission Edit Interface（BlueWhale 4.4.1.8.26）</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D28" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Branch / Department (Dropdown)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E28" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">分店／部門</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F28" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">組織歸屬（資料範圍用）</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G28" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">bigint ID，可清空</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H28" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">所選公司的啟用分店／部門</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I28" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.65.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J28" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K28" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.65.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B29" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.65</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C29" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">User Permission Edit Interface（BlueWhale 4.4.1.8.26）</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D29" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Roles (Multi-select)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E29" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">角色</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F29" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">整組取代該公司的角色</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G29" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">bigint ID 陣列</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H29" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">啟用角色；可為空（無權限）</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I29" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J29" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K29" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.65.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B30" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.65</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C30" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">User Permission Edit Interface（BlueWhale 4.4.1.8.26）</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D30" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Default Company (Checkbox)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E30" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">預設公司</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F30" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">登入後預設的操作公司</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G30" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Boolean</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H30" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">設定後取消其他預設</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I30" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J30" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K30" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.65.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B31" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.65</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C31" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">User Permission Edit Interface（BlueWhale 4.4.1.8.26）</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D31" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Access Active (Checkbox)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E31" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">啟用存取</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F31" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">停用後該公司不授權</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G31" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Boolean</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H31" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">不可停用自己</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I31" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J31" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K31" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Developer</x:t>
         </x:is>
@@ -4690,22 +5653,22 @@
       </x:c>
       <x:c r="D25" s="2" t="inlineStr">
         <x:is>
+          <x:t xml:space="preserve">4.4.1.8.64</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E25" s="2" t="inlineStr">
+        <x:is>
           <x:t xml:space="preserve"/>
         </x:is>
       </x:c>
-      <x:c r="E25" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
       <x:c r="F25" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-PERM-004, SYS-PERM-011, SYS-PERM-024</x:t>
+          <x:t xml:space="preserve">SYS-PERM-004, SYS-PERM-011, SYS-PERM-024, SYS-PERM-025</x:t>
         </x:is>
       </x:c>
       <x:c r="G25" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Partial</x:t>
+          <x:t xml:space="preserve">Covered</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -4727,22 +5690,22 @@
       </x:c>
       <x:c r="D26" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">4.4.1.8.64</x:t>
         </x:is>
       </x:c>
       <x:c r="E26" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">REQ_IO_A8.64.1, REQ_IO_A8.64.2, REQ_IO_A8.64.3, REQ_IO_A8.64.4, REQ_IO_A8.64.5</x:t>
         </x:is>
       </x:c>
       <x:c r="F26" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-PERM-011, SYS-PERM-024</x:t>
+          <x:t xml:space="preserve">SYS-PERM-011, SYS-PERM-024, SYS-PERM-025</x:t>
         </x:is>
       </x:c>
       <x:c r="G26" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Partial</x:t>
+          <x:t xml:space="preserve">Covered</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -4764,22 +5727,22 @@
       </x:c>
       <x:c r="D27" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">4.4.1.8.64</x:t>
         </x:is>
       </x:c>
       <x:c r="E27" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">REQ_IO_A8.64.2, REQ_IO_A8.64.5</x:t>
         </x:is>
       </x:c>
       <x:c r="F27" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-PERM-011, SYS-PERM-024</x:t>
+          <x:t xml:space="preserve">SYS-PERM-011, SYS-PERM-024, SYS-PERM-025</x:t>
         </x:is>
       </x:c>
       <x:c r="G27" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Partial</x:t>
+          <x:t xml:space="preserve">Covered</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -4801,22 +5764,22 @@
       </x:c>
       <x:c r="D28" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">4.4.1.8.64</x:t>
         </x:is>
       </x:c>
       <x:c r="E28" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">REQ_IO_A8.64.6</x:t>
         </x:is>
       </x:c>
       <x:c r="F28" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-PERM-012, SYS-PERM-024</x:t>
+          <x:t xml:space="preserve">SYS-PERM-012, SYS-PERM-024, SYS-PERM-025</x:t>
         </x:is>
       </x:c>
       <x:c r="G28" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Partial</x:t>
+          <x:t xml:space="preserve">Covered</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -4875,22 +5838,22 @@
       </x:c>
       <x:c r="D30" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">4.4.1.8.65</x:t>
         </x:is>
       </x:c>
       <x:c r="E30" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">REQ_IO_A8.65.1, REQ_IO_A8.65.2, REQ_IO_A8.65.3, REQ_IO_A8.65.4, REQ_IO_A8.65.5</x:t>
         </x:is>
       </x:c>
       <x:c r="F30" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-PERM-015, SYS-PERM-016, SYS-PERM-024</x:t>
+          <x:t xml:space="preserve">SYS-PERM-015, SYS-PERM-016, SYS-PERM-017, SYS-PERM-018, SYS-PERM-026, SYS-PERM-027</x:t>
         </x:is>
       </x:c>
       <x:c r="G30" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Partial</x:t>
+          <x:t xml:space="preserve">Covered</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -4926,6 +5889,302 @@
         </x:is>
       </x:c>
       <x:c r="G31" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.25.8</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B32" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to view a user's company access, organization and roles.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C32" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.92, REQ_DS43.93</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D32" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.65</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E32" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.65.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F32" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-PERM-017, SYS-PERM-018, SYS-PERM-026, SYS-PERM-027</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G32" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.26.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B33" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enforce HTTPS with HSTS outside the development environment.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C33" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="D33" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E33" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F33" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-SEC-004</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G33" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.26.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B34" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow cross-origin requests only from configured frontend origins.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C34" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="D34" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E34" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F34" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-SEC-002, SYS-SEC-003, SYS-SEC-006</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G34" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.26.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B35" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should rate-limit login, token refresh and captcha requests per client IP.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C35" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="D35" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E35" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F35" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-SEC-003, SYS-SEC-005, SYS-SEC-006, SYS-SEC-007, SYS-SEC-011, SYS-SEC-012</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G35" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.26.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B36" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should rate-limit authenticated API requests per user.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C36" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="D36" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E36" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F36" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-SEC-010</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G36" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.26.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B37" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should add security headers to every API response.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C37" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="D37" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E37" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F37" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-SEC-001, SYS-SEC-014</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G37" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.26.6</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B38" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should honour X-Forwarded-For only from configured proxies.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C38" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="D38" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E38" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F38" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-SEC-003, SYS-SEC-008, SYS-SEC-009</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G38" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.26.7</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B39" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should show a trilingual "too many requests" message when an API call is rate-limited.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C39" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="D39" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E39" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F39" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-SEC-013, SYS-SEC-014</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G39" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Partial</x:t>
         </x:is>

</xml_diff>

<commit_message>
docs(sys): document audit log backend (ADR-019) for WU-SYS-007 part 1
Adds ADR-019, REQ_F4118.27.1-6, REQ_DS43.94 sys_audit_log, audit API docs,
SYS-AUDIT test plan, optimization log entries, and updates backlog,
progress and state (audit page remains for part 2).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R3d774857c42f45a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Rc7f5663132064e7a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R309afbf6b838471e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R57122998222b4ce0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R2e150bdb38594b7d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R370a3df8acf24061"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Ra29eb8a22c69427f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="Rcfe04b2e8a5f4caf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Redfc728c80a040fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Rd2c593d0bbd14126"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R273907d1562f4530"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Rac5af4f4a32446a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Rc25761c568e64636"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R608cfff5c9fa4300"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="Rd581ee1065db474d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R90a4c51e3475470e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R5fa75bb9ba4349e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R0d72eb9cabbb4a4b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1028,7 +1028,7 @@
       </x:c>
       <x:c r="G23" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Captcha:MasterCode 只在 Development 生效且須為 4–6 位數字；其他環境有設定即寫 Error 並拒絕啟動；每次使用寫 Warning（帳號、IP），稽核日誌於 WU-SYS-007 補上。</x:t>
+          <x:t xml:space="preserve">Captcha:MasterCode 只在 Development 生效且須為 4–6 位數字；其他環境有設定即寫 Error 並拒絕啟動；每次使用寫 Warning（帳號、IP），並寫 sys_audit_log 安全事件 MASTER_CODE_LOGIN（REQ_F4118.27.3）。</x:t>
         </x:is>
       </x:c>
       <x:c r="H23" s="2" t="inlineStr">
@@ -1706,6 +1706,258 @@
       <x:c r="H39" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:102</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.27.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B40" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C40" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Audit Log</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D40" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E40" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should record every data change in sys_audit_log within the same transaction.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F40" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G40" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">透過 EF 新增、修改、刪除（含軟刪除）都寫一筆記錄，內容包括公司、用戶（背景程序為系統用戶）、時間（IClock）、表名、記錄 Id、操作類型（CREATE／UPDATE／DELETE，可由 Application 指定 VOID／APPROVE／POST）、欄位差異 JSON（修改只列有變更的欄位）、來源 IP、TraceId。沒有欄位變更不寫記錄。交易回滾或 SaveChanges 失敗（含樂觀鎖衝突）不留記錄，重試時也不會重複（ADR-019）。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H40" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:114</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.27.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B41" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C41" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Audit Log</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D41" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E41" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should protect audit records and sensitive values.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F41" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G41" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">[SensitiveData] 欄位（例如 password_hash）的值以 * 遮蔽；主鍵、審計欄位、version、company_id 不記錄差異。sys_audit_log 只能新增，UPDATE 或 DELETE 由 trigger 拒絕（append-only）；changes 必須是 JSON。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H41" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:115</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.27.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B42" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C42" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Audit Log</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D42" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E42" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should record login, failed login, logout and captcha master-code login as security events.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F42" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G42" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">安全事件記錄帳號、IP、時間與 TraceId。LOGIN_FAILED 的原因只寫 INVALID_CREDENTIALS 或 PASSWORD_EXPIRED，不寫密碼。萬用碼登入不論結果都寫 MASTER_CODE_LOGIN（REQ_F4118.24.4）。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H42" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:116</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.27.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B43" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C43" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Audit Log</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D43" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E43" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to query audit logs of the current company.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F43" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G43" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">GET /api/v1/sys/audit-logs 需 SYS.AUDIT.VIEW，支援分頁、日期範圍（含頭尾）、類別、操作類型、表名＋記錄 Id（單據修改歷史）、用戶篩選，以時間排序。只列出目前公司的記錄，以及屬於目前公司用戶、沒有公司的安全事件；其他公司的記錄看不到。資料變更記錄會補上帳號。to 早於 from、類別未知或長度超限時回 400。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H43" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:117</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.27.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B44" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C44" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Audit Log</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D44" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E44" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should record role permission and user company access changes as security events.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F44" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G44" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">修改角色的權限、資料範圍、全權或啟用狀態，以及指派用戶公司授權，都寫 PERMISSION_CHANGE，與變更同一交易。記錄內容包括操作者、公司、新增與移除的權限，或指派後的角色、組織、預設公司與啟用狀態。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H44" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:118</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.27.6</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B45" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C45" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Audit Log</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D45" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E45" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should provide a trilingual audit log page with per-record change history.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F45" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G45" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">待第二段：三語稽核查詢頁（介面 8.66），可用篩選條件查詢，可展開欄位差異，並支援從單據查看修改歷史。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H45" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:119</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -2941,6 +3193,38 @@
       <x:c r="F9" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">REQ_F4118.25.6, REQ_F4118.25.7, REQ_F4118.25.8</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.94</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B10" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C10" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">sys_audit_log</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D10" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Append-only audit trail of data changes (field old/new values) and security events, with company, user, IP and trace id.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E10" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F10" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.27.1, REQ_F4118.27.2, REQ_F4118.27.3, REQ_F4118.27.4, REQ_F4118.27.5</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -6190,6 +6474,228 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.27.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B40" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should record every data change in sys_audit_log within the same transaction.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C40" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.94</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D40" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E40" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F40" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-AUDIT-001, SYS-AUDIT-002, SYS-AUDIT-003, SYS-AUDIT-004, SYS-AUDIT-005, SYS-AUDIT-006, SYS-AUDIT-010</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G40" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.27.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B41" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should protect audit records and sensitive values.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C41" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.94</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D41" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E41" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F41" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-AUDIT-003, SYS-AUDIT-008, SYS-AUDIT-011</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G41" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.27.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B42" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should record login, failed login, logout and captcha master-code login as security events.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C42" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.94</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D42" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E42" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F42" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-AUDIT-007, SYS-AUDIT-012</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G42" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.27.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B43" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to query audit logs of the current company.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C43" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.94</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D43" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E43" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F43" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-AUDIT-009, SYS-AUDIT-010</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G43" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.27.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B44" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should record role permission and user company access changes as security events.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C44" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.94</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D44" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E44" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F44" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-AUDIT-013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G44" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.27.6</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B45" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should provide a trilingual audit log page with per-record change history.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C45" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="D45" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E45" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F45" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-AUDIT-014</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G45" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
   </x:sheetData>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
docs(sys): document audit log page and complete WU-SYS-007
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Rd2c593d0bbd14126"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R273907d1562f4530"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Rac5af4f4a32446a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Rc25761c568e64636"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R608cfff5c9fa4300"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="Rd581ee1065db474d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R90a4c51e3475470e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R5fa75bb9ba4349e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R0d72eb9cabbb4a4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R0160f9f877f748f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R79f644a96dcd46b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Rb6b61804eb684750"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R3c5b21c9e5aa4814"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R5d5be2b6fd91449d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="Rb8338e706f51440b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R667e0de5a86a4bcc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R0db5d66091f44454"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R40c545e409324e32"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1952,7 +1952,7 @@
       </x:c>
       <x:c r="G45" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">待第二段：三語稽核查詢頁（介面 8.66），可用篩選條件查詢，可展開欄位差異，並支援從單據查看修改歷史。</x:t>
+          <x:t xml:space="preserve">三語稽核查詢頁 /sys/audit-logs（介面 8.66），需 SYS.AUDIT.VIEW，無權限時選單不顯示、直接進入顯示 403。可依日期範圍（含快選今天、近 7、30 天；結束日早於開始日時不送出）、類別、操作、資料表＋記錄 ID 篩選，伺服器端分頁並依時間排序。可展開欄位差異（修改前→修改後，* 照原樣顯示）或安全事件明細。?tableName=&amp;recordId= 開啟單筆記錄的修改歷史，供單據頁的稽核頁籤連結。操作與類別有三語標籤，未知操作顯示原代碼。切換公司後重新查詢。</x:t>
         </x:is>
       </x:c>
       <x:c r="H45" s="2" t="inlineStr">
@@ -3224,7 +3224,7 @@
       </x:c>
       <x:c r="F10" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.27.1, REQ_F4118.27.2, REQ_F4118.27.3, REQ_F4118.27.4, REQ_F4118.27.5</x:t>
+          <x:t xml:space="preserve">REQ_F4118.27.1, REQ_F4118.27.2, REQ_F4118.27.3, REQ_F4118.27.4, REQ_F4118.27.5, REQ_F4118.27.6</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -3238,10 +3238,10 @@
     <x:col min="1" max="1" width="16" customWidth="1"/>
     <x:col min="2" max="2" width="15" customWidth="1"/>
     <x:col min="3" max="3" width="54" customWidth="1"/>
-    <x:col min="4" max="4" width="32" customWidth="1"/>
+    <x:col min="4" max="4" width="42" customWidth="1"/>
     <x:col min="5" max="5" width="13" customWidth="1"/>
     <x:col min="6" max="6" width="23" customWidth="1"/>
-    <x:col min="7" max="7" width="40" customWidth="1"/>
+    <x:col min="7" max="7" width="60" customWidth="1"/>
     <x:col min="8" max="8" width="60" customWidth="1"/>
     <x:col min="9" max="9" width="16" customWidth="1"/>
     <x:col min="10" max="10" width="10" customWidth="1"/>
@@ -5010,6 +5010,348 @@
         </x:is>
       </x:c>
       <x:c r="K31" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.66.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B32" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.66</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C32" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Audit Log Query Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D32" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Date Range (Date inputs + quick buttons)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E32" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">開始／結束日期</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F32" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">限制查詢期間</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G32" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">yyyy-MM-dd</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H32" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">含頭尾；結束日不可早於開始日；快選今天、近 7、30 天</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I32" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J32" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K32" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.66.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B33" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.66</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C33" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Audit Log Query Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D33" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Category (Dropdown)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E33" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">類別</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F33" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">區分資料變更與安全事件</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G33" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">DATA／SECURITY</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H33" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">可清空</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I33" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J33" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K33" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.66.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B34" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.66</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C34" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Audit Log Query Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D34" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Action (Dropdown)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E34" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">操作</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F34" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">依操作類型篩選</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G34" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">CREATE、UPDATE、DELETE、VOID、APPROVE、POST、LOGIN、LOGIN_FAILED、MASTER_CODE_LOGIN、LOGOUT、PERMISSION_CHANGE、EXPORT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H34" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">可清空</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I34" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J34" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K34" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.66.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B35" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.66</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C35" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Audit Log Query Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D35" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Table / Record ID (Input)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E35" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">資料表、記錄 ID</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F35" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">查看單據修改歷史</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G35" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Text</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H35" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">資料表最多 128 字元、記錄 ID 最多 100 字元；去除前後空白</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I35" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.66.6</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J35" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K35" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.66.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B36" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.66</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C36" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Audit Log Query Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D36" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Changes (Expandable row)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E36" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">欄位差異</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F36" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">顯示修改前後的值</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G36" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">欄位／修改前／修改後</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H36" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">敏感欄位顯示 *；空值顯示「（空）」</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I36" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J36" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K36" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.66.6</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B37" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.66</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C37" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Audit Log Query Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D37" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Record History (Link / query string)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E37" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">修改歷史</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F37" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">由單據或列開啟單筆記錄歷史</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G37" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">?tableName=&amp;recordId=</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H37" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">安全事件沒有記錄 ID，不可開啟</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I37" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.66.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J37" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K37" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Developer</x:t>
         </x:is>
@@ -6534,7 +6876,7 @@
       </x:c>
       <x:c r="E41" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">REQ_IO_A8.66.5</x:t>
         </x:is>
       </x:c>
       <x:c r="F41" s="2" t="inlineStr">
@@ -6544,7 +6886,7 @@
       </x:c>
       <x:c r="G41" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Partial</x:t>
+          <x:t xml:space="preserve">Covered</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -6603,12 +6945,12 @@
       </x:c>
       <x:c r="D43" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">4.4.1.8.66</x:t>
         </x:is>
       </x:c>
       <x:c r="E43" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">REQ_IO_A8.66.1</x:t>
         </x:is>
       </x:c>
       <x:c r="F43" s="2" t="inlineStr">
@@ -6618,7 +6960,7 @@
       </x:c>
       <x:c r="G43" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Partial</x:t>
+          <x:t xml:space="preserve">Covered</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -6672,17 +7014,17 @@
       </x:c>
       <x:c r="C45" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">REQ_DS43.94</x:t>
         </x:is>
       </x:c>
       <x:c r="D45" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">4.4.1.8.66</x:t>
         </x:is>
       </x:c>
       <x:c r="E45" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">REQ_IO_A8.66.1, REQ_IO_A8.66.2, REQ_IO_A8.66.3, REQ_IO_A8.66.4, REQ_IO_A8.66.5, REQ_IO_A8.66.6</x:t>
         </x:is>
       </x:c>
       <x:c r="F45" s="2" t="inlineStr">
@@ -6692,7 +7034,7 @@
       </x:c>
       <x:c r="G45" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Partial</x:t>
+          <x:t xml:space="preserve">Covered</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
feat(sys): add document number rules with concurrency-safe generator
WU-SYS-008 part 1: sys_number_rule / sys_number_sequence (REQ_DS43.95-96),
shared INumberGenerator implemented by an atomic MERGE WITH (HOLDLOCK) inside
the caller's transaction (no duplicates, no gaps on rollback, ADR-021),
number rule management API and 9 integration tests (REQ_F4118.28.1-5).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R0160f9f877f748f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R79f644a96dcd46b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Rb6b61804eb684750"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R3c5b21c9e5aa4814"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R5d5be2b6fd91449d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="Rb8338e706f51440b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R667e0de5a86a4bcc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R0db5d66091f44454"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R40c545e409324e32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Rc570eda35bf6429e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R854030b7482948a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Re6032a99bb98458f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R4ce832cd45d74977"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R49b03cd0c4d148a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R01b9977fee3645ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R48e32ff94c214d9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R2847e4b2f2754818"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rc12e25fcfb3546c5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1961,6 +1961,258 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.28.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B46" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C46" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Document Number Rule</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D46" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E46" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow user to view document number rules of the current company.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F46" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G46" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="H46" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:132</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.28.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B47" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C47" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Document Number Rule</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D47" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E47" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow user to create a document number rule with prefix, date format, sequence length and reset period.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F47" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G47" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="H47" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:133</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.28.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B48" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C48" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Document Number Rule</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D48" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E48" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow user to edit or deactivate a document number rule without breaking issued numbers.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F48" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G48" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="H48" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:134</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.28.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B49" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C49" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Document Number Rule</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D49" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E49" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow user to preview the next document number for a business date.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F49" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G49" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="H49" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:135</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.28.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B50" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C50" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Document Number Rule</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D50" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E50" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should generate unique, gap-free document numbers for every module under concurrency.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F50" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G50" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="H50" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:136</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.28.6</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B51" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C51" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Document Number Rule</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D51" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E51" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should provide a trilingual number rule maintenance page.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F51" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G51" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="H51" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:137</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
   </x:sheetData>
 </x:worksheet>
 </file>
@@ -3225,6 +3477,70 @@
       <x:c r="F10" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">REQ_F4118.27.1, REQ_F4118.27.2, REQ_F4118.27.3, REQ_F4118.27.4, REQ_F4118.27.5, REQ_F4118.27.6</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.95</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B11" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C11" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">sys_number_rule</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D11" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Document number rule per company and document type: prefix, date format, sequence length, reset period and active flag.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E11" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F11" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.28.1, REQ_F4118.28.2, REQ_F4118.28.3, REQ_F4118.28.4, REQ_F4118.28.5</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.96</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B12" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C12" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">sys_number_sequence</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D12" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Running sequence counter per number rule and reset period, updated atomically when a number is issued.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E12" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F12" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.28.3, REQ_F4118.28.4, REQ_F4118.28.5</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -5370,7 +5686,7 @@
     <x:col min="4" max="4" width="12" customWidth="1"/>
     <x:col min="5" max="5" width="60" customWidth="1"/>
     <x:col min="6" max="6" width="60" customWidth="1"/>
-    <x:col min="7" max="7" width="10" customWidth="1"/>
+    <x:col min="7" max="7" width="13" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -7035,6 +7351,228 @@
       <x:c r="G45" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.28.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B46" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow user to view document number rules of the current company.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C46" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.95</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D46" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E46" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F46" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-NUM-006, SYS-NUM-008</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G46" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.28.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B47" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow user to create a document number rule with prefix, date format, sequence length and reset period.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C47" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.95</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D47" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E47" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F47" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-NUM-006, SYS-NUM-007, SYS-NUM-008</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G47" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.28.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B48" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow user to edit or deactivate a document number rule without breaking issued numbers.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C48" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.95, REQ_DS43.96</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D48" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E48" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F48" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-NUM-006, SYS-NUM-008, SYS-NUM-009</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G48" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.28.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B49" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow user to preview the next document number for a business date.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C49" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.95, REQ_DS43.96</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D49" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E49" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F49" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-NUM-006, SYS-NUM-008</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G49" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.28.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B50" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should generate unique, gap-free document numbers for every module under concurrency.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C50" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.95, REQ_DS43.96</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D50" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E50" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F50" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-NUM-001, SYS-NUM-002, SYS-NUM-003, SYS-NUM-004, SYS-NUM-005, SYS-NUM-009</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G50" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.28.6</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B51" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should provide a trilingual number rule maintenance page.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C51" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="D51" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E51" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F51" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="G51" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Not covered</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
refactor(sys): require whole-number sequence length and document number rule page
- shared sequenceLengthValidators with integer check and step=1
- extra tests: decimal length, 404 and over-long name on edit
- ui-spec interface 8.67 (REQ_IO_A8.67.1-9), test-plan SYS-NUM-010/011,
  requirements, optimization log, trace REQ_F4118.28.6 to REQ_DS43.95
- regenerate docgen output (0 errors)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Rc570eda35bf6429e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R854030b7482948a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Re6032a99bb98458f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R4ce832cd45d74977"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R49b03cd0c4d148a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R01b9977fee3645ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R48e32ff94c214d9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R2847e4b2f2754818"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rc12e25fcfb3546c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R4484eb9e401d42dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Rda699110a72945d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R33275d44c5a34e3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R76b67ad55c5b4430"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R668c5f6cf1d4465a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R5b2e7626cc464fe1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R122bcbbe87b4458c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R201716bea0474bcf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Reb0e219635e04bc7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3508,7 +3508,7 @@
       </x:c>
       <x:c r="F11" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.28.1, REQ_F4118.28.2, REQ_F4118.28.3, REQ_F4118.28.4, REQ_F4118.28.5</x:t>
+          <x:t xml:space="preserve">REQ_F4118.28.1, REQ_F4118.28.2, REQ_F4118.28.3, REQ_F4118.28.4, REQ_F4118.28.5, REQ_F4118.28.6</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -5673,6 +5673,519 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.67.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B38" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.67</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C38" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Document Number Rule Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D38" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Document Type (Input)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E38" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">單據類型</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F38" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">識別規則所屬單據</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G38" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">{PREFIX}.{DOCUMENT}，例如 SD.ORDER</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H38" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">英文字母、數字、底線，最多 50 字；保存為大寫；公司內唯一；建立後不可修改</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I38" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J38" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K38" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.67.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B39" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.67</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C39" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Document Number Rule Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D39" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Name (Input)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E39" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">名稱</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F39" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">規則說明</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G39" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Text</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H39" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1–100 字元，去除前後空白</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I39" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J39" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K39" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.67.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B40" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.67</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C40" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Document Number Rule Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D40" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Prefix (Input)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E40" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">前綴</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F40" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">單號開頭</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G40" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Text</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H40" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">0–10 個英數字、-、_；保存為大寫</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I40" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.67.7</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J40" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K40" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.67.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B41" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.67</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C41" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Document Number Rule Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D41" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Date Format (Dropdown)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E41" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">日期格式</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F41" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">單號的日期部分</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G41" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None／yyyy／yyyyMM／yyyyMMdd／yyMM／yyMMdd</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H41" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">已發號時不可修改</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I41" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.67.6</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J41" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K41" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.67.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B42" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.67</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C42" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Document Number Rule Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D42" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Sequence Length (Number)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E42" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">流水號長度</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F42" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">補零位數</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G42" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">整數</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H42" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">3–10；已發號時不可小於原長度</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I42" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.67.7</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J42" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K42" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.67.6</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B43" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.67</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C43" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Document Number Rule Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D43" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Reset Period (Dropdown)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E43" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">重設週期</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F43" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">流水號歸 1 的時機</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G43" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">不重設／每年／每月／每日</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H43" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">必須包含在日期格式內；已發號時不可修改</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I43" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.67.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J43" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K43" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.67.7</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B44" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.67</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C44" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Document Number Rule Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D44" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Sample (Text)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E44" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">樣式</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F44" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">即時顯示今天第 1 號</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G44" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">前綴＋日期＋補零流水號</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H44" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">唯讀</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I44" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.67.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J44" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K44" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.67.8</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B45" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.67</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C45" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Document Number Rule Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D45" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Active (Checkbox)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E45" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">啟用</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F45" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">停用後各模組不可再取號</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G45" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Boolean</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H45" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">只在編輯時顯示</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I45" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J45" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K45" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.67.9</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B46" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.67</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C46" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Document Number Rule Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D46" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Preview Date (Date input)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E46" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">單據日期</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F46" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">預覽該日期的下一個單號</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G46" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">yyyy-MM-dd</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H46" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">預設今天；可清空（後端用今天）；不佔號</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I46" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J46" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K46" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
   </x:sheetData>
 </x:worksheet>
 </file>
@@ -5686,7 +6199,7 @@
     <x:col min="4" max="4" width="12" customWidth="1"/>
     <x:col min="5" max="5" width="60" customWidth="1"/>
     <x:col min="6" max="6" width="60" customWidth="1"/>
-    <x:col min="7" max="7" width="13" customWidth="1"/>
+    <x:col min="7" max="7" width="10" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -7372,22 +7885,22 @@
       </x:c>
       <x:c r="D46" s="2" t="inlineStr">
         <x:is>
+          <x:t xml:space="preserve">4.4.1.8.67</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E46" s="2" t="inlineStr">
+        <x:is>
           <x:t xml:space="preserve"/>
         </x:is>
       </x:c>
-      <x:c r="E46" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
       <x:c r="F46" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-NUM-006, SYS-NUM-008</x:t>
+          <x:t xml:space="preserve">SYS-NUM-006, SYS-NUM-008, SYS-NUM-010</x:t>
         </x:is>
       </x:c>
       <x:c r="G46" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Partial</x:t>
+          <x:t xml:space="preserve">Covered</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -7409,22 +7922,22 @@
       </x:c>
       <x:c r="D47" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">4.4.1.8.67</x:t>
         </x:is>
       </x:c>
       <x:c r="E47" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">REQ_IO_A8.67.1, REQ_IO_A8.67.2, REQ_IO_A8.67.3, REQ_IO_A8.67.4, REQ_IO_A8.67.5, REQ_IO_A8.67.6</x:t>
         </x:is>
       </x:c>
       <x:c r="F47" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-NUM-006, SYS-NUM-007, SYS-NUM-008</x:t>
+          <x:t xml:space="preserve">SYS-NUM-006, SYS-NUM-007, SYS-NUM-008, SYS-NUM-010, SYS-NUM-011</x:t>
         </x:is>
       </x:c>
       <x:c r="G47" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Partial</x:t>
+          <x:t xml:space="preserve">Covered</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -7446,22 +7959,22 @@
       </x:c>
       <x:c r="D48" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">4.4.1.8.67</x:t>
         </x:is>
       </x:c>
       <x:c r="E48" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">REQ_IO_A8.67.2, REQ_IO_A8.67.3, REQ_IO_A8.67.4, REQ_IO_A8.67.5, REQ_IO_A8.67.6, REQ_IO_A8.67.8</x:t>
         </x:is>
       </x:c>
       <x:c r="F48" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-NUM-006, SYS-NUM-008, SYS-NUM-009</x:t>
+          <x:t xml:space="preserve">SYS-NUM-006, SYS-NUM-008, SYS-NUM-009, SYS-NUM-010, SYS-NUM-011</x:t>
         </x:is>
       </x:c>
       <x:c r="G48" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Partial</x:t>
+          <x:t xml:space="preserve">Covered</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -7483,22 +7996,22 @@
       </x:c>
       <x:c r="D49" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">4.4.1.8.67</x:t>
         </x:is>
       </x:c>
       <x:c r="E49" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">REQ_IO_A8.67.9</x:t>
         </x:is>
       </x:c>
       <x:c r="F49" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-NUM-006, SYS-NUM-008</x:t>
+          <x:t xml:space="preserve">SYS-NUM-006, SYS-NUM-008, SYS-NUM-010, SYS-NUM-011</x:t>
         </x:is>
       </x:c>
       <x:c r="G49" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Partial</x:t>
+          <x:t xml:space="preserve">Covered</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -7552,27 +8065,27 @@
       </x:c>
       <x:c r="C51" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">REQ_DS43.95</x:t>
         </x:is>
       </x:c>
       <x:c r="D51" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">4.4.1.8.67</x:t>
         </x:is>
       </x:c>
       <x:c r="E51" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">REQ_IO_A8.67.1, REQ_IO_A8.67.7</x:t>
         </x:is>
       </x:c>
       <x:c r="F51" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">SYS-NUM-010, SYS-NUM-011</x:t>
         </x:is>
       </x:c>
       <x:c r="G51" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not covered</x:t>
+          <x:t xml:space="preserve">Covered</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
feat(sys): add trilingual approval flow, delegation and inbox pages (WU-SYS-009 part 2)
Interfaces 8.68-8.70: multi-step flow editor with role/user approvers
and amount thresholds, delegation maintenance, and an approval inbox
with approve/reject and history. Menu items accept any of several
permissions; tasks now return the delegator username.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R4484eb9e401d42dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Rda699110a72945d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R33275d44c5a34e3d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R76b67ad55c5b4430"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R668c5f6cf1d4465a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R5b2e7626cc464fe1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R122bcbbe87b4458c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R201716bea0474bcf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Reb0e219635e04bc7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R8a9a72e8b02c4c69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Rc6df7f0a79b84077"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R10fb1a1c96c94949"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Rd3e86666e15f4683"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R4d657a0aa340424e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R34090fe3330d4462"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R58ba9181f4334e76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="Rdfa9fec9ace84aff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R3e9de798a3a240e6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1999,7 +1999,7 @@
       </x:c>
       <x:c r="H46" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:132</x:t>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:153</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -2041,7 +2041,7 @@
       </x:c>
       <x:c r="H47" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:133</x:t>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:154</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -2083,7 +2083,7 @@
       </x:c>
       <x:c r="H48" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:134</x:t>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:155</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -2125,7 +2125,7 @@
       </x:c>
       <x:c r="H49" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:135</x:t>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:156</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -2167,7 +2167,7 @@
       </x:c>
       <x:c r="H50" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:136</x:t>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:157</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -2209,7 +2209,385 @@
       </x:c>
       <x:c r="H51" s="2" t="inlineStr">
         <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:158</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.29.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B52" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C52" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Approval Workflow</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D52" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E52" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow user to view and create multi-level approval flows with amount thresholds.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F52" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G52" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="H52" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:132</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.29.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B53" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C53" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Approval Workflow</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D53" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E53" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow user to edit or deactivate an approval flow without affecting pending approvals.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F53" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G53" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="H53" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:133</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.29.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B54" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C54" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Approval Workflow</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D54" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E54" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow user to assign an approval delegate for a date range.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F54" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G54" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="H54" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:134</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.29.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B55" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C55" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Approval Workflow</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D55" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E55" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable every module to submit documents for approval through the shared workflow engine.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F55" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G55" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="H55" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:135</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.29.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B56" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C56" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Approval Workflow</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D56" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E56" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow approvers or their delegates to approve or reject the current approval step.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F56" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G56" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="H56" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:136</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.29.6</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B57" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C57" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Approval Workflow</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D57" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E57" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should list the pending approval tasks of the current user.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F57" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G57" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="H57" s="2" t="inlineStr">
+        <x:is>
           <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:137</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.29.7</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B58" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C58" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Approval Workflow</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D58" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E58" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow user to view the approval history of a document.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F58" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G58" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="H58" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:138</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.29.8</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B59" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C59" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Approval Workflow</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D59" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E59" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should provide trilingual approval flow and delegation maintenance pages.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F59" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G59" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="H59" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:139</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.29.9</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B60" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C60" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Approval Workflow</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D60" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E60" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should provide a trilingual approval inbox with approval history.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F60" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G60" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="H60" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:140</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -3154,7 +3532,7 @@
   <x:cols>
     <x:col min="1" max="1" width="16" customWidth="1"/>
     <x:col min="2" max="2" width="10" customWidth="1"/>
-    <x:col min="3" max="3" width="21" customWidth="1"/>
+    <x:col min="3" max="3" width="28" customWidth="1"/>
     <x:col min="4" max="4" width="60" customWidth="1"/>
     <x:col min="5" max="5" width="11" customWidth="1"/>
     <x:col min="6" max="6" width="60" customWidth="1"/>
@@ -3541,6 +3919,166 @@
       <x:c r="F12" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">REQ_F4118.28.3, REQ_F4118.28.4, REQ_F4118.28.5</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.97</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B13" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C13" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">sys_approval_flow</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D13" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Approval flow per company and document type, with the self-approval setting and active flag.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E13" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F13" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.29.1, REQ_F4118.29.2, REQ_F4118.29.4, REQ_F4118.29.8</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.98</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">sys_approval_flow_step</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Ordered steps of an approval flow: approver role or user and the optional minimum amount that makes the step apply.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F14" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.29.1, REQ_F4118.29.2, REQ_F4118.29.4, REQ_F4118.29.8</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.99</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B15" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C15" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">sys_approval_delegation</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D15" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Approval delegation from one user to another within a date range.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E15" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F15" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.29.3, REQ_F4118.29.5, REQ_F4118.29.6, REQ_F4118.29.8</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.100</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B16" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C16" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">sys_approval_instance</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D16" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">One submission of a document for approval: document reference, amount, status, current step, submitter and completion time.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E16" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F16" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.29.4, REQ_F4118.29.5, REQ_F4118.29.6, REQ_F4118.29.7, REQ_F4118.29.9</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.101</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B17" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C17" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">sys_approval_instance_step</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D17" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Snapshot of the applicable flow steps of an approval instance with each step's decision, actor, delegator, time and comment.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E17" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F17" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.29.4, REQ_F4118.29.5, REQ_F4118.29.6, REQ_F4118.29.7, REQ_F4118.29.9</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -6186,6 +6724,804 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.68.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B47" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.68</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C47" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Approval Flow Maintenance Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D47" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Document Type (Input)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E47" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">單據類型</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F47" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">流程所屬單據</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G47" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">{PREFIX}.{DOCUMENT}，例如 PUR.ORDER</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H47" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">英文字母、數字、底線，最多 50 字；保存為大寫；公司內唯一；建立後不可修改</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I47" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J47" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K47" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.68.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B48" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.68</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C48" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Approval Flow Maintenance Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D48" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Flow Name (Input)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E48" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">流程名稱</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F48" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">流程說明</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G48" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Text</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H48" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1–100 字元，去除前後空白</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I48" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J48" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K48" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.68.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B49" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.68</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C49" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Approval Flow Maintenance Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D49" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Allow Self-approval (Checkbox)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E49" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">允許自審</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F49" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">送審人可否審批自己的單據</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G49" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Boolean</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H49" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">預設否</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I49" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J49" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K49" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.68.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B50" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.68</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C50" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Approval Flow Maintenance Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D50" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Step Name (Input)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E50" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">步驟名稱</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F50" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">顯示於待辦與記錄</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G50" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Text</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H50" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1–100 字元</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I50" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J50" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K50" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.68.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B51" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.68</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C51" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Approval Flow Maintenance Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D51" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Approver Type (Dropdown)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E51" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">審批人類型</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F51" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">角色或指定用戶</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G51" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Role／User</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H51" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">必填</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I51" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.68.6</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J51" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K51" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.68.6</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B52" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.68</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C52" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Approval Flow Maintenance Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D52" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Approver (Dropdown)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E52" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">審批人</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F52" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">處理該步驟的角色或用戶</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G52" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">bigint ID</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H52" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">啟用角色或本公司啟用用戶</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I52" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.68.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J52" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K52" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.68.7</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B53" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.68</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C53" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Approval Flow Maintenance Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D53" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Minimum Amount (Input)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E53" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">最低金額</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F53" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">金額門檻（本位幣）</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G53" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">數字</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H53" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">選填；≥ 0，最多 11 位整數、4 位小數</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I53" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J53" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K53" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.68.8</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B54" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.68</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C54" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Approval Flow Maintenance Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D54" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Active (Checkbox)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E54" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">啟用</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F54" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">停用後送審自動核准</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G54" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Boolean</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H54" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">只在編輯時顯示</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I54" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J54" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K54" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.69.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B55" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.69</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C55" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Approval Delegation Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D55" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Delegator (Dropdown)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E55" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">被代理人</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F55" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">交出審批工作的用戶</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G55" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">bigint ID</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H55" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">本公司啟用用戶；建立後不可修改</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I55" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.69.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J55" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K55" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.69.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B56" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.69</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C56" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Approval Delegation Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D56" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Delegate (Dropdown)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E56" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">代理人</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F56" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">代為審批的用戶</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G56" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">bigint ID</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H56" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">本公司啟用用戶，不可與被代理人相同；建立後不可修改</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I56" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.69.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J56" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K56" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.69.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B57" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.69</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C57" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Approval Delegation Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D57" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Start / End Date (Date input)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E57" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">開始／結束日期</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F57" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">代理期間（含頭尾）</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G57" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">yyyy-MM-dd</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H57" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">結束不早於開始；同一被代理人的啟用期間不可重疊</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I57" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J57" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K57" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.69.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B58" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.69</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C58" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Approval Delegation Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D58" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Remark (Textarea)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E58" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">備註</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F58" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">代理原因</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G58" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Text</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H58" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">0–200 字元</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I58" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J58" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K58" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.70.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B59" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.70</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C59" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Approval Inbox Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D59" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Comment (Textarea)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E59" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">意見</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F59" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">核准或駁回的說明</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G59" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Text</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H59" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">0–500 字元；駁回必填</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I59" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J59" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K59" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.70.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B60" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.70</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C60" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Approval Inbox Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D60" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Status Filter (Dropdown)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E60" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">狀態</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F60" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">篩選審批歷史</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G60" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">審批中／已核准／已駁回／已撤回</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H60" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">可清除</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I60" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J60" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K60" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
   </x:sheetData>
 </x:worksheet>
 </file>
@@ -6195,8 +7531,8 @@
   <x:cols>
     <x:col min="1" max="1" width="16" customWidth="1"/>
     <x:col min="2" max="2" width="60" customWidth="1"/>
-    <x:col min="3" max="3" width="39" customWidth="1"/>
-    <x:col min="4" max="4" width="12" customWidth="1"/>
+    <x:col min="3" max="3" width="54" customWidth="1"/>
+    <x:col min="4" max="4" width="24" customWidth="1"/>
     <x:col min="5" max="5" width="60" customWidth="1"/>
     <x:col min="6" max="6" width="60" customWidth="1"/>
     <x:col min="7" max="7" width="10" customWidth="1"/>
@@ -8084,6 +9420,339 @@
         </x:is>
       </x:c>
       <x:c r="G51" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.29.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B52" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow user to view and create multi-level approval flows with amount thresholds.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C52" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.97, REQ_DS43.98</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D52" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.68</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E52" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.68.1, REQ_IO_A8.68.2, REQ_IO_A8.68.3, REQ_IO_A8.68.4, REQ_IO_A8.68.5, REQ_IO_A8.68.6, REQ_IO_A8.68.7</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F52" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-APR-008, SYS-APR-010, SYS-APR-012, SYS-APR-013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G52" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.29.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B53" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow user to edit or deactivate an approval flow without affecting pending approvals.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C53" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.97, REQ_DS43.98</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D53" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.68</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E53" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.68.2, REQ_IO_A8.68.3, REQ_IO_A8.68.8</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F53" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-APR-003, SYS-APR-008, SYS-APR-010, SYS-APR-012, SYS-APR-013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G53" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.29.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B54" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow user to assign an approval delegate for a date range.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C54" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.99</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D54" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.69</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E54" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.69.1, REQ_IO_A8.69.2, REQ_IO_A8.69.3, REQ_IO_A8.69.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F54" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-APR-005, SYS-APR-010, SYS-APR-012, SYS-APR-013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G54" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.29.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B55" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable every module to submit documents for approval through the shared workflow engine.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C55" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.97, REQ_DS43.98, REQ_DS43.100, REQ_DS43.101</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D55" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E55" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F55" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-APR-001, SYS-APR-002, SYS-APR-003, SYS-APR-007, SYS-APR-011</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G55" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.29.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B56" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow approvers or their delegates to approve or reject the current approval step.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C56" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.99, REQ_DS43.100, REQ_DS43.101</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D56" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.70</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E56" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.70.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F56" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-APR-001, SYS-APR-002, SYS-APR-004, SYS-APR-005, SYS-APR-006, SYS-APR-007, SYS-APR-011, SYS-APR-012, SYS-APR-013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G56" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.29.6</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B57" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should list the pending approval tasks of the current user.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C57" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.99, REQ_DS43.100, REQ_DS43.101</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D57" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.70</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E57" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F57" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-APR-004, SYS-APR-005, SYS-APR-011, SYS-APR-012, SYS-APR-013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G57" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.29.7</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B58" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow user to view the approval history of a document.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C58" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.100, REQ_DS43.101</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D58" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.70</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E58" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.70.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F58" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-APR-001, SYS-APR-002, SYS-APR-008, SYS-APR-011, SYS-APR-012, SYS-APR-013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G58" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.29.8</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B59" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should provide trilingual approval flow and delegation maintenance pages.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C59" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.97, REQ_DS43.98, REQ_DS43.99</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D59" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.68, 4.4.1.8.69</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E59" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.68.1, REQ_IO_A8.68.4, REQ_IO_A8.68.5, REQ_IO_A8.68.6, REQ_IO_A8.68.7</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F59" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-APR-012, SYS-APR-013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G59" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.29.9</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B60" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should provide a trilingual approval inbox with approval history.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C60" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.100, REQ_DS43.101</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D60" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.70</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E60" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.70.1, REQ_IO_A8.70.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F60" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-APR-012, SYS-APR-013</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G60" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Covered</x:t>
         </x:is>

</xml_diff>

<commit_message>
docs(sys): complete WU-SYS-013 seed data (ADR-023) and update progress
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R8a9a72e8b02c4c69"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Rc6df7f0a79b84077"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R10fb1a1c96c94949"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Rd3e86666e15f4683"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R4d657a0aa340424e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R34090fe3330d4462"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R58ba9181f4334e76"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="Rdfa9fec9ace84aff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R3e9de798a3a240e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Re6ad69b918224735"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Ra7e0587e88734a7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R423e4857fb234118"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Rc6d76449e44e44f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R23ab5dcbf37a43de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R30c151c9f1d643f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R99918af3ec494258"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="Rde99fb97f5d249a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R06a8653ffa9849c8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2591,6 +2591,132 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="61">
+      <x:c r="A61" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.30.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B61" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C61" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Development Seed Data</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D61" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E61" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should load demo companies, branches, departments and roles for the Development environment.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F61" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G61" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="H61" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:172</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.30.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B62" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C62" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Development Seed Data</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D62" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E62" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should create the test accounts of the SeedUsers setting with hashed passwords and company assignments.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F62" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G62" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="H62" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:173</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.30.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B63" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C63" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Development Seed Data</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D63" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E63" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow the seed to run repeatedly without duplicating or overwriting data.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F63" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G63" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="H63" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:174</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
   </x:sheetData>
 </x:worksheet>
 </file>
@@ -3598,7 +3724,7 @@
       </x:c>
       <x:c r="F2" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.20.1, REQ_F4118.20.2, REQ_F4118.20.3, REQ_F4118.20.4</x:t>
+          <x:t xml:space="preserve">REQ_F4118.20.1, REQ_F4118.20.2, REQ_F4118.20.3, REQ_F4118.20.4, REQ_F4118.30.1, REQ_F4118.30.3</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -3630,7 +3756,7 @@
       </x:c>
       <x:c r="F3" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.22.1, REQ_F4118.22.2, REQ_F4118.22.3</x:t>
+          <x:t xml:space="preserve">REQ_F4118.22.1, REQ_F4118.22.2, REQ_F4118.22.3, REQ_F4118.30.1</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -3662,7 +3788,7 @@
       </x:c>
       <x:c r="F4" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.23.1, REQ_F4118.23.2, REQ_F4118.23.3, REQ_F4118.23.4, REQ_F4118.23.5, REQ_F4118.23.6, REQ_F4118.23.7, REQ_F4118.23.8</x:t>
+          <x:t xml:space="preserve">REQ_F4118.23.1, REQ_F4118.23.2, REQ_F4118.23.3, REQ_F4118.23.4, REQ_F4118.23.5, REQ_F4118.23.6, REQ_F4118.23.7, REQ_F4118.23.8, REQ_F4118.30.2, REQ_F4118.30.3</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -3694,7 +3820,7 @@
       </x:c>
       <x:c r="F5" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.21.1, REQ_F4118.21.2, REQ_F4118.21.3</x:t>
+          <x:t xml:space="preserve">REQ_F4118.21.1, REQ_F4118.21.2, REQ_F4118.21.3, REQ_F4118.30.1</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -3726,7 +3852,7 @@
       </x:c>
       <x:c r="F6" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.25.1, REQ_F4118.25.2, REQ_F4118.25.3, REQ_F4118.25.4</x:t>
+          <x:t xml:space="preserve">REQ_F4118.25.1, REQ_F4118.25.2, REQ_F4118.25.3, REQ_F4118.25.4, REQ_F4118.30.1</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -3758,7 +3884,7 @@
       </x:c>
       <x:c r="F7" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.25.2, REQ_F4118.25.3, REQ_F4118.25.7</x:t>
+          <x:t xml:space="preserve">REQ_F4118.25.2, REQ_F4118.25.3, REQ_F4118.25.7, REQ_F4118.30.1, REQ_F4118.30.3</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -3790,7 +3916,7 @@
       </x:c>
       <x:c r="F8" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.23.5, REQ_F4118.23.6, REQ_F4118.25.5, REQ_F4118.25.6, REQ_F4118.25.7, REQ_F4118.25.8</x:t>
+          <x:t xml:space="preserve">REQ_F4118.23.5, REQ_F4118.23.6, REQ_F4118.25.5, REQ_F4118.25.6, REQ_F4118.25.7, REQ_F4118.25.8, REQ_F4118.30.2</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -3822,7 +3948,7 @@
       </x:c>
       <x:c r="F9" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.25.6, REQ_F4118.25.7, REQ_F4118.25.8</x:t>
+          <x:t xml:space="preserve">REQ_F4118.25.6, REQ_F4118.25.7, REQ_F4118.25.8, REQ_F4118.30.2</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -7531,7 +7657,7 @@
   <x:cols>
     <x:col min="1" max="1" width="16" customWidth="1"/>
     <x:col min="2" max="2" width="60" customWidth="1"/>
-    <x:col min="3" max="3" width="54" customWidth="1"/>
+    <x:col min="3" max="3" width="60" customWidth="1"/>
     <x:col min="4" max="4" width="24" customWidth="1"/>
     <x:col min="5" max="5" width="60" customWidth="1"/>
     <x:col min="6" max="6" width="60" customWidth="1"/>
@@ -9755,6 +9881,117 @@
       <x:c r="G60" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.30.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B61" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should load demo companies, branches, departments and roles for the Development environment.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C61" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.20, REQ_DS43.22, REQ_DS43.89, REQ_DS43.90, REQ_DS43.91</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D61" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E61" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F61" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-SEED-001, SYS-SEED-002, SYS-SEED-003, SYS-SEED-006</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G61" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.30.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B62" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should create the test accounts of the SeedUsers setting with hashed passwords and company assignments.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C62" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.82, REQ_DS43.92, REQ_DS43.93</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D62" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E62" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F62" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-SEED-001, SYS-SEED-005</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G62" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.30.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B63" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow the seed to run repeatedly without duplicating or overwriting data.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C63" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.20, REQ_DS43.82, REQ_DS43.91</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D63" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E63" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F63" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-SEED-001, SYS-SEED-003, SYS-SEED-004</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G63" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
feat(ui): add shared dialogs, list/document page templates (WU-SYS-014)
- ErpDialogService: confirm / alert / success toast / select dialog (BlueWhale 4.4.1.9)
- erp-list-page + table-query helpers, erp-document-page + adjacentIds + unsavedChangesGuard
- erp-date-range quick ranges, erp-status-tag
- role list adopts the list template and shared confirm dialog (replaces popconfirm)
- trilingual keys, ADR-024, REQ_F4118.31.1-6, interfaces 8.71-8.74

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Re6ad69b918224735"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Ra7e0587e88734a7f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R423e4857fb234118"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Rc6d76449e44e44f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R23ab5dcbf37a43de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R30c151c9f1d643f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R99918af3ec494258"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="Rde99fb97f5d249a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R06a8653ffa9849c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Rabb65e98e90d4fe9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Rc72b1a7703fc47e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R493857cb06894759"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R62568a8a0f2c4ab5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Rda8e9146e6924d5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R79b7869c7ddd44b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Rfd4740dbeb1046a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="Ra2b7c817e6dd4108"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rda868abf61bf4eb0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2717,6 +2717,258 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="64">
+      <x:c r="A64" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.31.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B64" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C64" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Shared Dialogs and Page Templates</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D64" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E64" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should ask for confirmation in a shared trilingual confirmation box before dangerous actions.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F64" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G64" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="H64" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:186</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.31.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B65" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C65" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Shared Dialogs and Page Templates</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D65" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E65" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should show results that need the user's attention in a shared prompt box, and short success messages as toasts.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F65" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G65" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="H65" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:187</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.31.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B66" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C66" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Shared Dialogs and Page Templates</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D66" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E66" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should provide a shared selection window for choosing master data with search and server-side paging.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F66" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G66" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="H66" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:188</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.31.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B67" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C67" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Shared Dialogs and Page Templates</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D67" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E67" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should provide a standard list page template reused by every module.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F67" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G67" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="H67" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:189</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.31.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B68" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C68" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Shared Dialogs and Page Templates</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D68" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E68" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should provide a standard document page template with status, previous / next navigation and unsaved-change protection.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F68" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G68" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="H68" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:190</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.31.6</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B69" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C69" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Shared Dialogs and Page Templates</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D69" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E69" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should provide a date range filter with quick ranges and a document status tag following the macaron status colours.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F69" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G69" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="H69" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:191</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
   </x:sheetData>
 </x:worksheet>
 </file>
@@ -4217,7 +4469,7 @@
   <x:cols>
     <x:col min="1" max="1" width="16" customWidth="1"/>
     <x:col min="2" max="2" width="15" customWidth="1"/>
-    <x:col min="3" max="3" width="54" customWidth="1"/>
+    <x:col min="3" max="3" width="60" customWidth="1"/>
     <x:col min="4" max="4" width="42" customWidth="1"/>
     <x:col min="5" max="5" width="13" customWidth="1"/>
     <x:col min="6" max="6" width="23" customWidth="1"/>
@@ -7643,6 +7895,348 @@
         </x:is>
       </x:c>
       <x:c r="K60" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.71.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B61" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.71</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C61" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Confirmation / Prompt Box Interface（BlueWhale 4.4.1.9）</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D61" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">OK / Cancel (Button)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E61" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">確定／取消</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F61" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">確認或放棄動作</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G61" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Button</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H61" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">確認框兩個按鈕，提示框只有確定；Esc 等同取消</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I61" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J61" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K61" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.72.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B62" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.72</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C62" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Select Dialog Interface（BlueWhale 4.4.1.9 Select Client / Supplier / Item）</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D62" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Keyword (Input)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E62" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">關鍵字</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F62" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">搜尋主檔</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G62" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Text</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H62" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">去除前後空白；查詢回到第 1 頁</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I62" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J62" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K62" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.72.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B63" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.72</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C63" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Select Dialog Interface（BlueWhale 4.4.1.9 Select Client / Supplier / Item）</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D63" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Selection (Checkbox / Row)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E63" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">選取</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F63" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">選擇主檔資料</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G63" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Row key</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H63" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">單選 1 筆、多選跨頁累積；至少 1 筆才可確定</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I63" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.72.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J63" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K63" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.73.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B64" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.73</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C64" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Standard List Page Template</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D64" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Date Range (Date inputs + quick buttons)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E64" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">開始／結束日期</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F64" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">限制查詢期間</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G64" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">yyyy-MM-dd</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H64" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">含頭尾；快選今天、本週、本月、上月、本季、本年；開始晚於結束時提示</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I64" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J64" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K64" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.73.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B65" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.73</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C65" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Standard List Page Template</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D65" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Page Size (Dropdown)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E65" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">每頁筆數</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F65" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">分頁</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G65" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">整數</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H65" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">10／20／50／100／200</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I65" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J65" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K65" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.74.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B66" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.74</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C66" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Standard Document Page Template</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D66" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Previous / Next (Button)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E66" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">上一筆／下一筆</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F66" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">依列表順序切換單據</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G66" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Button</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H66" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">第一筆停用上一筆、最後一筆停用下一筆</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I66" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">None</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J66" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K66" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Developer</x:t>
         </x:is>
@@ -9995,6 +10589,228 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="64">
+      <x:c r="A64" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.31.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B64" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should ask for confirmation in a shared trilingual confirmation box before dangerous actions.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C64" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="D64" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.71</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E64" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.71.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F64" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-UI-001, SYS-UI-002, SYS-UI-003</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G64" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.31.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B65" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should show results that need the user's attention in a shared prompt box, and short success messages as toasts.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C65" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="D65" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.71</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E65" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.71.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F65" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-UI-001</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G65" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.31.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B66" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should provide a shared selection window for choosing master data with search and server-side paging.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C66" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="D66" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.72</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E66" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.72.1, REQ_IO_A8.72.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F66" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-UI-001</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G66" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.31.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B67" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should provide a standard list page template reused by every module.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C67" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="D67" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.73</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E67" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.73.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F67" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-UI-001, SYS-UI-002</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G67" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.31.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B68" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should provide a standard document page template with status, previous / next navigation and unsaved-change protection.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C68" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="D68" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.74</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E68" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.74.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F68" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-UI-001</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G68" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.31.6</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B69" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should provide a date range filter with quick ranges and a document status tag following the macaron status colours.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C69" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="D69" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.73, 4.4.1.8.74</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E69" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.73.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F69" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-UI-001</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G69" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
   </x:sheetData>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
feat(sys): add IP whitelist backend and access enforcement
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Rabb65e98e90d4fe9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Rc72b1a7703fc47e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R493857cb06894759"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R62568a8a0f2c4ab5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Rda8e9146e6924d5c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R79b7869c7ddd44b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Rfd4740dbeb1046a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="Ra2b7c817e6dd4108"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rda868abf61bf4eb0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R9e0a3cbb52f34d01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R0f8903d72c5e4cda"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R925b97ca4f234f51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Rd70b9cec24c048b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Rb937b9c7d9264b64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="Rfc921749e0584fc1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R2cf9e3ea83cd44f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R4a004cc7daa44c89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R201018fe333f46dd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2969,6 +2969,258 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="70">
+      <x:c r="A70" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.32.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B70" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C70" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">IP Whitelist</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D70" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E70" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to view IP whitelist rules.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F70" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G70" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="H70" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:203</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.32.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B71" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C71" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">IP Whitelist</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D71" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E71" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to create and deactivate IP whitelist rules.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F71" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G71" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="H71" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:204</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.32.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B72" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C72" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">IP Whitelist</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D72" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E72" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow single IPv4 or IPv6 addresses and CIDR networks in system, role or user scope.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F72" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G72" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="H72" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:205</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.32.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B73" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C73" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">IP Whitelist</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D73" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E73" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should reject disallowed requests and audit each rejection.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F73" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G73" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="H73" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:206</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.32.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B74" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C74" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">IP Whitelist</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D74" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E74" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow operators to disable IP filtering through server configuration.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F74" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G74" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="H74" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:207</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.32.6</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B75" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C75" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">IP Whitelist</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D75" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E75" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should provide a trilingual IP whitelist maintenance page.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F75" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G75" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="H75" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:208</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
   </x:sheetData>
 </x:worksheet>
 </file>
@@ -4457,6 +4709,38 @@
       <x:c r="F17" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">REQ_F4118.29.4, REQ_F4118.29.5, REQ_F4118.29.6, REQ_F4118.29.7, REQ_F4118.29.9</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.102</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B18" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C18" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">sys_ip_whitelist</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D18" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System-wide IP ranges scoped to the system, a role, or a user, with inclusive effective dates and audit/version fields.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E18" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F18" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.32.1, REQ_F4118.32.2, REQ_F4118.32.3, REQ_F4118.32.4</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -10811,6 +11095,228 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="70">
+      <x:c r="A70" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.32.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B70" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to view IP whitelist rules.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C70" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.102</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D70" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E70" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F70" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-IPW-004</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G70" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.32.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B71" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow authorized users to create and deactivate IP whitelist rules.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C71" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.102</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D71" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E71" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F71" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-IPW-004, SYS-IPW-005</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G71" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.32.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B72" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow single IPv4 or IPv6 addresses and CIDR networks in system, role or user scope.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C72" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.102</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D72" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E72" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F72" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-IPW-001, SYS-IPW-002, SYS-IPW-005</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G72" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.32.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B73" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should reject disallowed requests and audit each rejection.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C73" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.102</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D73" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E73" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F73" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-IPW-003, SYS-IPW-006</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G73" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.32.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B74" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should allow operators to disable IP filtering through server configuration.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C74" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="D74" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E74" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F74" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-IPW-006</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G74" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.32.6</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B75" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should provide a trilingual IP whitelist maintenance page.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C75" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="D75" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E75" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F75" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-IPW-007</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G75" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
   </x:sheetData>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
feat(sys): add company-scoped notification publisher
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R6882f1b0ae264c8e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R25557b6dbdec4d20"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Ra60262dec98e4c15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R2e9cf23ed85d4651"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R7544f24ec07443a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R092b782c6af74c03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R8b268be8799e4b2f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R32345f7fc087498f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R788440bfd9874bae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Ra8c920fbf8bc4a64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R88b2b476cffe4ca1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Rc9e22068e48d4d10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Rd0a1695fef854f71"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R967f051e10d14b02"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="Rac599ffce0274b1a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Rc3f0375624ce4839"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="Rd51fd2db64414f55"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R8c4e1e597e1843a3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3767,6 +3767,132 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="89">
+      <x:c r="A89" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.33.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B89" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C89" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">In-app Notification</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D89" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E89" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable modules to publish notifications to a user.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F89" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G89" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="H89" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:278</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="90">
+      <x:c r="A90" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.33.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B90" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C90" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">In-app Notification</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D90" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E90" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to view notifications.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F90" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G90" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="H90" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:279</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="91">
+      <x:c r="A91" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.33.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B91" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C91" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">In-app Notification</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D91" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E91" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to mark notifications as read.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F91" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G91" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="H91" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/SYS/requirements.md:280</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
   </x:sheetData>
 </x:worksheet>
 </file>
@@ -5351,6 +5477,38 @@
       <x:c r="F20" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">REQ_F4118.19.1, REQ_F4118.19.2, REQ_F4118.19.3</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.104</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B21" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C21" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">sys_notification</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D21" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">One recipient's company-scoped notification, source identity, read time and expiry.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E21" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F21" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.33.1, REQ_F4118.33.2, REQ_F4118.33.3</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -14631,6 +14789,117 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="89">
+      <x:c r="A89" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.33.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B89" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable modules to publish notifications to a user.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C89" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.104</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D89" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E89" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F89" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">SYS-NOTIFY-001, SYS-NOTIFY-002, SYS-NOTIFY-003</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G89" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="90">
+      <x:c r="A90" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.33.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B90" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to view notifications.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C90" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.104</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D90" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E90" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F90" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="G90" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="91">
+      <x:c r="A91" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.33.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B91" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to mark notifications as read.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C91" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.104</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D91" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E91" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F91" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="G91" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
   </x:sheetData>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
feat(sys): add notification inbox, unread badge and expiry cleanup
- GET /api/v1/sys/notifications (paged, unread filter), unread-count,
  single and read-all endpoints scoped to the current user and company
- daily background cleanup of expired notifications
- header bell badge and trilingual /sys/notifications inbox
- seed roles get personal notification permissions
- API integration, frontend unit and E2E coverage (SYS-NOTIFY-004..007)
- stabilise approval delegation E2E dropdown selection

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Ra8c920fbf8bc4a64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R88b2b476cffe4ca1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Rc9e22068e48d4d10"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Rd0a1695fef854f71"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R967f051e10d14b02"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="Rac599ffce0274b1a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Rc3f0375624ce4839"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="Rd51fd2db64414f55"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R8c4e1e597e1843a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R92a32419cf0544fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R6ade4a7194f444bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R560d1c22942148d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R82b6ca4308084c85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Red931584e52b44cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R422d027e019a431f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Rfbfa4b7545c740a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R216092e974ac4c82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R39acce8a69084017"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3827,7 +3827,7 @@
       </x:c>
       <x:c r="D90" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">1.0</x:t>
+          <x:t xml:space="preserve">1.1</x:t>
         </x:is>
       </x:c>
       <x:c r="E90" s="2" t="inlineStr">
@@ -3869,7 +3869,7 @@
       </x:c>
       <x:c r="D91" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">1.0</x:t>
+          <x:t xml:space="preserve">1.1</x:t>
         </x:is>
       </x:c>
       <x:c r="E91" s="2" t="inlineStr">
@@ -5523,7 +5523,7 @@
     <x:col min="2" max="2" width="15" customWidth="1"/>
     <x:col min="3" max="3" width="60" customWidth="1"/>
     <x:col min="4" max="4" width="42" customWidth="1"/>
-    <x:col min="5" max="5" width="13" customWidth="1"/>
+    <x:col min="5" max="5" width="16" customWidth="1"/>
     <x:col min="6" max="6" width="23" customWidth="1"/>
     <x:col min="7" max="7" width="60" customWidth="1"/>
     <x:col min="8" max="8" width="60" customWidth="1"/>
@@ -11512,6 +11512,348 @@
         </x:is>
       </x:c>
       <x:c r="K105" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="106">
+      <x:c r="A106" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.76.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B106" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.76</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C106" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Notification View Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D106" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Unread Badge (Label)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E106" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">頂列未讀數</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F106" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">快速辨識新通知</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G106" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Integer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H106" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">0 隱藏；超過 99 顯示 99+</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I106" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">收件箱</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J106" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K106" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="107">
+      <x:c r="A107" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.76.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B107" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.76</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C107" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Notification View Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D107" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Unread Only (Button)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E107" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">未讀篩選</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F107" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">切換全部／未讀</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G107" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Button</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H107" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">切換後回第 1 頁</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I107" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">通知列表</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J107" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K107" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="108">
+      <x:c r="A108" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.76.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B108" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.76</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C108" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Notification View Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D108" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Notification List (Table)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E108" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">類別、標題、內文、時間、狀態</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F108" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">瀏覽本人通知</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G108" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Paged table</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H108" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">每頁 20，伺服器分頁</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I108" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">未讀篩選</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J108" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K108" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="109">
+      <x:c r="A109" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.76.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B109" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.76</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C109" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Notification View Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D109" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Mark Read (Button)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E109" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">單則已讀</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F109" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">清除該筆未讀狀態</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G109" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Button</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H109" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">只在未讀且有 READ 權限時顯示</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I109" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">通知列表</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J109" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K109" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="110">
+      <x:c r="A110" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.76.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B110" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.76</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C110" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Notification View Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D110" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Mark All Read (Button)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E110" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">全部已讀</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F110" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">清除目前公司本人未讀狀態</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G110" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Button</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H110" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">未讀數為 0 時停用</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I110" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">通知列表</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J110" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K110" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="111">
+      <x:c r="A111" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.76.6</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B111" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.76</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C111" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Notification View Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D111" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Open (Link)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E111" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">站內目標</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F111" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">跳至通知相關頁</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G111" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Internal route</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H111" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">無路徑則隱藏</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I111" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">通知列表</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J111" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K111" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Developer</x:t>
         </x:is>
@@ -14844,22 +15186,22 @@
       </x:c>
       <x:c r="D90" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">4.4.1.8.76</x:t>
         </x:is>
       </x:c>
       <x:c r="E90" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">REQ_IO_A8.76.1, REQ_IO_A8.76.2, REQ_IO_A8.76.3, REQ_IO_A8.76.6</x:t>
         </x:is>
       </x:c>
       <x:c r="F90" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">SYS-NOTIFY-004, SYS-NOTIFY-005, SYS-NOTIFY-006, SYS-NOTIFY-007</x:t>
         </x:is>
       </x:c>
       <x:c r="G90" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Partial</x:t>
+          <x:t xml:space="preserve">Covered</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -14881,22 +15223,22 @@
       </x:c>
       <x:c r="D91" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">4.4.1.8.76</x:t>
         </x:is>
       </x:c>
       <x:c r="E91" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">REQ_IO_A8.76.4, REQ_IO_A8.76.5</x:t>
         </x:is>
       </x:c>
       <x:c r="F91" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">SYS-NOTIFY-004, SYS-NOTIFY-005, SYS-NOTIFY-006, SYS-NOTIFY-007</x:t>
         </x:is>
       </x:c>
       <x:c r="G91" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Partial</x:t>
+          <x:t xml:space="preserve">Covered</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
chore(sys): complete full regression and module handoff
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R92a32419cf0544fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R6ade4a7194f444bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R560d1c22942148d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R82b6ca4308084c85"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Red931584e52b44cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R422d027e019a431f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Rfbfa4b7545c740a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R216092e974ac4c82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R39acce8a69084017"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R6c2d2eaa9fed4ac7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R40c85577b7784da3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R258271d03688483f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Rc637c690780043b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Rd46752d7adf64763"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="Rb3d18b34b69b480d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R3c1c1f1926ad4edd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R6fb13e6667884e21"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Ra6d0736215244ec9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -131,7 +131,7 @@
       </x:c>
       <x:c r="D2" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">1.1</x:t>
+          <x:t xml:space="preserve">1.2</x:t>
         </x:is>
       </x:c>
       <x:c r="E2" s="2" t="inlineStr">
@@ -146,7 +146,7 @@
       </x:c>
       <x:c r="G2" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">已登入用戶須提供目前密碼與符合政策、不同於舊密碼的新密碼；目前密碼錯誤計入五次鎖定。成功後重設到期日、寫不含密碼的安全稽核、撤銷先前簽發的全部 Refresh Token，回傳目前工作階段的新 Token，前端立即替換 Session。密碼到期不能登入時，登入頁提供入口，以帳號、舊密碼與一次性 Captcha 修改並登入；帳密錯誤維持相同 401。失敗後清空密碼並重新載入 Captcha。</x:t>
+          <x:t xml:space="preserve">已登入用戶須提供目前密碼與符合政策、不同於舊密碼的新密碼；目前密碼錯誤計入五次鎖定，並寫 LOGIN_FAILED 安全稽核（原因 CURRENT_PASSWORD_INVALID，不含密碼）。成功後重設到期日、寫不含密碼的安全稽核、撤銷先前簽發的全部 Refresh Token，回傳目前工作階段的新 Token，前端立即替換 Session。密碼到期不能登入時，登入頁提供入口，以帳號、舊密碼與一次性 Captcha 修改並登入；帳密錯誤維持相同 401。失敗後清空密碼並重新載入 Captcha。</x:t>
         </x:is>
       </x:c>
       <x:c r="H2" s="2" t="inlineStr">
@@ -761,7 +761,7 @@
       </x:c>
       <x:c r="D17" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">1.1</x:t>
+          <x:t xml:space="preserve">1.2</x:t>
         </x:is>
       </x:c>
       <x:c r="E17" s="2" t="inlineStr">
@@ -776,7 +776,7 @@
       </x:c>
       <x:c r="G17" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">版本不符回 409；審計欄位記錄修改者；目標公司不是用戶獲授權的公司時回 404。</x:t>
+          <x:t xml:space="preserve">版本不符回 409；審計欄位記錄修改者；目標公司不是用戶獲授權的公司時回 404；操作者在被修改的公司（含已停用）亦須有 SYS.COMPANY.EDIT，否則 403（ADR-032）。</x:t>
         </x:is>
       </x:c>
       <x:c r="H17" s="2" t="inlineStr">
@@ -1349,7 +1349,7 @@
       </x:c>
       <x:c r="D31" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">1.0</x:t>
+          <x:t xml:space="preserve">1.1</x:t>
         </x:is>
       </x:c>
       <x:c r="E31" s="2" t="inlineStr">
@@ -1364,7 +1364,7 @@
       </x:c>
       <x:c r="G31" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">需 SYS.USER.EDIT 並帶 version（過期 409）；停用後不可登入與刷新，重新啟用後可登入；不可停用自己 422 SYS.USER.SELF_DEACTIVATION；他公司用戶 404。</x:t>
+          <x:t xml:space="preserve">需 SYS.USER.EDIT 並帶 version（過期 409）；停用後不可登入與刷新，重新啟用後可登入；不可停用自己 422 SYS.USER.SELF_DEACTIVATION；他公司用戶 404；用戶亦屬於其他公司時，操作者在每間已啟用關聯的公司都要有 SYS.USER.EDIT（否則 403 COMMON.PERMISSION.DENIED），且用戶角色不超出操作者權限（否則 403 SYS.ROLE.BEYOND_AUTHORITY），ADR-032。</x:t>
         </x:is>
       </x:c>
       <x:c r="H31" s="2" t="inlineStr">
@@ -1391,7 +1391,7 @@
       </x:c>
       <x:c r="D32" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">1.0</x:t>
+          <x:t xml:space="preserve">1.1</x:t>
         </x:is>
       </x:c>
       <x:c r="E32" s="2" t="inlineStr">
@@ -1406,7 +1406,7 @@
       </x:c>
       <x:c r="G32" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">重設密碼需 SYS.USER.RESET_PASSWORD，依密碼政策驗證，重新起算到期並清除鎖定，舊密碼即失效；解鎖需 SYS.USER.EDIT，清除失敗計數與鎖定，未鎖定時亦回 204；他公司用戶 404。</x:t>
+          <x:t xml:space="preserve">重設密碼需 SYS.USER.RESET_PASSWORD，依密碼政策驗證，重新起算到期並清除鎖定，舊密碼即失效；解鎖需 SYS.USER.EDIT，清除失敗計數與鎖定，未鎖定時亦回 204；他公司用戶 404；跨公司與角色上限檢查同 REQ_F4118.23.7（ADR-032）。</x:t>
         </x:is>
       </x:c>
       <x:c r="H32" s="2" t="inlineStr">
@@ -1742,7 +1742,7 @@
       </x:c>
       <x:c r="G40" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">需 SYS.ROLE.EDIT；帶 version，不符回 409，且權限集合不變（同一交易）；停用角色立即不再授予權限。</x:t>
+          <x:t xml:space="preserve">需 SYS.ROLE.EDIT；帶 version，不符回 409，且權限集合不變（同一交易）；停用角色立即不再授予權限。角色是全系統定義：操作者在角色已指派的每間公司都必須全權，否則 403 SYS.AUTHORITY.FULL_ACCESS_REQUIRED（ADR-033）。</x:t>
         </x:is>
       </x:c>
       <x:c r="H40" s="2" t="inlineStr">
@@ -1853,7 +1853,7 @@
       </x:c>
       <x:c r="D43" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">1.0</x:t>
+          <x:t xml:space="preserve">1.1</x:t>
         </x:is>
       </x:c>
       <x:c r="E43" s="2" t="inlineStr">
@@ -1868,7 +1868,7 @@
       </x:c>
       <x:c r="G43" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">需 SYS.USER.EDIT；公司必須啟用；分店／部門必須屬於該公司且啟用；角色必須存在且啟用；角色整組取代；每位用戶最多一間預設公司（設定新預設會取消舊預設）。用戶不存在或不屬於目前公司回 404 SYS.USER.NOT_FOUND；目標公司不是操作者獲授權的公司回 404 SYS.COMPANY.NOT_FOUND；不可停用自己的公司授權（422 SYS.USER.SELF_DEACTIVATION）（ADR-017）。</x:t>
+          <x:t xml:space="preserve">需 SYS.USER.EDIT；公司必須啟用；分店／部門必須屬於該公司且啟用；角色必須存在且啟用；角色整組取代；每位用戶最多一間預設公司（設定新預設會取消舊預設）。用戶不存在或不屬於目前公司回 404 SYS.USER.NOT_FOUND；目標公司不是操作者獲授權的公司回 404 SYS.COMPANY.NOT_FOUND；不可停用自己的公司授權（422 SYS.USER.SELF_DEACTIVATION）（ADR-017）。操作者在目標公司亦須有 SYS.USER.EDIT（否則 403 COMMON.PERMISSION.DENIED）；新增或移除的角色須在操作者權限之內（全權角色只限全權操作者；一般角色的每個權限操作者都有且範圍不窄於角色），否則 403 SYS.ROLE.BEYOND_AUTHORITY；不可變更自己的角色（422 SYS.USER.SELF_ROLE_CHANGE），角色不變時可改組織與預設公司（ADR-032）。</x:t>
         </x:is>
       </x:c>
       <x:c r="H43" s="2" t="inlineStr">
@@ -3785,7 +3785,7 @@
       </x:c>
       <x:c r="D89" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">1.0</x:t>
+          <x:t xml:space="preserve">1.1</x:t>
         </x:is>
       </x:c>
       <x:c r="E89" s="2" t="inlineStr">
@@ -12495,7 +12495,7 @@
       </x:c>
       <x:c r="F17" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-ORG-005, SYS-ORG-009, SYS-ORG-013, SYS-ORG-021</x:t>
+          <x:t xml:space="preserve">SYS-ORG-005, SYS-ORG-009, SYS-ORG-013, SYS-ORG-021, SYS-PERM-030</x:t>
         </x:is>
       </x:c>
       <x:c r="G17" s="2" t="inlineStr">
@@ -12569,7 +12569,7 @@
       </x:c>
       <x:c r="F19" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-ORG-002, SYS-ORG-004, SYS-ORG-010, SYS-ORG-012, SYS-ORG-020, SYS-ORG-022, SYS-ORG-024, SYS-ORG-025</x:t>
+          <x:t xml:space="preserve">SYS-ORG-002, SYS-ORG-004, SYS-ORG-010, SYS-ORG-012, SYS-ORG-020, SYS-ORG-022, SYS-ORG-024, SYS-ORG-025, SYS-ORG-027</x:t>
         </x:is>
       </x:c>
       <x:c r="G19" s="2" t="inlineStr">
@@ -12680,7 +12680,7 @@
       </x:c>
       <x:c r="F22" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-ORG-002, SYS-ORG-004, SYS-ORG-010, SYS-ORG-012, SYS-ORG-020, SYS-ORG-023, SYS-ORG-026</x:t>
+          <x:t xml:space="preserve">SYS-ORG-002, SYS-ORG-004, SYS-ORG-010, SYS-ORG-012, SYS-ORG-020, SYS-ORG-023, SYS-ORG-026, SYS-ORG-027</x:t>
         </x:is>
       </x:c>
       <x:c r="G22" s="2" t="inlineStr">
@@ -12791,7 +12791,7 @@
       </x:c>
       <x:c r="F25" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-USER-001, SYS-USER-004, SYS-USER-012</x:t>
+          <x:t xml:space="preserve">SYS-ORG-027, SYS-USER-001, SYS-USER-004, SYS-USER-012</x:t>
         </x:is>
       </x:c>
       <x:c r="G25" s="2" t="inlineStr">
@@ -13013,7 +13013,7 @@
       </x:c>
       <x:c r="F31" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-USER-006, SYS-USER-010, SYS-USER-013, SYS-USER-015</x:t>
+          <x:t xml:space="preserve">SYS-USER-006, SYS-USER-010, SYS-USER-013, SYS-USER-015, SYS-PERM-029</x:t>
         </x:is>
       </x:c>
       <x:c r="G31" s="2" t="inlineStr">
@@ -13050,7 +13050,7 @@
       </x:c>
       <x:c r="F32" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-USER-006, SYS-USER-010, SYS-USER-014</x:t>
+          <x:t xml:space="preserve">SYS-USER-006, SYS-USER-010, SYS-USER-014, SYS-PERM-029</x:t>
         </x:is>
       </x:c>
       <x:c r="G32" s="2" t="inlineStr">
@@ -13272,7 +13272,7 @@
       </x:c>
       <x:c r="F38" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-PERM-004, SYS-PERM-011, SYS-PERM-024, SYS-PERM-025</x:t>
+          <x:t xml:space="preserve">SYS-ORG-027, SYS-PERM-004, SYS-PERM-011, SYS-PERM-024, SYS-PERM-025</x:t>
         </x:is>
       </x:c>
       <x:c r="G38" s="2" t="inlineStr">
@@ -13346,7 +13346,7 @@
       </x:c>
       <x:c r="F40" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-PERM-011, SYS-PERM-024, SYS-PERM-025</x:t>
+          <x:t xml:space="preserve">SYS-PERM-011, SYS-PERM-024, SYS-PERM-025, SYS-PERM-031, SYS-PERM-032</x:t>
         </x:is>
       </x:c>
       <x:c r="G40" s="2" t="inlineStr">
@@ -13457,7 +13457,7 @@
       </x:c>
       <x:c r="F43" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-PERM-015, SYS-PERM-016, SYS-PERM-017, SYS-PERM-018, SYS-PERM-026, SYS-PERM-027</x:t>
+          <x:t xml:space="preserve">SYS-PERM-015, SYS-PERM-016, SYS-PERM-017, SYS-PERM-018, SYS-PERM-026, SYS-PERM-027, SYS-PERM-028</x:t>
         </x:is>
       </x:c>
       <x:c r="G43" s="2" t="inlineStr">
@@ -14937,7 +14937,7 @@
       </x:c>
       <x:c r="F83" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-IPW-004</x:t>
+          <x:t xml:space="preserve">SYS-IPW-004, SYS-IPW-009</x:t>
         </x:is>
       </x:c>
       <x:c r="G83" s="2" t="inlineStr">
@@ -14974,7 +14974,7 @@
       </x:c>
       <x:c r="F84" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SYS-IPW-004, SYS-IPW-005</x:t>
+          <x:t xml:space="preserve">SYS-PERM-032, SYS-IPW-004, SYS-IPW-005, SYS-IPW-008, SYS-IPW-009</x:t>
         </x:is>
       </x:c>
       <x:c r="G84" s="2" t="inlineStr">
@@ -15312,12 +15312,12 @@
       </x:c>
       <x:c r="E2" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4111.1.1</x:t>
+          <x:t xml:space="preserve">REQ_F4118.24.1</x:t>
         </x:is>
       </x:c>
       <x:c r="F2" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">未開始</x:t>
+          <x:t xml:space="preserve">完成</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -15349,7 +15349,7 @@
       </x:c>
       <x:c r="F3" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">未開始</x:t>
+          <x:t xml:space="preserve">完成</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -15376,12 +15376,12 @@
       </x:c>
       <x:c r="E4" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4111.1.3</x:t>
+          <x:t xml:space="preserve">REQ_F4118.24.3</x:t>
         </x:is>
       </x:c>
       <x:c r="F4" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">未開始</x:t>
+          <x:t xml:space="preserve">完成</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -20880,12 +20880,12 @@
       </x:c>
       <x:c r="E176" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.6.1</x:t>
+          <x:t xml:space="preserve">REQ_F4118.23.5</x:t>
         </x:is>
       </x:c>
       <x:c r="F176" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">未開始</x:t>
+          <x:t xml:space="preserve">完成</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -20912,12 +20912,12 @@
       </x:c>
       <x:c r="E177" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.6.2</x:t>
+          <x:t xml:space="preserve">REQ_F4118.23.6</x:t>
         </x:is>
       </x:c>
       <x:c r="F177" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">未開始</x:t>
+          <x:t xml:space="preserve">完成</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -20944,12 +20944,12 @@
       </x:c>
       <x:c r="E178" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.6.3</x:t>
+          <x:t xml:space="preserve">REQ_F4118.25.6</x:t>
         </x:is>
       </x:c>
       <x:c r="F178" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">未開始</x:t>
+          <x:t xml:space="preserve">完成</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -20976,12 +20976,12 @@
       </x:c>
       <x:c r="E179" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.6.4</x:t>
+          <x:t xml:space="preserve">REQ_F4118.23.7</x:t>
         </x:is>
       </x:c>
       <x:c r="F179" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">未開始</x:t>
+          <x:t xml:space="preserve">完成</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -22160,12 +22160,12 @@
       </x:c>
       <x:c r="E216" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.16.1</x:t>
+          <x:t xml:space="preserve">REQ_F4118.27.6</x:t>
         </x:is>
       </x:c>
       <x:c r="F216" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">未開始</x:t>
+          <x:t xml:space="preserve">完成</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -22192,12 +22192,12 @@
       </x:c>
       <x:c r="E217" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_F4118.16.2</x:t>
+          <x:t xml:space="preserve">-</x:t>
         </x:is>
       </x:c>
       <x:c r="F217" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">未開始</x:t>
+          <x:t xml:space="preserve">WONT_DO</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -22416,12 +22416,12 @@
       </x:c>
       <x:c r="E224" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.1.1</x:t>
+          <x:t xml:space="preserve">4.4.1.8.62</x:t>
         </x:is>
       </x:c>
       <x:c r="F224" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">未開始</x:t>
+          <x:t xml:space="preserve">完成</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -22453,7 +22453,7 @@
       </x:c>
       <x:c r="F225" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">未開始</x:t>
+          <x:t xml:space="preserve">完成</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -22485,7 +22485,7 @@
       </x:c>
       <x:c r="F226" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">未開始</x:t>
+          <x:t xml:space="preserve">完成</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -26000,12 +26000,12 @@
       </x:c>
       <x:c r="E336" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.8.23</x:t>
+          <x:t xml:space="preserve">4.4.1.8.63</x:t>
         </x:is>
       </x:c>
       <x:c r="F336" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">未開始</x:t>
+          <x:t xml:space="preserve">完成</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -26032,12 +26032,12 @@
       </x:c>
       <x:c r="E337" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.8.24</x:t>
+          <x:t xml:space="preserve">4.4.1.8.61</x:t>
         </x:is>
       </x:c>
       <x:c r="F337" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">未開始</x:t>
+          <x:t xml:space="preserve">完成</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -26064,12 +26064,12 @@
       </x:c>
       <x:c r="E338" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.8.25</x:t>
+          <x:t xml:space="preserve">4.4.1.8.63</x:t>
         </x:is>
       </x:c>
       <x:c r="F338" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">未開始</x:t>
+          <x:t xml:space="preserve">完成</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -26096,12 +26096,12 @@
       </x:c>
       <x:c r="E339" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.8.26</x:t>
+          <x:t xml:space="preserve">4.4.1.8.65</x:t>
         </x:is>
       </x:c>
       <x:c r="F339" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">未開始</x:t>
+          <x:t xml:space="preserve">完成</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -26992,12 +26992,12 @@
       </x:c>
       <x:c r="E367" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.8.54</x:t>
+          <x:t xml:space="preserve">4.4.1.8.66</x:t>
         </x:is>
       </x:c>
       <x:c r="F367" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">未開始</x:t>
+          <x:t xml:space="preserve">完成</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -27829,7 +27829,7 @@
       </x:c>
       <x:c r="F393" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">進行中</x:t>
+          <x:t xml:space="preserve">完成</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -27893,7 +27893,7 @@
       </x:c>
       <x:c r="F395" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">進行中</x:t>
+          <x:t xml:space="preserve">完成</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -27920,12 +27920,12 @@
       </x:c>
       <x:c r="E396" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">sys_operation_log</x:t>
+          <x:t xml:space="preserve">sys_audit_log</x:t>
         </x:is>
       </x:c>
       <x:c r="F396" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">未開始</x:t>
+          <x:t xml:space="preserve">完成</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -28080,12 +28080,12 @@
       </x:c>
       <x:c r="E401" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">sys_announcement</x:t>
+          <x:t xml:space="preserve">—</x:t>
         </x:is>
       </x:c>
       <x:c r="F401" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">未開始</x:t>
+          <x:t xml:space="preserve">WONT_DO</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -28304,12 +28304,12 @@
       </x:c>
       <x:c r="E408" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">sys_announcement</x:t>
+          <x:t xml:space="preserve">sys_notification</x:t>
         </x:is>
       </x:c>
       <x:c r="F408" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">未開始</x:t>
+          <x:t xml:space="preserve">完成</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -28368,12 +28368,12 @@
       </x:c>
       <x:c r="E410" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">sys_menu</x:t>
+          <x:t xml:space="preserve">sys_role_permission</x:t>
         </x:is>
       </x:c>
       <x:c r="F410" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">未開始</x:t>
+          <x:t xml:space="preserve">完成</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -29296,12 +29296,12 @@
       </x:c>
       <x:c r="E439" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">sys_role_permission</x:t>
+          <x:t xml:space="preserve">sys_user_role</x:t>
         </x:is>
       </x:c>
       <x:c r="F439" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">未開始</x:t>
+          <x:t xml:space="preserve">完成</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -29461,7 +29461,7 @@
       </x:c>
       <x:c r="F444" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">未開始</x:t>
+          <x:t xml:space="preserve">完成</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -29557,7 +29557,7 @@
       </x:c>
       <x:c r="F447" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">未開始</x:t>
+          <x:t xml:space="preserve">完成</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -29776,12 +29776,12 @@
       </x:c>
       <x:c r="E454" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">sys_permission</x:t>
+          <x:t xml:space="preserve">sys_role_permission</x:t>
         </x:is>
       </x:c>
       <x:c r="F454" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">未開始</x:t>
+          <x:t xml:space="preserve">完成</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -29813,7 +29813,7 @@
       </x:c>
       <x:c r="F455" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">進行中</x:t>
+          <x:t xml:space="preserve">完成</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
feat(md): add multilingual currency and exchange rate pages
- /md/currencies page (interfaces 8.79-8.81) with base currency tag,
  ISO code and decimal validation, locked base checkbox and versioned
  edit/delete showing BASE_LOCKED / IN_USE
- exchange rate dialog (interface 8.82) with effective-on filter,
  period and 6+8 digit rate validation, OVERLAP message and
  inactive-currency guard; read-only users see rates only
- menu entry, trilingual md/errors/layout texts, Vitest and Playwright
- ui-spec, test plan, optimization log, docgen outputs and status

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Re203fd047cdb4f52"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R77eb2bd63ee143a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Ra616986e7388439c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Rf0060c6df84a47ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Rab28e20f391544b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R42588197280c4018"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R98fcf46b1b744484"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="Rfd385159b10740d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rce3f74d82bb54c50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R6eb35489d94843ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R063bec3fe220488f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R14cd5036934849d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Re085d3a521de45ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R9af716dafb32427a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R999523d0be2a4c9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Re42952122eaa4e60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R9d5c2224e67b43f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R72d35c93ae484d54"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5405,6 +5405,384 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="128">
+      <x:c r="A128" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.35.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B128" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C128" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Currency</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D128" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E128" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to view currencies.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F128" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G128" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">具 MD.CURRENCY.VIEW 可按目前公司以代碼或名稱搜尋、按代碼／名稱排序及分頁幣別（含停用），顯示符號、金額小數位與本位幣標記；排除軟刪除及別公司資料；未選公司回 403。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H128" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/MD/requirements.md:147</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="129">
+      <x:c r="A129" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.35.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B129" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C129" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Currency</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D129" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E129" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to create currencies.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F129" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G129" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">具 MD.CURRENCY.CREATE 可建立 ISO 4217 三個英文字母代碼（轉大寫，公司內永久唯一含已刪除，409 MD.CURRENCY.DUPLICATE_CODE；格式不符 400 code）、非空白名稱（200）、可空符號（10，400 symbol）、金額小數位 0–4（400 decimalPlaces），可同時設為本位幣。不同公司可用相同代碼。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H129" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/MD/requirements.md:148</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="130">
+      <x:c r="A130" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.35.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B130" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C130" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Currency</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D130" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E130" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to edit currencies and set the base currency.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F130" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G130" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">具 MD.CURRENCY.EDIT 可帶版本修改名稱、符號、小數位、啟用狀態與本位幣；代碼不可變。每間公司最多一個本位幣，設定新本位幣時自動取消舊的；公司已有匯率後不可更換本位幣（409 MD.CURRENCY.BASE_LOCKED）；不可直接取消本位幣（422 MD.CURRENCY.BASE_REQUIRED），本位幣必須啟用（422 MD.CURRENCY.BASE_INACTIVE）。舊版本 409，別公司或已刪除 404 MD.CURRENCY.NOT_FOUND。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H130" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/MD/requirements.md:149</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="131">
+      <x:c r="A131" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.35.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B131" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C131" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Currency</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D131" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E131" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to delete currencies.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F131" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G131" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">具 MD.CURRENCY.DELETE 可帶版本軟刪除幣別，代碼仍保留；本位幣 409 MD.CURRENCY.IS_BASE；有未刪除匯率 409 MD.CURRENCY.IN_USE。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H131" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/MD/requirements.md:150</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="132">
+      <x:c r="A132" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.36.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B132" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C132" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Exchange Rate</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D132" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E132" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to view exchange rates of a currency.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F132" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G132" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MD.CURRENCY.VIEW 可查看某幣別的匯率（1 外幣 = 匯率 本位幣），預設按生效日新到舊、可改舊到新，可篩選某日適用的匯率，分頁；幣別不屬目前公司 404 MD.CURRENCY.NOT_FOUND。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H132" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/MD/requirements.md:151</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="133">
+      <x:c r="A133" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.36.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B133" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C133" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Exchange Rate</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D133" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E133" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to create exchange rates.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F133" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G133" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MD.CURRENCY.EDIT 可為啟用的外幣新增匯率：生效日、可空到期日（含當日；早於生效日 400 effectiveTo）、匯率大於 0、最多 11 位整數及 8 位小數（400 rate）。同幣別未刪除的期間不可重疊（409 MD.EXCHANGE_RATE.OVERLAP）；本位幣 422 MD.EXCHANGE_RATE.BASE_CURRENCY；公司未設本位幣 422 MD.EXCHANGE_RATE.NO_BASE_CURRENCY；停用幣別 422 MD.EXCHANGE_RATE.CURRENCY_INACTIVE。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H133" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/MD/requirements.md:152</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="134">
+      <x:c r="A134" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.36.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B134" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C134" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Exchange Rate</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D134" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E134" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to edit exchange rates.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F134" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G134" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MD.CURRENCY.EDIT 可帶版本修改生效日、到期日與匯率，驗證與重疊規則同新增（排除自己）；幣別不可修改；匯率不屬該幣別 404 MD.EXCHANGE_RATE.NOT_FOUND；舊版本 409。已存單據保存自己的成交匯率，不受影響。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H134" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/MD/requirements.md:153</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="135">
+      <x:c r="A135" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.36.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B135" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C135" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Exchange Rate</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D135" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E135" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to delete exchange rates.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F135" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G135" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MD.CURRENCY.EDIT 可帶版本軟刪除匯率，刪除後該期間可重新設定；不屬該幣別 404。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H135" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/MD/requirements.md:154</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="136">
+      <x:c r="A136" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.36.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B136" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C136" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Exchange Rate</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D136" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E136" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable other modules and users to look up the exchange rate of a business date.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F136" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G136" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">ICurrencyLookup.GetRateAsync 與 GET /api/v1/md/exchange-rates/lookup?currencyCode=&amp;date=（MD.CURRENCY.VIEW）回傳涵蓋該業務日期的匯率，代碼不分大小寫，本位幣回 1；停用幣別仍可查詢；幣別不存在 404 MD.CURRENCY.NOT_FOUND；沒有本位幣或沒有匯率 422 MD.EXCHANGE_RATE.NO_BASE_CURRENCY／MD.EXCHANGE_RATE.NOT_FOUND。GetPrecisionAsync 以主檔小數位提供 Money.Round 的捨入設定。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H136" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/MD/requirements.md:155</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
   </x:sheetData>
 </x:worksheet>
 </file>
@@ -7408,6 +7786,70 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.117</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B34" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C34" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">md_currency</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D34" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">This table stores currencies and the base currency of a company.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E34" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F34" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.35.1, REQ_F4118.35.2, REQ_F4118.35.3, REQ_F4118.35.4</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.118</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B35" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C35" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">md_exchange_rate</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D35" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">This table stores exchange rates of foreign currencies against the base currency.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E35" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F35" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.36.1, REQ_F4118.36.2, REQ_F4118.36.3, REQ_F4118.36.4, REQ_F4118.36.5</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
   </x:sheetData>
 </x:worksheet>
 </file>
@@ -7418,7 +7860,7 @@
     <x:col min="1" max="1" width="17" customWidth="1"/>
     <x:col min="2" max="2" width="15" customWidth="1"/>
     <x:col min="3" max="3" width="60" customWidth="1"/>
-    <x:col min="4" max="4" width="42" customWidth="1"/>
+    <x:col min="4" max="4" width="49" customWidth="1"/>
     <x:col min="5" max="5" width="60" customWidth="1"/>
     <x:col min="6" max="6" width="23" customWidth="1"/>
     <x:col min="7" max="7" width="60" customWidth="1"/>
@@ -18823,6 +19265,804 @@
         </x:is>
       </x:c>
       <x:c r="K200" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="201">
+      <x:c r="A201" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.79.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B201" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.79</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C201" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Currency View Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D201" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Search (Input)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E201" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">搜尋代碼或名稱。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F201" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">找到目前公司幣別。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G201" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Text</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H201" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">任意文字</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I201" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.79.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J201" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K201" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="202">
+      <x:c r="A202" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.79.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B202" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.79</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C202" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Currency View Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D202" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Currency List (Table)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E202" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">代碼（本位幣加標籤）、名稱、符號、金額小數位、狀態；代碼與名稱可排序，伺服器分頁；外幣列有匯率／編輯／刪除，本位幣列只有編輯。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F202" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">查看幣別與本位幣。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G202" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Table</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H202" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">每頁 10／20／50／100／200</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I202" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.80.1, REQ_IO_A8.81.1, REQ_IO_A8.82.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J202" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K202" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="203">
+      <x:c r="A203" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.79.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B203" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.79</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C203" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Currency View Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D203" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Delete (Button)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E203" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">二次確認後帶版本軟刪除；有匯率時顯示錯誤。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F203" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">移除未使用的外幣。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G203" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Button</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H203" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">DELETE 權限，本位幣不顯示</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I203" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.79.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J203" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K203" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="204">
+      <x:c r="A204" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.80.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B204" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.80</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C204" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Currency Create Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D204" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Code (Input)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E204" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">ISO 4217 代碼，送出時轉大寫，公司內永久唯一。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F204" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">識別幣別。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G204" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Text</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H204" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">3 個英文字母</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I204" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.79.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J204" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K204" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="205">
+      <x:c r="A205" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.80.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B205" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.80</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C205" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Currency Create Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D205" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Name / Symbol (Input)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E205" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">名稱必填；符號可空，空白送 null。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F205" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">顯示幣別。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G205" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Text</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H205" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">名稱非空白最多 200 字；符號最多 10 字</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I205" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.79.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J205" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K205" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="206">
+      <x:c r="A206" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.80.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B206" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.80</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C206" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Currency Create Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D206" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Amount Decimals (Input)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E206" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">金額小數位，供 Money.Round 按幣別捨入。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F206" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">設定金額精度。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G206" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Number</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H206" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">0–4 的整數，預設 2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I206" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.79.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J206" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K206" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="207">
+      <x:c r="A207" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.80.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B207" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.80</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C207" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Currency Create Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D207" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Base Currency (Checkbox)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E207" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">設為本位幣；會取代原本位幣。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F207" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">設定公司本位幣。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G207" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Boolean</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H207" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">已有匯率時後端回 BASE_LOCKED</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I207" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.79.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J207" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K207" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="208">
+      <x:c r="A208" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.81.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B208" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.81</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C208" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Currency Edit Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D208" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Code (Label)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E208" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">編輯時不可修改。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F208" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">保留既有識別。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G208" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Text</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H208" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">3 字</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I208" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.79.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J208" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K208" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="209">
+      <x:c r="A209" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.81.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B209" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.81</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C209" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Currency Edit Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D209" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Name / Symbol / Decimals / Base / Active (Form)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E209" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">修改名稱、符號、小數位、本位幣與啟用狀態；帶 version。本位幣的勾選鎖定並提示「把另一個幣別設為本位幣」。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F209" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">維護幣別與更換本位幣。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G209" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Text／Number／Boolean</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H209" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">同建立</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I209" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.79.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J209" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K209" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="210">
+      <x:c r="A210" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.82.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B210" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.82</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C210" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Exchange Rate Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D210" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Rate List (Table)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E210" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">生效日、到期日（空白顯示持續有效）、匯率、編輯／刪除；按生效日新到舊，伺服器分頁。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F210" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">查看外幣匯率。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G210" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Table</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H210" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">每頁 10</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I210" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.79.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J210" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K210" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="211">
+      <x:c r="A211" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.82.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B211" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.82</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C211" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Exchange Rate Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D211" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Effective On (Date Picker)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E211" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">只列出該日適用的匯率；「顯示全部」清除。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F211" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">查單據日的匯率。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G211" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Date</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H211" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">yyyy-MM-dd</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I211" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.82.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J211" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K211" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="212">
+      <x:c r="A212" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.82.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B212" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.82</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C212" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Exchange Rate Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D212" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">From / To (Date Picker)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E212" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">生效日必填；到期日可空（持續有效），不可早於生效日。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F212" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">設定匯率期間。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G212" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Date</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H212" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">期間含首尾，不可與同幣別重疊</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I212" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.82.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J212" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K212" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="213">
+      <x:c r="A213" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.82.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B213" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.82</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C213" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Exchange Rate Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D213" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Rate (Input)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E213" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1 外幣 = 匯率 × 本位幣。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F213" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">設定記帳匯率。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G213" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Decimal</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H213" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">大於 0，最多 6 位整數及 8 位小數</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I213" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.82.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J213" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K213" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="214">
+      <x:c r="A214" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.82.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B214" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.82</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C214" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Exchange Rate Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D214" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Delete (Button)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E214" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">確認後帶版本刪除匯率。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F214" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">移除錯誤匯率，期間可重設。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G214" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Action</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H214" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MD.CURRENCY.EDIT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I214" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.82.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J214" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K214" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Developer</x:t>
         </x:is>
@@ -23543,6 +24783,339 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="128">
+      <x:c r="A128" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.35.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B128" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to view currencies.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C128" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.117</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D128" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.79</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E128" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.79.1, REQ_IO_A8.79.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F128" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MD-CUR-001, MD-CUR-005, MD-CUR-UI-001, MD-CUR-UI-002</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G128" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="129">
+      <x:c r="A129" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.35.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B129" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to create currencies.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C129" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.117</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D129" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.80</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E129" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.80.1, REQ_IO_A8.80.2, REQ_IO_A8.80.3, REQ_IO_A8.80.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F129" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MD-CUR-001, MD-CUR-UI-001, MD-CUR-UI-002</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G129" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="130">
+      <x:c r="A130" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.35.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B130" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to edit currencies and set the base currency.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C130" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.117</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D130" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.81</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E130" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.81.1, REQ_IO_A8.81.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F130" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MD-CUR-001, MD-CUR-002, MD-CUR-UI-001, MD-CUR-UI-002</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G130" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="131">
+      <x:c r="A131" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.35.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B131" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to delete currencies.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C131" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.117</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D131" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.79</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E131" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.79.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F131" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MD-CUR-001, MD-CUR-002, MD-CUR-UI-001, MD-CUR-UI-002</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G131" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="132">
+      <x:c r="A132" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.36.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B132" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to view exchange rates of a currency.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C132" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.118</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D132" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.82</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E132" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.82.1, REQ_IO_A8.82.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F132" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MD-CUR-003, MD-CUR-005, MD-CUR-UI-001, MD-CUR-UI-002</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G132" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="133">
+      <x:c r="A133" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.36.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B133" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to create exchange rates.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C133" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.118</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D133" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.82</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E133" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.82.3, REQ_IO_A8.82.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F133" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MD-CUR-002, MD-CUR-003, MD-CUR-UI-001, MD-CUR-UI-002</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G133" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="134">
+      <x:c r="A134" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.36.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B134" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to edit exchange rates.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C134" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.118</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D134" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.82</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E134" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.82.3, REQ_IO_A8.82.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F134" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MD-CUR-003, MD-CUR-UI-001, MD-CUR-UI-002</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G134" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="135">
+      <x:c r="A135" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.36.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B135" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to delete exchange rates.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C135" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.118</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D135" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.82</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E135" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.82.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F135" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MD-CUR-003, MD-CUR-UI-001, MD-CUR-UI-002</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G135" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="136">
+      <x:c r="A136" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.36.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B136" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable other modules and users to look up the exchange rate of a business date.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C136" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.118</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D136" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E136" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F136" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MD-CUR-003, MD-CUR-004</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G136" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
   </x:sheetData>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
feat(md): add multilingual tax code, tax rate and tax calculation pages
- /md/tax-codes page (interfaces 8.83-8.86) with tax rate dialog and
  line tax calculator; menu, route, i18n in three languages
- TaxDirection serialized by name (Output/Input) in JSON
- Vitest +13, Playwright +3; WU-MD-017 done

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R6eb35489d94843ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R063bec3fe220488f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R14cd5036934849d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Re085d3a521de45ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R9af716dafb32427a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R999523d0be2a4c9b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Re42952122eaa4e60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R9d5c2224e67b43f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R72d35c93ae484d54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R09e6252ba4e345f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R30ab56a53ed843a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R6d383a82735d47e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R87bc465cc6b44c50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R81f8081167b84d64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="Rcbf00d4129584089"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Rbf2c5905ee584023"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R170bafd45e1c42fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Re40c38ed64ba45b2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5783,6 +5783,426 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="137">
+      <x:c r="A137" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.37.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B137" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C137" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Tax Code</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D137" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E137" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to view tax codes.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F137" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G137" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">具 MD.TAX_CODE.VIEW 可按目前公司以代碼或名稱搜尋、按代碼／名稱排序及分頁稅別（含停用），顯示稅別類型（銷項／進項／兩者）與今日適用稅率；排除軟刪除及別公司資料；未選公司回 403。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H137" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/MD/requirements.md:168</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="138">
+      <x:c r="A138" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.37.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B138" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C138" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Tax Code</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D138" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E138" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to create tax codes.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F138" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G138" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">具 MD.TAX_CODE.CREATE 可建立代碼（1–30 位英數、-、_，轉大寫，公司內永久唯一含已刪除，409 MD.TAX_CODE.DUPLICATE_CODE；格式不符 400 code）、非空白名稱（200，400 name）及類型 Output／Input／Both（400 taxType）。不同公司可用相同代碼。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H138" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/MD/requirements.md:169</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="139">
+      <x:c r="A139" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.37.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B139" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C139" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Tax Code</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D139" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E139" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to edit tax codes.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F139" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G139" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">具 MD.TAX_CODE.EDIT 可帶版本修改名稱、類型與啟用狀態；代碼不可變。舊版本 409 COMMON.CONCURRENCY.CONFLICT，別公司或已刪除 404 MD.TAX_CODE.NOT_FOUND。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H139" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/MD/requirements.md:170</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="140">
+      <x:c r="A140" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.37.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B140" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C140" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Tax Code</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D140" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E140" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to delete tax codes.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F140" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G140" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">具 MD.TAX_CODE.DELETE 可帶版本軟刪除稅別，代碼仍保留；有未刪除稅率 409 MD.TAX_CODE.IN_USE。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H140" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/MD/requirements.md:171</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="141">
+      <x:c r="A141" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.38.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B141" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C141" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Tax Rate</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D141" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E141" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to view tax rates of a tax code.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F141" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G141" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MD.TAX_CODE.VIEW 可查看某稅別的稅率期間（百分比），預設按生效日新到舊、可改舊到新，可篩選某日適用的稅率，分頁；稅別不屬目前公司 404 MD.TAX_CODE.NOT_FOUND。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H141" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/MD/requirements.md:172</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="142">
+      <x:c r="A142" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.38.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B142" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C142" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Tax Rate</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D142" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E142" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to create tax rates.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F142" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G142" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MD.TAX_CODE.EDIT 可為啟用的稅別新增稅率：生效日、可空到期日（含當日；早於生效日 400 effectiveTo）、稅率 0–100 且最多 4 位小數（400 ratePercent）。同稅別未刪除的期間不可重疊（409 MD.TAX_RATE.OVERLAP）；停用稅別 422 MD.TAX_RATE.TAX_CODE_INACTIVE。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H142" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/MD/requirements.md:173</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="143">
+      <x:c r="A143" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.38.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B143" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C143" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Tax Rate</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D143" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E143" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to edit tax rates.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F143" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G143" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MD.TAX_CODE.EDIT 可帶版本修改生效日、到期日與稅率，驗證與重疊規則同新增（排除自己）；稅別不可修改；稅率不屬該稅別 404 MD.TAX_RATE.NOT_FOUND；舊版本 409。已存單據保存自己的稅率與稅額，不受影響。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H143" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/MD/requirements.md:174</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="144">
+      <x:c r="A144" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.38.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B144" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C144" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Tax Rate</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D144" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E144" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to delete tax rates.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F144" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G144" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MD.TAX_CODE.EDIT 可帶版本軟刪除稅率，刪除後該期間可重新設定；不屬該稅別 404。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H144" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/MD/requirements.md:175</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="145">
+      <x:c r="A145" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.38.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B145" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C145" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Tax Rate</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D145" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E145" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable other modules and users to look up the tax rate of a business date and direction.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F145" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G145" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">ITaxRateLookup.GetRatePercentAsync 與 GET /api/v1/md/tax-rates/lookup?taxCode=&amp;direction=&amp;date=（MD.TAX_CODE.VIEW）回傳涵蓋該業務日期的稅率百分比，代碼不分大小寫；停用稅別仍可查詢；稅別不存在 404 MD.TAX_CODE.NOT_FOUND；銷項查進項專用稅別（或相反）422 MD.TAX_RATE.DIRECTION_MISMATCH；沒有稅率 422 MD.TAX_RATE.NOT_FOUND。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H145" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/MD/requirements.md:176</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="146">
+      <x:c r="A146" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.38.6</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B146" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C146" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Tax Rate</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D146" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E146" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should calculate line tax amounts with decimal and currency rounding.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F146" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G146" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Tax.Calculate 與 ITaxRateLookup.CalculateAsync、POST /api/v1/md/tax-rates/calculate（MD.TAX_CODE.VIEW）：未稅金額 → 未稅 = 取整（金額）、稅額 = 取整（未稅 × 稅率 ÷ 100）、含稅 = 未稅 + 稅額；含稅金額 → 含稅 = 取整（金額）、未稅 = 取整（含稅 × 100 ÷（100 + 稅率））、稅額 = 含稅 − 未稅。取整用 Money.Round 與 ICurrencyLookup.GetPrecisionAsync 的幣別小數位（AwayFromZero），負數對稱；幣別代碼格式錯誤 400 currencyCode。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H146" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/MD/requirements.md:177</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
   </x:sheetData>
 </x:worksheet>
 </file>
@@ -7850,6 +8270,70 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.119</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B36" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C36" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">md_tax_code</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D36" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">This table stores tax codes and whether they apply to output tax, input tax or both.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E36" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F36" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.37.1, REQ_F4118.37.2, REQ_F4118.37.3, REQ_F4118.37.4</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.120</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B37" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C37" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">md_tax_rate</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D37" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">This table stores the effective periods and percentages of tax codes.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E37" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F37" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.38.1, REQ_F4118.38.2, REQ_F4118.38.3, REQ_F4118.38.4, REQ_F4118.38.5, REQ_F4118.38.6</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
   </x:sheetData>
 </x:worksheet>
 </file>
@@ -7860,7 +8344,7 @@
     <x:col min="1" max="1" width="17" customWidth="1"/>
     <x:col min="2" max="2" width="15" customWidth="1"/>
     <x:col min="3" max="3" width="60" customWidth="1"/>
-    <x:col min="4" max="4" width="49" customWidth="1"/>
+    <x:col min="4" max="4" width="52" customWidth="1"/>
     <x:col min="5" max="5" width="60" customWidth="1"/>
     <x:col min="6" max="6" width="23" customWidth="1"/>
     <x:col min="7" max="7" width="60" customWidth="1"/>
@@ -20063,6 +20547,861 @@
         </x:is>
       </x:c>
       <x:c r="K214" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="215">
+      <x:c r="A215" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.83.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B215" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.83</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C215" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Tax Code View Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D215" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Search (Input)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E215" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">搜尋代碼或名稱。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F215" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">找到目前公司稅別。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G215" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Text</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H215" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">任意文字</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I215" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.83.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J215" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K215" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="216">
+      <x:c r="A216" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.83.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B216" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.83</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C216" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Tax Code View Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D216" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Tax Code List (Table)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E216" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">代碼、名稱、適用類型、今日稅率、狀態；代碼與名稱可排序，伺服器分頁；每列有稅率／試算／編輯／刪除。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F216" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">查看稅別與目前稅率。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G216" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Table</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H216" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">每頁 10／20／50／100／200</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I216" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.84.1, REQ_IO_A8.85.1, REQ_IO_A8.86.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J216" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K216" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="217">
+      <x:c r="A217" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.83.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B217" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.83</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C217" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Tax Code View Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D217" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Delete (Button)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E217" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">二次確認後帶版本軟刪除；有稅率時顯示 IN_USE。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F217" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">移除未使用的稅別。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G217" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Button</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H217" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">DELETE 權限</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I217" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.83.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J217" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K217" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="218">
+      <x:c r="A218" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.84.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B218" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.84</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C218" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Tax Code Edit Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D218" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Code (Input)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E218" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">建立時填寫並轉大寫，編輯時唯讀。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F218" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">公司內永久唯一識別。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G218" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Text</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H218" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1–30 位英數、-、_</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I218" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.83.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J218" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K218" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="219">
+      <x:c r="A219" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.84.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B219" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.84</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C219" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Tax Code Edit Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D219" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Name (Input)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E219" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">名稱必填。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F219" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">顯示稅別。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G219" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Text</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H219" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">非空白，最多 200 字</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I219" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.83.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J219" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K219" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="220">
+      <x:c r="A220" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.84.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B220" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.84</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C220" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Tax Code Edit Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D220" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Applies To (Select)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E220" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">銷項（Output）、進項（Input）或兩者（Both），預設兩者。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F220" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">限制可用的單據方向。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G220" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Enum</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H220" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Output／Input／Both</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I220" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.83.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J220" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K220" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="221">
+      <x:c r="A221" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.84.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B221" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.84</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C221" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Tax Code Edit Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D221" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Active (Checkbox)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E221" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">只在編輯時出現；帶 version 送出。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F221" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">停用不再使用的稅別。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G221" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Boolean</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H221" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">啟用／停用</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I221" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.83.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J221" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K221" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="222">
+      <x:c r="A222" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.85.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B222" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.85</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C222" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Tax Rate Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D222" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Rate List (Table)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E222" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">生效日、到期日（空白顯示持續有效）、稅率百分比、編輯／刪除；按生效日新到舊，伺服器分頁。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F222" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">查看稅率期間。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G222" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Table</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H222" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">每頁 10</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I222" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.83.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J222" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K222" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="223">
+      <x:c r="A223" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.85.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B223" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.85</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C223" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Tax Rate Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D223" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Effective On (Date Picker)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E223" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">只列出該日適用的稅率；「顯示全部」清除。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F223" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">查單據日的稅率。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G223" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Date</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H223" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">yyyy-MM-dd</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I223" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.85.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J223" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K223" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="224">
+      <x:c r="A224" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.85.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B224" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.85</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C224" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Tax Rate Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D224" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">From / To (Date Picker)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E224" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">生效日必填；到期日可空（持續有效），不可早於生效日。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F224" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">設定稅率期間。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G224" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Date</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H224" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">期間含首尾，不可與同稅別重疊</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I224" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.85.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J224" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K224" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="225">
+      <x:c r="A225" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.85.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B225" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.85</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C225" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Tax Rate Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D225" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Rate % (Input)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E225" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">稅率百分比。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F225" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">設定稅率。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G225" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Decimal</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H225" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">0–100，最多 4 位小數</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I225" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.85.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J225" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K225" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="226">
+      <x:c r="A226" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.85.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B226" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.85</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C226" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Tax Rate Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D226" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Delete (Button)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E226" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">確認後帶版本刪除稅率。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F226" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">移除錯誤稅率，期間可重設。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G226" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Action</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H226" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MD.TAX_CODE.EDIT</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I226" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.85.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J226" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K226" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="227">
+      <x:c r="A227" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.86.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B227" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.86</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C227" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Tax Calculation Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D227" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Direction / Date (Select, Date Picker)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E227" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">方向依稅別類型限制；業務日期預設今日。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F227" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">取得該日適用稅率。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G227" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Enum／Date</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H227" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Output／Input；yyyy-MM-dd</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I227" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.86.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J227" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K227" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="228">
+      <x:c r="A228" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.86.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B228" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.86</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C228" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Tax Calculation Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D228" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Currency / Amount / Includes Tax (Input, Checkbox)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E228" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">幣別代碼轉大寫；金額可為負數；勾選表示金額已含稅。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F228" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">依幣別精度試算。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G228" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Text／Decimal／Boolean</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H228" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">3 個英文字母；最多 11 位整數及 4 位小數</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I228" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.86.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J228" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K228" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="229">
+      <x:c r="A229" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.86.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B229" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.86</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C229" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Tax Calculation Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D229" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Result (Label)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E229" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">稅率、未稅、稅額、含稅；含稅 = 未稅 + 稅額；方向不符或無稅率顯示錯誤。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F229" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">確認稅額計算。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G229" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Decimal</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H229" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">依幣別小數位捨入</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I229" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.86.1, REQ_IO_A8.86.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J229" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K229" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Developer</x:t>
         </x:is>
@@ -25116,6 +26455,376 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="137">
+      <x:c r="A137" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.37.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B137" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to view tax codes.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C137" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.119</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D137" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.83</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E137" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.83.1, REQ_IO_A8.83.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F137" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MD-TAX-001, MD-TAX-004, MD-TAX-UI-001, MD-TAX-UI-002</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G137" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="138">
+      <x:c r="A138" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.37.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B138" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to create tax codes.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C138" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.119</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D138" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.84</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E138" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.84.1, REQ_IO_A8.84.2, REQ_IO_A8.84.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F138" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MD-TAX-001, MD-TAX-UI-001, MD-TAX-UI-002</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G138" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="139">
+      <x:c r="A139" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.37.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B139" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to edit tax codes.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C139" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.119</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D139" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.84</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E139" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.84.1, REQ_IO_A8.84.2, REQ_IO_A8.84.3, REQ_IO_A8.84.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F139" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MD-TAX-003, MD-TAX-UI-001, MD-TAX-UI-002</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G139" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="140">
+      <x:c r="A140" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.37.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B140" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to delete tax codes.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C140" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.119</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D140" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.83</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E140" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.83.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F140" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MD-TAX-001, MD-TAX-UI-001, MD-TAX-UI-002</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G140" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="141">
+      <x:c r="A141" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.38.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B141" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to view tax rates of a tax code.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C141" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.120</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D141" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.85</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E141" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.85.1, REQ_IO_A8.85.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F141" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MD-TAX-001, MD-TAX-004, MD-TAX-UI-001, MD-TAX-UI-002</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G141" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="142">
+      <x:c r="A142" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.38.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B142" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to create tax rates.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C142" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.120</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D142" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.85</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E142" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.85.3, REQ_IO_A8.85.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F142" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MD-TAX-001, MD-TAX-003, MD-TAX-UI-001, MD-TAX-UI-002</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G142" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="143">
+      <x:c r="A143" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.38.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B143" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to edit tax rates.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C143" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.120</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D143" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.85</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E143" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.85.3, REQ_IO_A8.85.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F143" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MD-TAX-003, MD-TAX-UI-001, MD-TAX-UI-002</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G143" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="144">
+      <x:c r="A144" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.38.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B144" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to delete tax rates.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C144" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.120</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D144" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.85</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E144" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.85.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F144" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MD-TAX-001, MD-TAX-UI-001, MD-TAX-UI-002</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G144" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="145">
+      <x:c r="A145" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.38.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B145" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable other modules and users to look up the tax rate of a business date and direction.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C145" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.120</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D145" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.86</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E145" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.86.1, REQ_IO_A8.86.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F145" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MD-TAX-002, MD-TAX-003, MD-TAX-005</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G145" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="146">
+      <x:c r="A146" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.38.6</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B146" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should calculate line tax amounts with decimal and currency rounding.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C146" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.120</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D146" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.86</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E146" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.86.2, REQ_IO_A8.86.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F146" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MD-TAX-CALC-001, MD-TAX-002, MD-TAX-005, MD-TAX-UI-001, MD-TAX-UI-002</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G146" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
   </x:sheetData>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
feat(md): add multilingual chart of accounts page
- /md/accounts tree page (interfaces 8.87-8.88): add top-level account
  with type default direction, add subaccount with parent code prefix
  and inherited read-only type, edit name/direction/status, delete
- Generic tree helpers shared with item categories
- MD.ACCOUNT.* error codes in three languages; menu and route
- Vitest +11, Playwright +2; WU-MD-019 done

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R09e6252ba4e345f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R30ab56a53ed843a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R6d383a82735d47e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R87bc465cc6b44c50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R81f8081167b84d64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="Rcbf00d4129584089"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Rbf2c5905ee584023"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R170bafd45e1c42fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Re40c38ed64ba45b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R6cd25e8e122f499b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R97a6fbdf10b04522"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Rb1c58337db4a4d94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R1d9276d2804f476c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R663088a6b7d84060"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R60c1064d6c0a4779"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Rcabbc8648a384c9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R568360d0203f4a1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Raaed4ca29ab04f72"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -6203,6 +6203,216 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="147">
+      <x:c r="A147" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.39.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B147" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C147" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Chart of Accounts</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D147" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E147" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to view the chart of accounts.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F147" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G147" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">具 MD.ACCOUNT.VIEW 可一次取得目前公司全部未刪除科目（含停用，按代碼排序），每筆有上層、類別、借貸方向、啟用狀態與是否可過帳（啟用且沒有子科目）；排除別公司資料；未選公司回 403。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H147" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/MD/requirements.md:189</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="148">
+      <x:c r="A148" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.39.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B148" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C148" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Chart of Accounts</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D148" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E148" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to create accounts.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F148" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G148" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">具 MD.ACCOUNT.CREATE 可建立科目：代碼 1–30 位數字（400 code），公司內永久唯一含已刪除（409 MD.ACCOUNT.DUPLICATE_CODE）；名稱必填（400 name）；上層可空，若有須為本公司啟用科目（422 MD.ACCOUNT.INVALID_PARENT），代碼須以上層代碼開頭且較長（422 MD.ACCOUNT.CODE_PREFIX），上層已被使用不可再分子科目（422 MD.ACCOUNT.PARENT_IN_USE）。根科目必填類別 Asset／Liability／Equity／Cost／Revenue／Expense（400 accountType）；子科目可省略類別而沿用上層，不同則 422 MD.ACCOUNT.TYPE_MISMATCH。借貸方向 Debit／Credit 可省略，按類別預設（資產、成本、費用借方；其餘貸方）。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H148" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/MD/requirements.md:190</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="149">
+      <x:c r="A149" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.39.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B149" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C149" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Chart of Accounts</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D149" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E149" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to edit accounts.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F149" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G149" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">具 MD.ACCOUNT.EDIT 可帶版本修改名稱、借貸方向與啟用狀態；代碼、上層與類別不可修改。已被使用的科目不可改方向（409 MD.ACCOUNT.IN_USE）；有啟用子科目不可停用（422 MD.ACCOUNT.HAS_ACTIVE_CHILDREN）；上層停用時不可啟用（422 MD.ACCOUNT.PARENT_INACTIVE）。舊版本 409 COMMON.CONCURRENCY.CONFLICT，別公司或已刪除 404 MD.ACCOUNT.NOT_FOUND。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H149" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/MD/requirements.md:191</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="150">
+      <x:c r="A150" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.39.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B150" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C150" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Chart of Accounts</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D150" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E150" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to delete accounts.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F150" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G150" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">具 MD.ACCOUNT.DELETE 可帶版本軟刪除末級科目，代碼仍保留；有子科目 409 MD.ACCOUNT.HAS_CHILDREN；已被使用 409 MD.ACCOUNT.IN_USE。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H150" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/MD/requirements.md:192</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="151">
+      <x:c r="A151" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.39.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B151" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C151" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Chart of Accounts</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D151" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E151" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable other modules to look up accounts and validate postable accounts.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F151" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G151" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">IChartOfAccounts.FindAsync(code) 回傳科目資料（含停用，不存在回 null）；RequirePostableAsync(code) 不存在 404 MD.ACCOUNT.NOT_FOUND、停用 422 MD.ACCOUNT.INACTIVE、有子科目 422 MD.ACCOUNT.NOT_POSTABLE。使用檢查經使用方實作的 IAccountUsage，MD 不讀 FI 表。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H151" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/MD/requirements.md:193</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
   </x:sheetData>
 </x:worksheet>
 </file>
@@ -8331,6 +8541,38 @@
       <x:c r="F37" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">REQ_F4118.38.1, REQ_F4118.38.2, REQ_F4118.38.3, REQ_F4118.38.4, REQ_F4118.38.5, REQ_F4118.38.6</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.121</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B38" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C38" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">md_account</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D38" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">This table stores the chart of accounts with parent accounts, account types and normal balance directions.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E38" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F38" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.39.1, REQ_F4118.39.2, REQ_F4118.39.3, REQ_F4118.39.4, REQ_F4118.39.5</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -21407,6 +21649,462 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="230">
+      <x:c r="A230" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.87.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B230" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.87</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C230" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Account View Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D230" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Search (Input)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E230" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">搜尋代碼或名稱（不分大小寫），保留命中科目的上層。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F230" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">在科目樹中找到科目。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G230" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Text</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H230" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">任意文字</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I230" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.87.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J230" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K230" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="231">
+      <x:c r="A231" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.87.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B231" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.87</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C231" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Account View Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D231" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Account Tree (Table)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E231" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">代碼（按層縮排）、名稱、類別、餘額方向、過帳（可過帳／彙總）、狀態；每列有新增子科目（只限啟用科目）／編輯／刪除。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F231" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">查看科目階層與可過帳科目。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G231" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Tree Table</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H231" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">不分頁，含停用</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I231" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.88.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J231" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K231" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="232">
+      <x:c r="A232" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.87.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B232" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.87</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C232" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Account View Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D232" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Delete (Button)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E232" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">二次確認後帶版本軟刪除；有子科目顯示 HAS_CHILDREN，已被使用顯示 IN_USE。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F232" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">移除未使用的末級科目。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G232" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Button</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H232" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">DELETE 權限</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I232" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.87.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J232" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K232" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="233">
+      <x:c r="A233" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.88.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B233" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.88</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C233" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Account Edit Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D233" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Code (Input)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E233" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">新增時填寫，子科目預填上層代碼；編輯時唯讀。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F233" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">公司內永久唯一識別。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G233" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Text</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H233" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1–30 位數字；子科目須以上層代碼開頭且較長</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I233" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.87.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J233" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K233" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="234">
+      <x:c r="A234" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.88.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B234" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.88</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C234" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Account Edit Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D234" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Name (Input)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E234" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">名稱必填。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F234" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">顯示科目。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G234" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Text</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H234" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">非空白，最多 200 字</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I234" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.87.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J234" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K234" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="235">
+      <x:c r="A235" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.88.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B235" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.88</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C235" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Account Edit Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D235" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Type (Select)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E235" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">一級科目必選；子科目沿用上層並唯讀；編輯時唯讀。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F235" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">決定科目在報表中的分類與預設方向。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G235" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Enum</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H235" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Asset／Liability／Equity／Cost／Revenue／Expense</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I235" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.88.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J235" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K235" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="236">
+      <x:c r="A236" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.88.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B236" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.88</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C236" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Account Edit Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D236" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Normal Balance (Select)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E236" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">按類別預設，可改；已被使用時改方向顯示 IN_USE。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F236" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">決定餘額正負方向。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G236" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Enum</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H236" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Debit／Credit</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I236" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.88.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J236" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K236" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="237">
+      <x:c r="A237" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.88.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B237" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.88</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C237" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Account Edit Interface</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D237" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Active (Checkbox)</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E237" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">只在編輯時出現；有啟用子科目不可停用，上層停用時不可啟用。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F237" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">停用不再使用的科目。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G237" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Boolean</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H237" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">啟用／停用</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="I237" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.87.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="J237" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="K237" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
   </x:sheetData>
 </x:worksheet>
 </file>
@@ -26825,6 +27523,191 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="147">
+      <x:c r="A147" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.39.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B147" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to view the chart of accounts.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C147" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.121</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D147" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.87</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E147" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.87.1, REQ_IO_A8.87.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F147" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MD-ACC-001, MD-ACC-005, MD-ACC-UI-001, MD-ACC-UI-002, MD-ACC-008</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G147" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="148">
+      <x:c r="A148" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.39.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B148" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to create accounts.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C148" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.121</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D148" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.88</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E148" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.88.1, REQ_IO_A8.88.2, REQ_IO_A8.88.3, REQ_IO_A8.88.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F148" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MD-ACC-001, MD-ACC-002, MD-ACC-003, MD-ACC-005, MD-ACC-UI-001, MD-ACC-UI-002, MD-ACC-006, MD-ACC-007</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G148" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="149">
+      <x:c r="A149" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.39.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B149" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to edit accounts.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C149" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.121</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D149" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.88</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E149" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.88.2, REQ_IO_A8.88.4, REQ_IO_A8.88.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F149" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MD-ACC-001, MD-ACC-002, MD-ACC-003, MD-ACC-UI-001, MD-ACC-UI-002</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G149" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="150">
+      <x:c r="A150" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.39.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B150" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to delete accounts.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C150" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.121</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D150" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.8.87</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E150" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_IO_A8.87.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F150" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MD-ACC-002, MD-ACC-003, MD-ACC-UI-001, MD-ACC-UI-002, MD-ACC-007</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G150" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Covered</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="151">
+      <x:c r="A151" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.39.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B151" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable other modules to look up accounts and validate postable accounts.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C151" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.121</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D151" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E151" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F151" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">MD-ACC-003, MD-ACC-004, MD-ACC-008</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G151" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
   </x:sheetData>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
feat(md): add item images backend
WU-MD-013a (ADR-045): md_item_image with content-based PNG/JPEG checks,
2 MB / 16-4096 px / 10 per item limits, exactly one primary image,
upload/content(ETag)/update/delete API under MD.ITEM.VIEW/EDIT.
Move ImageInspector to MyERP.Shared.Infrastructure.Imaging for reuse.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R9be6f2215b7a4fa1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R8a1965e9ef60496e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R54fa6d0a70e549af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Ra9c08508de7b4389"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R934e91dfd9b14603"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="Rfec75186042b4423"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Re763ecc9eeb641af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R3396eca424d24ac4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rf035e1b72f38454c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R0f323d4f917f484e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Rbbeeb282436844df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R53039d33f01c4685"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R91f40e4f79994389"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Re5b84a9570f64884"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R4596265e77364586"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R95125555f4c24d29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R01d81f9cc15e4158"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rc60a5999908142f3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -8219,6 +8219,174 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="195">
+      <x:c r="A195" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.44.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B195" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C195" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Product Image（Product Image Interface 8.15）</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D195" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E195" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to view the images of a product.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F195" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G195" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">具 MD.ITEM.VIEW 可列出目前公司某物料的圖片中繼資料（類型、檔名、大小、寬高、排序號、主圖、版本，不含內容），主圖排第一，其餘按排序號、id；可下載內容（image/png／image/jpeg inline，ETag 為版本，帶 If-None-Match 未變更回 304）。物料不存在或屬別公司 404 MD.ITEM.NOT_FOUND；圖片不屬該物料 404 MD.ITEM_IMAGE.NOT_FOUND；未選公司 403。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H195" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/MD/requirements.md:333</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="196">
+      <x:c r="A196" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.44.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B196" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C196" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Product Image（Product Image Interface 8.15）</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D196" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E196" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to upload images for a product.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F196" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G196" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">具 MD.ITEM.EDIT 可上傳 multipart file（可選 sortOrder 0–9999、isPrimary）。以檔案內容判斷，只接受 PNG／JPEG（422 MD.ITEM_IMAGE.UNSUPPORTED_TYPE）；1 B–2 MB（空檔或沒有檔案 400 file，超過 422 TOO_LARGE）；寬高各 16–4096 像素（422 INVALID_DIMENSIONS）；每物料最多 10 張（422 LIMIT_REACHED）。排序號省略時為目前最大值 + 1；第一張或要求主圖時成為主圖並取消原主圖。檔名只保留最後一段、去除控制字元、最多 200 字。停用物料仍可上傳。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H196" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/MD/requirements.md:334</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="197">
+      <x:c r="A197" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.44.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B197" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C197" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Product Image（Product Image Interface 8.15）</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D197" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E197" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to set the primary image and display order of product images.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F197" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G197" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">具 MD.ITEM.EDIT 可帶版本修改排序號（0–9999，400 sortOrder）或把圖片設為主圖（原主圖自動取消並遞增版本）；不可直接取消主圖（400 isPrimary）；舊版本 409。併發上傳或修改以公司鎖序列化，有圖片的物料恰好一張主圖。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H197" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/MD/requirements.md:335</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="198">
+      <x:c r="A198" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.44.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B198" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C198" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Product Image（Product Image Interface 8.15）</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D198" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E198" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to delete product images.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F198" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G198" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">具 MD.ITEM.EDIT 可帶版本實體刪除圖片（稽核記錄 DELETE）；刪除主圖時由排序號最小（相同時 id 最小）的圖片接任主圖；圖片不存在 404 MD.ITEM_IMAGE.NOT_FOUND；舊版本 409。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H198" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/MD/requirements.md:336</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
   </x:sheetData>
 </x:worksheet>
 </file>
@@ -10667,6 +10835,38 @@
       <x:c r="F47" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">REQ_F4118.43.1, REQ_F4118.43.2, REQ_F4118.43.3, REQ_F4118.43.4</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.131</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B48" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C48" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">md_item_image</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D48" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">This table stores the images of products.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E48" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F48" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.44.1, REQ_F4118.44.2, REQ_F4118.44.3, REQ_F4118.44.4</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -34072,6 +34272,154 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="195">
+      <x:c r="A195" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.44.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B195" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to view the images of a product.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C195" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.131</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D195" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E195" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F195" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="G195" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="196">
+      <x:c r="A196" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.44.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B196" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to upload images for a product.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C196" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.131</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D196" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E196" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F196" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="G196" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="197">
+      <x:c r="A197" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.44.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B197" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to set the primary image and display order of product images.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C197" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.131</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D197" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E197" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F197" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="G197" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="198">
+      <x:c r="A198" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.44.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B198" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to delete product images.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C198" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.131</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D198" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E198" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F198" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="G198" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
   </x:sheetData>
 </x:worksheet>
 </file>
@@ -34084,7 +34432,7 @@
     <x:col min="3" max="3" width="60" customWidth="1"/>
     <x:col min="4" max="4" width="14" customWidth="1"/>
     <x:col min="5" max="5" width="32" customWidth="1"/>
-    <x:col min="6" max="6" width="26" customWidth="1"/>
+    <x:col min="6" max="6" width="33" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -44579,7 +44927,7 @@
       </x:c>
       <x:c r="F328" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">未開始</x:t>
+          <x:t xml:space="preserve">進行中（API 完成 WU-MD-013a，頁面待 013c）</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -47939,7 +48287,7 @@
       </x:c>
       <x:c r="F433" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">未開始</x:t>
+          <x:t xml:space="preserve">後端完成（WU-MD-013a；頁面待 013c）</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
feat(md): add item attributes backend
WU-MD-013b (ADR-045 11-13): md_item_attribute definitions (sort order,
item count, delete blocked when used) and md_item_attribute_value
(one value per item x attribute). API /api/v1/md/item-attributes under
MD.ITEM_ATTRIBUTE.* and GET/PUT /api/v1/md/items/{itemId}/attributes
(bulk replace, max 50, new attributes must be active, company applock).
REQ_F4118.45.1-6, REQ_DS43.132-133, MD-ATTR-001..004.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R0f323d4f917f484e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Rbbeeb282436844df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R53039d33f01c4685"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R91f40e4f79994389"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Re5b84a9570f64884"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R4596265e77364586"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R95125555f4c24d29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R01d81f9cc15e4158"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rc60a5999908142f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R41a4ad5029934391"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Rd173e0028c9f46ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R25ac6b2193244a05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R056afaffc558426c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R5e08c231c96344ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R834fe5442a5b40fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Rfbcff870837a4661"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R4712b83df6644a5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R255d24aba3b44e2a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -8387,6 +8387,258 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="199">
+      <x:c r="A199" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.45.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B199" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C199" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Product Attribute（Product Details Interface 8.16）</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D199" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E199" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to view the list of product attributes.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F199" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G199" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">具 MD.ITEM_ATTRIBUTE.VIEW 可分頁查詢目前公司未刪除的屬性（含停用），回傳代碼、名稱、排序號、使用物料數、啟用、版本；預設按排序號、同號按代碼，可按 sortOrder／code／name（含倒序），其他欄位 400 sort；關鍵字比對代碼與名稱。未選公司 403。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H199" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/MD/requirements.md:350</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="200">
+      <x:c r="A200" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.45.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B200" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C200" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Product Attribute（Product Details Interface 8.16）</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D200" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E200" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to create product attributes.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F200" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G200" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">具 MD.ITEM_ATTRIBUTE.CREATE 可建立屬性：代碼 1–30 個英數字／-／_，轉大寫，公司內永久唯一（含已刪除，409 MD.ITEM_ATTRIBUTE.DUPLICATE_CODE）；名稱必填、最多 200 字；排序號 0–9999（400 sortOrder）。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H200" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/MD/requirements.md:351</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="201">
+      <x:c r="A201" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.45.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B201" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C201" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Product Attribute（Product Details Interface 8.16）</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D201" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E201" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to edit product attributes.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F201" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G201" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">具 MD.ITEM_ATTRIBUTE.EDIT 可帶版本修改名稱、排序號與啟用狀態，代碼不可改；被物料使用的屬性也可停用；舊版本 409；不存在或屬別公司 404 MD.ITEM_ATTRIBUTE.NOT_FOUND。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H201" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/MD/requirements.md:352</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="202">
+      <x:c r="A202" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.45.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B202" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C202" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Product Attribute（Product Details Interface 8.16）</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D202" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E202" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to delete product attributes.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F202" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G202" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">具 MD.ITEM_ATTRIBUTE.DELETE 可帶版本軟刪除；任何物料仍有該屬性值時 409 MD.ITEM_ATTRIBUTE.IN_USE（請改為停用）。刪除與物料屬性整批取代共用公司鎖 md_item_attribute。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H202" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/MD/requirements.md:353</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="203">
+      <x:c r="A203" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.45.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B203" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C203" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Product Attribute（Product Details Interface 8.16）</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D203" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E203" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to view the attribute values of a product.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F203" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G203" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">具 MD.ITEM.VIEW 可列出物料的屬性值（屬性 id、代碼、名稱、排序號、屬性是否啟用、值），按屬性排序號、代碼；含已停用屬性。物料不存在或屬別公司 404 MD.ITEM.NOT_FOUND。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H203" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/MD/requirements.md:354</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="204">
+      <x:c r="A204" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.45.6</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B204" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Settings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C204" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Product Attribute（Product Details Interface 8.16）</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D204" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E204" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to set the attribute values of a product.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F204" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="G204" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">具 MD.ITEM.EDIT 可以完整集合 PUT 取代物料的屬性值：未列出的刪除、值改變的更新、新屬性新增，空集合清除全部；最多 50 個（400 attributes）；同一屬性只可出現一次、屬性 id 必填（400 attributes[i].attributeId）；值去除前後空白後必填、最多 200 字（400 attributes[i].value）；新設定的屬性須為本公司未刪除的啟用屬性，原有值的屬性停用後仍可保留與修改值（否則 400 attributes[i].attributeId）。停用物料仍可維護。取代在公司鎖內進行，並發取代不會產生重複值；整批驗證失敗時不寫入任何資料。</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="H204" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">docs/02-modules/MD/requirements.md:355</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
   </x:sheetData>
 </x:worksheet>
 </file>
@@ -10867,6 +11119,70 @@
       <x:c r="F48" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">REQ_F4118.44.1, REQ_F4118.44.2, REQ_F4118.44.3, REQ_F4118.44.4</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.132</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B49" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C49" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">md_item_attribute</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D49" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">This table stores the attribute definitions of products.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E49" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F49" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.45.1, REQ_F4118.45.2, REQ_F4118.45.3, REQ_F4118.45.4</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.133</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B50" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C50" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">md_item_attribute_value</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D50" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">This table stores the attribute values of products.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E50" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F50" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.45.5, REQ_F4118.45.6</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -34420,6 +34736,228 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="199">
+      <x:c r="A199" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.45.1</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B199" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to view the list of product attributes.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C199" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.132</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D199" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E199" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F199" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="G199" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="200">
+      <x:c r="A200" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.45.2</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B200" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to create product attributes.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C200" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.132</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D200" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E200" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F200" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="G200" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="201">
+      <x:c r="A201" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.45.3</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B201" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to edit product attributes.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C201" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.132</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D201" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E201" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F201" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="G201" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="202">
+      <x:c r="A202" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.45.4</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B202" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to delete product attributes.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C202" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.132</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D202" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E202" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F202" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="G202" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="203">
+      <x:c r="A203" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.45.5</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B203" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to view the attribute values of a product.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C203" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.133</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D203" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E203" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F203" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="G203" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="204">
+      <x:c r="A204" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4118.45.6</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B204" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">System should enable user to set the attribute values of a product.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C204" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.133</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D204" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="E204" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="F204" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve"/>
+        </x:is>
+      </x:c>
+      <x:c r="G204" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Partial</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
   </x:sheetData>
 </x:worksheet>
 </file>
@@ -34432,7 +34970,7 @@
     <x:col min="3" max="3" width="60" customWidth="1"/>
     <x:col min="4" max="4" width="14" customWidth="1"/>
     <x:col min="5" max="5" width="32" customWidth="1"/>
-    <x:col min="6" max="6" width="33" customWidth="1"/>
+    <x:col min="6" max="6" width="38" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -44959,7 +45497,7 @@
       </x:c>
       <x:c r="F329" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">未開始</x:t>
+          <x:t xml:space="preserve">進行中（物料屬性 API 完成 WU-MD-013b，頁面待 013c）</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -47391,7 +47929,7 @@
       </x:c>
       <x:c r="F405" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">未開始</x:t>
+          <x:t xml:space="preserve">後端完成（WU-MD-013b；頁面待 013c）</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
feat(md): complete item import UI
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R2077458f4eec44f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Rdf9e75effaa24e96"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R06bc2edc435c455e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Rc2e1a4693df44182"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R561f0ff866d24608"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R486ad03fb1f84fab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R8cdc5c4768da4907"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="Rae7f8f9943144fc3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R5131dabb9efd4887"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R26a8a3a855d543d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R5eda09b967334182"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Ree7a2bba51af4401"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R6f75279eb11e4108"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R9e553dca94ba4a35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="Rddd244580ab945c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Ra329b7e91d5a4b06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R0824faac572447bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R6ff59ed5d9044996"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -28642,7 +28642,7 @@
       </x:c>
       <x:c r="F17" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MD-ITEM-IMPORT-001, MD-ITEM-IMPORT-002, MD-ITEM-IMPORT-003</x:t>
+          <x:t xml:space="preserve">MD-ITEM-IMPORT-001, MD-ITEM-IMPORT-002, MD-ITEM-IMPORT-003, MD-ITEM-IMPORT-UI-001, MD-ITEM-IMPORT-UI-002</x:t>
         </x:is>
       </x:c>
       <x:c r="G17" s="2" t="inlineStr">

</xml_diff>

<commit_message>
test(md): complete MD module regression (WU-MD-022e)
- Full regression: backend 761/761, frontend 586/586, mocked E2E 122 passed,
  real API E2E login 3/3 + MD 2/2.
- Fix duplicate test case ID MD-CUS-REV-004 -> 005 found by docgen.
- Add SRS 2.2 Setting Management narrative source; regenerate docs (0 errors).
- Parity check found product delete (REQ_F4118.3.4) missing: add WU-MD-028
  and move the v0.2.0-md tag to WU-MD-022f; initial stock interface moves to INV.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R1edbc55789b74e39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Recfd53f2a1384915"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Rf630f56dbe494149"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Rf2fb6afee4de4da5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R7afd951efd904f03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="Ra7c2cec4ef974efb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Rb60e4a718afe4b64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R74fd4e5893394944"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R18f5b51640c0496b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R1a0fa17dd865406d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R9050c45a0bbd4838"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Rad47735cad4d40fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R5b080b2ca0d14fbb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R31664874c71c44ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R99490abe423e4aa8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R502f5bfa8b1a4c47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="Rcae45b9c4ab04a53"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Re80d9ffaa8604125"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -398,7 +398,7 @@
       </x:c>
       <x:c r="G8" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">新客戶為 Pending、不可作交易；MD.CUSTOMER.APPROVE 帶版本送審，SYS 按 MD.CUSTOMER 流程核准，無適用步驟即自動核准。已核准不可重送；舊客戶遷移為 Approved。</x:t>
+          <x:t xml:space="preserve">新客戶為 Pending、不可作交易；MD.CUSTOMER.APPROVE 帶版本送審，SYS 按 MD.CUSTOMER 流程核准，無適用步驟即自動核准。已核准不可重送；舊客戶遷移為 Approved。審批中（SYS 實例為 Pending）修改回 422 MD.CUSTOMER.APPROVAL_PENDING，核准後的維護不需重審（ADR-048）。</x:t>
         </x:is>
       </x:c>
       <x:c r="H8" s="2" t="inlineStr">
@@ -482,7 +482,7 @@
       </x:c>
       <x:c r="G10" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MD.CUSTOMER.DELETE 帶版本軟刪除非待審客戶；由使用方 ICustomerUsage 契約回報單據引用，已引用回 409；代碼保留不可重用、列表不顯示。</x:t>
+          <x:t xml:space="preserve">MD.CUSTOMER.DELETE 帶版本軟刪除不在審批中的客戶（SYS 審批實例仍為 Pending 回 422 MD.CUSTOMER.APPROVAL_PENDING；從未送審或已撤回的待審客戶可刪，ADR-048）；由使用方 ICustomerUsage 契約回報單據引用，已引用回 409；代碼保留不可重用、列表不顯示。</x:t>
         </x:is>
       </x:c>
       <x:c r="H10" s="2" t="inlineStr">
@@ -734,7 +734,7 @@
       </x:c>
       <x:c r="G16" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">新供應商（含匯入）為 Pending、不可作交易；MD.SUPPLIER.APPROVE 帶版本送審，SYS 按 MD.SUPPLIER 流程核准，無適用步驟即自動核准。已核准再送審回 422 MD.SUPPLIER.ALREADY_APPROVED；舊供應商遷移為 Approved。交易模組經 ISupplierLookup.RequireApprovedAsync 只取得啟用且核准者，否則 422 MD.SUPPLIER.NOT_APPROVED。</x:t>
+          <x:t xml:space="preserve">新供應商（含匯入）為 Pending、不可作交易；MD.SUPPLIER.APPROVE 帶版本送審，SYS 按 MD.SUPPLIER 流程核准，無適用步驟即自動核准。已核准再送審回 422 MD.SUPPLIER.ALREADY_APPROVED；舊供應商遷移為 Approved。交易模組經 ISupplierLookup.RequireApprovedAsync 只取得啟用且核准者，否則 422 MD.SUPPLIER.NOT_APPROVED。審批中（SYS 實例為 Pending）修改回 422 MD.SUPPLIER.APPROVAL_PENDING，核准後的維護不需重審（ADR-048）。</x:t>
         </x:is>
       </x:c>
       <x:c r="H16" s="2" t="inlineStr">
@@ -818,7 +818,7 @@
       </x:c>
       <x:c r="G18" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MD.SUPPLIER.DELETE 帶版本軟刪除非待審供應商（待審 422 MD.SUPPLIER.APPROVAL_PENDING）；由使用方 ISupplierUsage 契約回報單據引用，已引用回 409 MD.SUPPLIER.IN_USE；代碼保留不可重用、列表不顯示。</x:t>
+          <x:t xml:space="preserve">MD.SUPPLIER.DELETE 帶版本軟刪除不在審批中的供應商（SYS 審批實例仍為 Pending 回 422 MD.SUPPLIER.APPROVAL_PENDING；從未送審或已撤回的待審供應商可刪，ADR-048）；由使用方 ISupplierUsage 契約回報單據引用，已引用回 409 MD.SUPPLIER.IN_USE；代碼保留不可重用、列表不顯示。</x:t>
         </x:is>
       </x:c>
       <x:c r="H18" s="2" t="inlineStr">
@@ -1013,7 +1013,7 @@
       </x:c>
       <x:c r="D23" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">1.0</x:t>
+          <x:t xml:space="preserve">1.1</x:t>
         </x:is>
       </x:c>
       <x:c r="E23" s="2" t="inlineStr">
@@ -1028,7 +1028,7 @@
       </x:c>
       <x:c r="G23" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MD.ITEM.EDIT 可帶版本修改名稱、規格、基本單位、品牌、分類、啟用狀態，代碼不可改；原參照停用後可保留，重新選擇須啟用。舊版本 409、別公司物料 404。已被物料引用的單位、品牌、分類不可刪除，只可停用。物料有專屬換算時修改基本單位回 409 MD.ITEM.BASE_UOM_LOCKED（WU-MD-012c）。</x:t>
+          <x:t xml:space="preserve">MD.ITEM.EDIT 可帶版本修改名稱、規格、基本單位、品牌、分類、啟用狀態，代碼不可改；原參照停用後可保留，重新選擇須啟用。舊版本 409、別公司物料 404。已被物料引用的單位、品牌、分類不可刪除，只可停用。物料有專屬換算（WU-MD-012c），或任何使用方 IItemUsage 回報已有庫存、交易或單據時，修改基本單位回 409 MD.ITEM.BASE_UOM_LOCKED（ADR-049）。</x:t>
         </x:is>
       </x:c>
       <x:c r="H23" s="2" t="inlineStr">
@@ -1265,7 +1265,7 @@
       </x:c>
       <x:c r="D29" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">1.0</x:t>
+          <x:t xml:space="preserve">1.1</x:t>
         </x:is>
       </x:c>
       <x:c r="E29" s="2" t="inlineStr">
@@ -1280,7 +1280,7 @@
       </x:c>
       <x:c r="G29" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">具 MD.WAREHOUSE.DELETE 可帶版本軟刪除倉庫，代碼仍保留；仍有未刪除儲位時回 409 MD.WAREHOUSE.HAS_LOCATIONS。INV 加入後，被庫存或單據引用的倉庫亦不可刪除（EP-INV 決定契約）。</x:t>
+          <x:t xml:space="preserve">具 MD.WAREHOUSE.DELETE 可帶版本軟刪除倉庫，代碼仍保留；仍有未刪除儲位時回 409 MD.WAREHOUSE.HAS_LOCATIONS；任何使用方 IWarehouseUsage 回報已被庫存或單據引用時回 409 MD.WAREHOUSE.IN_USE（ADR-049）。</x:t>
         </x:is>
       </x:c>
       <x:c r="H29" s="2" t="inlineStr">
@@ -1307,7 +1307,7 @@
       </x:c>
       <x:c r="D30" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">1.0</x:t>
+          <x:t xml:space="preserve">1.1</x:t>
         </x:is>
       </x:c>
       <x:c r="E30" s="2" t="inlineStr">
@@ -1322,7 +1322,7 @@
       </x:c>
       <x:c r="G30" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MD.WAREHOUSE.VIEW 可按倉庫以代碼或名稱搜尋、排序及分頁儲位（含停用）；MD.WAREHOUSE.EDIT 可新增（代碼規則同倉庫，在同一倉庫內永久唯一，409 MD.STORAGE_LOCATION.DUPLICATE_CODE；不同倉庫可重複）、帶版本修改名稱及啟用狀態、軟刪除。只能在啟用倉庫新增儲位（422 MD.STORAGE_LOCATION.WAREHOUSE_INACTIVE）；別公司或已刪除倉庫 404 MD.WAREHOUSE.NOT_FOUND；儲位不屬該倉庫 404 MD.STORAGE_LOCATION.NOT_FOUND；舊版本 409。</x:t>
+          <x:t xml:space="preserve">MD.WAREHOUSE.VIEW 可按倉庫以代碼或名稱搜尋、排序及分頁儲位（含停用）；MD.WAREHOUSE.EDIT 可新增（代碼規則同倉庫，在同一倉庫內永久唯一，409 MD.STORAGE_LOCATION.DUPLICATE_CODE；不同倉庫可重複）、帶版本修改名稱及啟用狀態、軟刪除（使用方 IStorageLocationUsage 回報已被庫存或交易引用時 409 MD.STORAGE_LOCATION.IN_USE，ADR-049）。只能在啟用倉庫新增儲位（422 MD.STORAGE_LOCATION.WAREHOUSE_INACTIVE）；別公司或已刪除倉庫 404 MD.WAREHOUSE.NOT_FOUND；儲位不屬該倉庫 404 MD.STORAGE_LOCATION.NOT_FOUND；舊版本 409。</x:t>
         </x:is>
       </x:c>
       <x:c r="H30" s="2" t="inlineStr">
@@ -7397,7 +7397,7 @@
       </x:c>
       <x:c r="D175" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">1.0</x:t>
+          <x:t xml:space="preserve">1.1</x:t>
         </x:is>
       </x:c>
       <x:c r="E175" s="2" t="inlineStr">
@@ -7412,7 +7412,7 @@
       </x:c>
       <x:c r="G175" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">具 MD.TAX_CODE.DELETE 可帶版本軟刪除稅別，代碼仍保留；有未刪除稅率 409 MD.TAX_CODE.IN_USE。</x:t>
+          <x:t xml:space="preserve">具 MD.TAX_CODE.DELETE 可帶版本軟刪除稅別，代碼仍保留；有未刪除稅率，或使用方 ITaxCodeUsage 回報有單據使用此稅別時 409 MD.TAX_CODE.IN_USE（ADR-049）。</x:t>
         </x:is>
       </x:c>
       <x:c r="H175" s="2" t="inlineStr">
@@ -7523,7 +7523,7 @@
       </x:c>
       <x:c r="D178" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">1.0</x:t>
+          <x:t xml:space="preserve">1.1</x:t>
         </x:is>
       </x:c>
       <x:c r="E178" s="2" t="inlineStr">
@@ -7538,7 +7538,7 @@
       </x:c>
       <x:c r="G178" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MD.TAX_CODE.EDIT 可帶版本修改生效日、到期日與稅率，驗證與重疊規則同新增（排除自己）；稅別不可修改；稅率不屬該稅別 404 MD.TAX_RATE.NOT_FOUND；舊版本 409。已存單據保存自己的稅率與稅額，不受影響。</x:t>
+          <x:t xml:space="preserve">MD.TAX_CODE.EDIT 可帶版本修改生效日、到期日與稅率，驗證與重疊規則同新增（排除自己）；稅別不可修改；稅率不屬該稅別 404 MD.TAX_RATE.NOT_FOUND；舊版本 409。已存單據保存自己的稅率與稅額，不受影響；但使用方 ITaxCodeUsage 回報有單據的業務日期落在會改變稅率的原期間部分（改百分比：整個原期間；只改期間：不再涵蓋的頭尾）時 409 MD.TAX_RATE.IN_USE（ADR-049）。</x:t>
         </x:is>
       </x:c>
       <x:c r="H178" s="2" t="inlineStr">
@@ -7565,7 +7565,7 @@
       </x:c>
       <x:c r="D179" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">1.0</x:t>
+          <x:t xml:space="preserve">1.1</x:t>
         </x:is>
       </x:c>
       <x:c r="E179" s="2" t="inlineStr">
@@ -7580,7 +7580,7 @@
       </x:c>
       <x:c r="G179" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MD.TAX_CODE.EDIT 可帶版本軟刪除稅率，刪除後該期間可重新設定；不屬該稅別 404。</x:t>
+          <x:t xml:space="preserve">MD.TAX_CODE.EDIT 可帶版本軟刪除稅率，刪除後該期間可重新設定；不屬該稅別 404；期間內已有單據 409 MD.TAX_RATE.IN_USE（ADR-049）。</x:t>
         </x:is>
       </x:c>
       <x:c r="H179" s="2" t="inlineStr">
@@ -7607,7 +7607,7 @@
       </x:c>
       <x:c r="D180" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">1.0</x:t>
+          <x:t xml:space="preserve">1.1</x:t>
         </x:is>
       </x:c>
       <x:c r="E180" s="2" t="inlineStr">
@@ -7622,7 +7622,7 @@
       </x:c>
       <x:c r="G180" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">ITaxRateLookup.GetRatePercentAsync 與 GET /api/v1/md/tax-rates/lookup?taxCode=&amp;direction=&amp;date=（MD.TAX_CODE.VIEW）回傳涵蓋該業務日期的稅率百分比，代碼不分大小寫；停用稅別仍可查詢；稅別不存在 404 MD.TAX_CODE.NOT_FOUND；銷項查進項專用稅別（或相反）422 MD.TAX_RATE.DIRECTION_MISMATCH；沒有稅率 422 MD.TAX_RATE.NOT_FOUND。</x:t>
+          <x:t xml:space="preserve">ITaxRateLookup.GetRatePercentAsync 與 GET /api/v1/md/tax-rates/lookup?taxCode=&amp;direction=&amp;date=（MD.TAX_CODE.VIEW）回傳涵蓋該業務日期的稅率百分比，代碼不分大小寫；契約預設對停用稅別回 422 MD.TAX_CODE.INACTIVE，重算歷史單據時傳 includeInactive；API 是維護頁試算工具，停用稅別仍可查詢（ADR-049）；稅別不存在 404 MD.TAX_CODE.NOT_FOUND；銷項查進項專用稅別（或相反）422 MD.TAX_RATE.DIRECTION_MISMATCH；沒有稅率 422 MD.TAX_RATE.NOT_FOUND。</x:t>
         </x:is>
       </x:c>
       <x:c r="H180" s="2" t="inlineStr">
@@ -7649,7 +7649,7 @@
       </x:c>
       <x:c r="D181" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">1.0</x:t>
+          <x:t xml:space="preserve">1.1</x:t>
         </x:is>
       </x:c>
       <x:c r="E181" s="2" t="inlineStr">
@@ -7664,7 +7664,7 @@
       </x:c>
       <x:c r="G181" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Tax.Calculate 與 ITaxRateLookup.CalculateAsync、POST /api/v1/md/tax-rates/calculate（MD.TAX_CODE.VIEW）：未稅金額 → 未稅 = 取整（金額）、稅額 = 取整（未稅 × 稅率 ÷ 100）、含稅 = 未稅 + 稅額；含稅金額 → 含稅 = 取整（金額）、未稅 = 取整（含稅 × 100 ÷（100 + 稅率））、稅額 = 含稅 − 未稅。取整用 Money.Round 與 ICurrencyLookup.GetPrecisionAsync 的幣別小數位（AwayFromZero），負數對稱；幣別代碼格式錯誤 400 currencyCode。</x:t>
+          <x:t xml:space="preserve">Tax.Calculate 與 ITaxRateLookup.CalculateAsync、POST /api/v1/md/tax-rates/calculate（MD.TAX_CODE.VIEW）：未稅金額 → 未稅 = 取整（金額）、稅額 = 取整（未稅 × 稅率 ÷ 100）、含稅 = 未稅 + 稅額；含稅金額 → 含稅 = 取整（金額）、未稅 = 取整（含稅 × 100 ÷（100 + 稅率））、稅額 = 含稅 − 未稅。取整用 Money.Round 與該幣別在幣別主檔的小數位（AwayFromZero，停用幣別仍可用），負數對稱；幣別代碼格式錯誤 400 currencyCode，不在幣別主檔 404 MD.CURRENCY.NOT_FOUND（ADR-049）；停用稅別規則同 REQ_F4118.38.5。</x:t>
         </x:is>
       </x:c>
       <x:c r="H181" s="2" t="inlineStr">
@@ -12348,7 +12348,7 @@
       </x:c>
       <x:c r="E14" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">非待審客戶二次確認後按版本軟刪除；已被單據引用顯示錯誤。</x:t>
+          <x:t xml:space="preserve">二次確認後按版本軟刪除。待審（Pending）也顯示，因為前端無法分辨「從未送審」與「審批中」：審批中由後端回 422 MD.CUSTOMER.APPROVAL_PENDING 並顯示訊息；已被單據引用顯示錯誤；資料已被刪除（404）或版本衝突時重新查詢列表（MD-B02、MD-F06）。</x:t>
         </x:is>
       </x:c>
       <x:c r="F14" s="2" t="inlineStr">
@@ -12363,7 +12363,7 @@
       </x:c>
       <x:c r="H14" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">DELETE 權限且非 Pending</x:t>
+          <x:t xml:space="preserve">DELETE 權限</x:t>
         </x:is>
       </x:c>
       <x:c r="I14" s="2" t="inlineStr">
@@ -13374,7 +13374,7 @@
       </x:c>
       <x:c r="E32" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">選擇本機檔案；換檔清除舊預覽。</x:t>
+          <x:t xml:space="preserve">選擇本機檔案；換檔清除舊預覽。副檔名不是 xlsx／csv 或超過 2 MB 時在前端即拒絕，顯示 COMMON.IMPORT.UNSUPPORTED_FORMAT／TOO_LARGE，不上傳（MD-F09）。</x:t>
         </x:is>
       </x:c>
       <x:c r="F32" s="2" t="inlineStr">
@@ -13431,7 +13431,7 @@
       </x:c>
       <x:c r="E33" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">顯示實際列號、代碼、名稱、Create／Skip／Error 與欄位錯誤。</x:t>
+          <x:t xml:space="preserve">顯示實際列號、代碼、名稱、Create／Skip／Error 與欄位錯誤；欄位名以三語顯示（如「分類代碼: 找不到」），未知欄位原樣顯示（MD-F08）。</x:t>
         </x:is>
       </x:c>
       <x:c r="F33" s="2" t="inlineStr">
@@ -13716,7 +13716,7 @@
       </x:c>
       <x:c r="E38" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">非待審供應商二次確認後按版本軟刪除；已被單據引用顯示錯誤。</x:t>
+          <x:t xml:space="preserve">二次確認後按版本軟刪除。待審（Pending）也顯示，審批中由後端回 422 MD.SUPPLIER.APPROVAL_PENDING 並顯示訊息；已被單據引用顯示錯誤；資料已被刪除（404）或版本衝突時重新查詢列表（MD-B02、MD-F06）。</x:t>
         </x:is>
       </x:c>
       <x:c r="F38" s="2" t="inlineStr">
@@ -13731,7 +13731,7 @@
       </x:c>
       <x:c r="H38" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">DELETE 權限且非 Pending</x:t>
+          <x:t xml:space="preserve">DELETE 權限</x:t>
         </x:is>
       </x:c>
       <x:c r="I38" s="2" t="inlineStr">
@@ -29104,7 +29104,7 @@
       </x:c>
       <x:c r="F5" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MD-CUS-001, MD-CUS-002, MD-CUS-003</x:t>
+          <x:t xml:space="preserve">MD-CUS-001, MD-CUS-002, MD-CUS-003, MD-FE-REV-001, MD-FE-REV-002</x:t>
         </x:is>
       </x:c>
       <x:c r="G5" s="2" t="inlineStr">
@@ -29215,7 +29215,7 @@
       </x:c>
       <x:c r="F8" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MD-CUS-REV-001, MD-CUS-REV-002, MD-CUS-REV-003</x:t>
+          <x:t xml:space="preserve">MD-CUS-REV-001, MD-CUS-REV-002, MD-CUS-REV-003, MD-CUS-REV-004, MD-REAL-001</x:t>
         </x:is>
       </x:c>
       <x:c r="G8" s="2" t="inlineStr">
@@ -29289,7 +29289,7 @@
       </x:c>
       <x:c r="F10" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MD-CUS-REV-001, MD-CUS-REV-002, MD-CUS-REV-003</x:t>
+          <x:t xml:space="preserve">MD-CUS-REV-001, MD-CUS-REV-002, MD-CUS-REV-003, MD-CUS-REV-005, MD-REAL-001</x:t>
         </x:is>
       </x:c>
       <x:c r="G10" s="2" t="inlineStr">
@@ -29326,7 +29326,7 @@
       </x:c>
       <x:c r="F11" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MD-IMP-001, MD-IMP-002, MD-IMP-003, MD-IMP-004, MD-IMP-005</x:t>
+          <x:t xml:space="preserve">MD-IMP-001, MD-IMP-002, MD-IMP-003, MD-IMP-004, MD-IMP-005, MD-FE-REV-004</x:t>
         </x:is>
       </x:c>
       <x:c r="G11" s="2" t="inlineStr">
@@ -29363,7 +29363,7 @@
       </x:c>
       <x:c r="F12" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MD-PAY-DEF-001, MD-PAY-DEF-002</x:t>
+          <x:t xml:space="preserve">MD-PAY-DEF-001, MD-PAY-DEF-002, MD-REAL-001</x:t>
         </x:is>
       </x:c>
       <x:c r="G12" s="2" t="inlineStr">
@@ -29511,7 +29511,7 @@
       </x:c>
       <x:c r="F16" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MD-SUP-REV-001, MD-SUP-REV-002, MD-SUP-REV-003</x:t>
+          <x:t xml:space="preserve">MD-SUP-REV-001, MD-SUP-REV-002, MD-SUP-REV-003, MD-SUP-REV-004, MD-REAL-002</x:t>
         </x:is>
       </x:c>
       <x:c r="G16" s="2" t="inlineStr">
@@ -29585,7 +29585,7 @@
       </x:c>
       <x:c r="F18" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MD-SUP-REV-001, MD-SUP-REV-002, MD-SUP-REV-003</x:t>
+          <x:t xml:space="preserve">MD-SUP-REV-001, MD-SUP-REV-002, MD-SUP-REV-003, MD-CUS-REV-005, MD-REAL-002</x:t>
         </x:is>
       </x:c>
       <x:c r="G18" s="2" t="inlineStr">
@@ -29659,7 +29659,7 @@
       </x:c>
       <x:c r="F20" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MD-PAY-DEF-001, MD-PAY-DEF-002</x:t>
+          <x:t xml:space="preserve">MD-PAY-DEF-001, MD-PAY-DEF-002, MD-REAL-002</x:t>
         </x:is>
       </x:c>
       <x:c r="G20" s="2" t="inlineStr">
@@ -29696,7 +29696,7 @@
       </x:c>
       <x:c r="F21" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MD-ITEM-001, MD-ITEM-UI-001</x:t>
+          <x:t xml:space="preserve">MD-ITEM-001, MD-ITEM-UI-001, MD-FE-REV-002, MD-FE-REV-005</x:t>
         </x:is>
       </x:c>
       <x:c r="G21" s="2" t="inlineStr">
@@ -29733,7 +29733,7 @@
       </x:c>
       <x:c r="F22" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MD-ITEM-001, MD-ITEM-002, MD-ITEM-UI-001</x:t>
+          <x:t xml:space="preserve">MD-ITEM-001, MD-ITEM-002, MD-ITEM-003, MD-ITEM-UI-001</x:t>
         </x:is>
       </x:c>
       <x:c r="G22" s="2" t="inlineStr">
@@ -29770,7 +29770,7 @@
       </x:c>
       <x:c r="F23" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MD-ITEM-001, MD-ITEM-002, MD-ITEM-UI-001, MD-ITEM-CONV-002, MD-ITEM-CONV-UI-001</x:t>
+          <x:t xml:space="preserve">MD-ITEM-001, MD-ITEM-002, MD-ITEM-003, MD-ITEM-UI-001, MD-ITEM-CONV-002, MD-ITEM-CONV-UI-001, MD-USAGE-001</x:t>
         </x:is>
       </x:c>
       <x:c r="G23" s="2" t="inlineStr">
@@ -29844,7 +29844,7 @@
       </x:c>
       <x:c r="F25" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MD-ITEM-IMPORT-001, MD-ITEM-IMPORT-002, MD-ITEM-IMPORT-003, MD-ITEM-IMPORT-UI-001, MD-ITEM-IMPORT-UI-002</x:t>
+          <x:t xml:space="preserve">MD-ITEM-IMPORT-001, MD-ITEM-IMPORT-002, MD-ITEM-IMPORT-003, MD-ITEM-IMPORT-UI-001, MD-ITEM-IMPORT-UI-002, MD-FE-REV-004</x:t>
         </x:is>
       </x:c>
       <x:c r="G25" s="2" t="inlineStr">
@@ -29881,7 +29881,7 @@
       </x:c>
       <x:c r="F26" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MD-WH-001, MD-WH-002, MD-WH-UI-001, MD-WH-UI-002</x:t>
+          <x:t xml:space="preserve">MD-WH-001, MD-WH-002, MD-WH-UI-001, MD-WH-UI-002, MD-FE-REV-002</x:t>
         </x:is>
       </x:c>
       <x:c r="G26" s="2" t="inlineStr">
@@ -29992,7 +29992,7 @@
       </x:c>
       <x:c r="F29" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MD-WH-001, MD-WH-003, MD-WH-UI-001, MD-WH-UI-002</x:t>
+          <x:t xml:space="preserve">MD-WH-001, MD-WH-003, MD-WH-UI-001, MD-WH-UI-002, MD-USAGE-002</x:t>
         </x:is>
       </x:c>
       <x:c r="G29" s="2" t="inlineStr">
@@ -30029,7 +30029,7 @@
       </x:c>
       <x:c r="F30" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MD-WH-003, MD-WH-004, MD-WH-UI-001, MD-WH-UI-002</x:t>
+          <x:t xml:space="preserve">MD-WH-003, MD-WH-004, MD-WH-UI-001, MD-WH-UI-002, MD-USAGE-003</x:t>
         </x:is>
       </x:c>
       <x:c r="G30" s="2" t="inlineStr">
@@ -30732,7 +30732,7 @@
       </x:c>
       <x:c r="F49" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MD-ICAT-001, MD-ICAT-004, MD-ICAT-005, MD-ICAT-006</x:t>
+          <x:t xml:space="preserve">MD-ICAT-001, MD-ICAT-004, MD-ICAT-005, MD-ICAT-006, MD-FE-REV-001</x:t>
         </x:is>
       </x:c>
       <x:c r="G49" s="2" t="inlineStr">
@@ -35394,7 +35394,7 @@
       </x:c>
       <x:c r="F175" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MD-TAX-001, MD-TAX-UI-001, MD-TAX-UI-002</x:t>
+          <x:t xml:space="preserve">MD-TAX-001, MD-USAGE-004, MD-TAX-UI-001, MD-TAX-UI-002</x:t>
         </x:is>
       </x:c>
       <x:c r="G175" s="2" t="inlineStr">
@@ -35505,7 +35505,7 @@
       </x:c>
       <x:c r="F178" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MD-TAX-003, MD-TAX-UI-001, MD-TAX-UI-002</x:t>
+          <x:t xml:space="preserve">MD-TAX-003, MD-USAGE-004, MD-TAX-UI-001, MD-TAX-UI-002</x:t>
         </x:is>
       </x:c>
       <x:c r="G178" s="2" t="inlineStr">
@@ -35542,7 +35542,7 @@
       </x:c>
       <x:c r="F179" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MD-TAX-001, MD-TAX-UI-001, MD-TAX-UI-002</x:t>
+          <x:t xml:space="preserve">MD-TAX-001, MD-USAGE-004, MD-TAX-UI-001, MD-TAX-UI-002</x:t>
         </x:is>
       </x:c>
       <x:c r="G179" s="2" t="inlineStr">
@@ -35616,7 +35616,7 @@
       </x:c>
       <x:c r="F181" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MD-TAX-CALC-001, MD-TAX-002, MD-TAX-005, MD-TAX-UI-001, MD-TAX-UI-002</x:t>
+          <x:t xml:space="preserve">MD-TAX-CALC-001, MD-TAX-002, MD-TAX-005, MD-TAX-UI-001, MD-TAX-UI-002, MD-FE-REV-005</x:t>
         </x:is>
       </x:c>
       <x:c r="G181" s="2" t="inlineStr">
@@ -36023,7 +36023,7 @@
       </x:c>
       <x:c r="F192" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MD-CONT-001, MD-CONT-UI-001, MD-CONT-UI-002</x:t>
+          <x:t xml:space="preserve">MD-CONT-001, MD-CONT-UI-001, MD-CONT-UI-002, MD-FE-REV-003</x:t>
         </x:is>
       </x:c>
       <x:c r="G192" s="2" t="inlineStr">
@@ -36578,7 +36578,7 @@
       </x:c>
       <x:c r="F207" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MD-IMG-001, MD-IMG-003, MD-IMG-UI-004</x:t>
+          <x:t xml:space="preserve">MD-IMG-001, MD-IMG-003, MD-IMG-005, MD-IMG-UI-004</x:t>
         </x:is>
       </x:c>
       <x:c r="G207" s="2" t="inlineStr">
@@ -42164,7 +42164,7 @@
       </x:c>
       <x:c r="F167" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">未開始</x:t>
+          <x:t xml:space="preserve">未開始（WU-MD-028，022e 回歸時發現缺口）</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -47274,17 +47274,17 @@
       </x:c>
       <x:c r="D327" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MD</x:t>
+          <x:t xml:space="preserve">INV</x:t>
         </x:is>
       </x:c>
       <x:c r="E327" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.8.14</x:t>
+          <x:t xml:space="preserve">待 EP-INV 分配</x:t>
         </x:is>
       </x:c>
       <x:c r="F327" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">未開始</x:t>
+          <x:t xml:space="preserve">未開始（期初庫存寫庫存異動帳，已自 EP-MD 移入 EP-INV）</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
feat(inv): add other receipt pages and exports
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R1b10391ed86642dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R50d6b71eb38c47ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Rb5d07d6e1d664087"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Rb060d8b2417e4fcd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R71185c0bc2f1487f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="Rfa31f01a902f4aea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Re21d6dba926548fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="Rb92277f4c72a45ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R1d6149d1b5d148b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R914f63c498ee4f2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R9c0617fbea854c4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R8fc41a63cf4943f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Rf9429afba7a34a13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R95ac6b7f97b4456d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R643efb879c564648"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R76a284cbd22147a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R7b27b38e289e49b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Ra4596200b7bc4f2d"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
feat(inv): add other issue frontend and coverage
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R76fb72e363e54f55"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R5480417bc84544aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Rc0ace4405de944e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R473a8963a6cd48b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R85108cca5a8145f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="Rddf4c4b8489f41a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R489198f8c76b46ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R6a854f05116b4889"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rb80f37f034764331"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Rc808ecec96dd4af7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Rfe1361f14a8c4049"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R4986bbf817a5410a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Re1ad2dad6df34662"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Rb9143564a9e749e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R87dc6e258a1845e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R993f909a43b54a07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R552991ee660f4534"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R27aa90976f774226"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -32006,7 +32006,7 @@
       </x:c>
       <x:c r="F12" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">INV-ISS-001, INV-ISS-004</x:t>
+          <x:t xml:space="preserve">INV-ISS-001, INV-ISS-005, INV-ISS-004</x:t>
         </x:is>
       </x:c>
       <x:c r="G12" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat(inv): add trilingual inventory transfer pages
- /inv/transfers list with keyword/date/status filters, server paging,
  draft submit/delete, print and formula-safe CSV export
- create/edit form with source and destination warehouse/location,
  same-balance-key guard, optional lot/serial capture for drafts
- menu entry, INV.TRANSFER.* permissions, i18n keys and error codes
- fix OnPush redraw race when edit detail arrives after MD options
  in other receipt/issue forms
- Vitest and Playwright INV-TRF-009; closes WU-INV-009

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R2e5fff14d6e54860"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Rea3de87e0cde4abf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R80a590e0136e4333"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Rd4a8221cf9ee4f06"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Rd81e9bd32a984b1c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="Rf83bd3dcfd444cbb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R5e993d2329cf4630"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R6558e6e8d40c4e02"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rfb7e79b04b454160"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R1d7e955cc8a2496e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Rc101d2e096374667"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R58baec637fde4301"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R2f0b7b4c580c4da1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Rf549bdb6058243a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R0b7ca8e27c2c4e68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Rc42314134cc74a2b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R672888688ef544cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R01ce1c8e23db44cd"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
feat(inv): add stocktake submit, variance posting and report
WU-INV-010a2 (closes WU-INV-010a): POST /stocktakes/{id}/submit with
INV.STOCKTAKE.SUBMIT checks draft+version, every line and lot/serial
counted (COUNT_MISSING), recomputes scope balances including added-line
keys and movements after the snapshot (SNAPSHOT_STALE with up to 50
changedKeys in ProblemDetails), and pre-checks the posting limits
(TOO_MANY_LINES) before the SYS workflow. StocktakeApprovalResultHandler
posts per-line gains as In and losses as Out (split by lot/serial,
source STOCKTAKE, no cost), rolls back on shortages and marks Posted or
Rejected. GET /stocktakes/{id}/variance returns Gain/Loss/Match/
Uncounted lines, totals and differenceOnly. ErpException.Extensions now
flow into ProblemDetails without overriding errorCode/errors.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R9a5bae83119d468e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Rb8462e9676a646ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Rb35a284446fe476a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Rc8f38f9afc464adc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Rf7c09c7a0cee41f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="Rdde405569f12438b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Rd581db2a87f84b8c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R6350656d52504bba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Ra2e589faebe34652"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Rbbe10b799b594105"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R8f5db828b0f24f96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Rbb52669d493d41e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R1bba9801874d4aee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R5d4bfa7a584843b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R1afba08147c74551"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R88e45f285da44f23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R34ed38995c2f4a7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rd1135bc5bed54a08"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
feat(inv): add stocktake counting flow
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Rbbe10b799b594105"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R8f5db828b0f24f96"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Rbb52669d493d41e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R1bba9801874d4aee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R5d4bfa7a584843b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R1afba08147c74551"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R88e45f285da44f23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R34ed38995c2f4a7d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rd1135bc5bed54a08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R32fb85148db44b6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R25daf946cf2b42c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R41fb75624c6345b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R31d31cf5ed134301"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R09bd73ead9994e86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R739675d75f684a62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R52f92848defd4f47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R603528ce817d4c70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Radd8f5ad66934f93"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19039,7 +19039,7 @@
       </x:c>
       <x:c r="E87" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Select labelled "Item" opening the item selection modal.</x:t>
+          <x:t xml:space="preserve">Scrollable multi-select checklist labelled "Items".</x:t>
         </x:is>
       </x:c>
       <x:c r="F87" s="2" t="inlineStr">
@@ -19210,7 +19210,7 @@
       </x:c>
       <x:c r="E90" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Input labelled "Remarks" under the stocktake table.</x:t>
+          <x:t xml:space="preserve">Input labelled "Remarks" in the stocktake header.</x:t>
         </x:is>
       </x:c>
       <x:c r="F90" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat(inv): complete stocktake report and list
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R32fb85148db44b6b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R25daf946cf2b42c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R41fb75624c6345b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R31d31cf5ed134301"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R09bd73ead9994e86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R739675d75f684a62"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R52f92848defd4f47"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R603528ce817d4c70"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Radd8f5ad66934f93"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Ra1eba1c03def4ce1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R2364a9fd138c40dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R0f98d6331bf14840"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Re968646a7fb147f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R4c17e7e7d2194e9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R47f92e8a81944893"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R60a70da91e3d4436"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R0e05d9e3aa5a4c3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R19de8b61722d4678"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19609,7 +19609,7 @@
       </x:c>
       <x:c r="E97" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Show paged company stocktakes, line and counted counts and approval state.</x:t>
+          <x:t xml:space="preserve">Show paged company stocktakes with line and counted counts; open detail to inspect approval state.</x:t>
         </x:is>
       </x:c>
       <x:c r="F97" s="2" t="inlineStr">
@@ -19624,7 +19624,7 @@
       </x:c>
       <x:c r="H97" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">VIEW</x:t>
+          <x:t xml:space="preserve">VIEW; server paging</x:t>
         </x:is>
       </x:c>
       <x:c r="I97" s="2" t="inlineStr">
@@ -19666,7 +19666,7 @@
       </x:c>
       <x:c r="E98" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Show book, counted, difference and type per line with gain and loss totals.</x:t>
+          <x:t xml:space="preserve">Show MD item, warehouse and location names, book, counted, net difference, gain/loss quantities and type per line, plus each lot or serial and full-document totals.</x:t>
         </x:is>
       </x:c>
       <x:c r="F98" s="2" t="inlineStr">
@@ -19681,7 +19681,7 @@
       </x:c>
       <x:c r="H98" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">VIEW; difference-only toggle</x:t>
+          <x:t xml:space="preserve">VIEW; difference-only toggle (gain/loss at tracking granularity)</x:t>
         </x:is>
       </x:c>
       <x:c r="I98" s="2" t="inlineStr">
@@ -19780,7 +19780,7 @@
       </x:c>
       <x:c r="E100" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Print the gain and loss report or export it to safe UTF-8 CSV.</x:t>
+          <x:t xml:space="preserve">Print the gain and loss report or fetch every page under current filters for UTF-8 CSV with spreadsheet formula neutralization.</x:t>
         </x:is>
       </x:c>
       <x:c r="F100" s="2" t="inlineStr">
@@ -37840,7 +37840,7 @@
       </x:c>
       <x:c r="F31" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">INV-STK-007</x:t>
+          <x:t xml:space="preserve">INV-STK-007, INV-STK-011</x:t>
         </x:is>
       </x:c>
       <x:c r="G31" s="2" t="inlineStr">

</xml_diff>

<commit_message>
fix(inv): reserve baseline interface numbers and renumber extensions
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Ra1eba1c03def4ce1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R2364a9fd138c40dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R0f98d6331bf14840"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Re968646a7fb147f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R4c17e7e7d2194e9b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R47f92e8a81944893"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R60a70da91e3d4436"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R0e05d9e3aa5a4c3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R19de8b61722d4678"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R93323bbc53b64a87"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Rc380c7bbc34143fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Rc7252465333347c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R6b11255eb4f94070"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R793823d680634f89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R80afc429a1a4467e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Rc2397dc065994687"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="Rce437d0eb47b41ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Refaa3c40998f44f8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17024,32 +17024,32 @@
     <x:row r="52">
       <x:c r="A52" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.8.1</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.15.1</x:t>
         </x:is>
       </x:c>
       <x:c r="B52" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.8</x:t>
+          <x:t xml:space="preserve">4.4.1.5.15</x:t>
         </x:is>
       </x:c>
       <x:c r="C52" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Product Initial Stock View Interface</x:t>
+          <x:t xml:space="preserve">Inventory Transfer Create Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D52" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Opening Date Range (Date Picker)</x:t>
+          <x:t xml:space="preserve">Business Date (Date Picker)</x:t>
         </x:is>
       </x:c>
       <x:c r="E52" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Filter batches by opening date inclusively.</x:t>
+          <x:t xml:space="preserve">Set transfer business date.</x:t>
         </x:is>
       </x:c>
       <x:c r="F52" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Narrow results.</x:t>
+          <x:t xml:space="preserve">Date both movements.</x:t>
         </x:is>
       </x:c>
       <x:c r="G52" s="2" t="inlineStr">
@@ -17059,7 +17059,7 @@
       </x:c>
       <x:c r="H52" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">From ≤ To</x:t>
+          <x:t xml:space="preserve">Valid business date</x:t>
         </x:is>
       </x:c>
       <x:c r="I52" s="2" t="inlineStr">
@@ -17081,42 +17081,42 @@
     <x:row r="53">
       <x:c r="A53" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.8.2</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.15.2</x:t>
         </x:is>
       </x:c>
       <x:c r="B53" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.8</x:t>
+          <x:t xml:space="preserve">4.4.1.5.15</x:t>
         </x:is>
       </x:c>
       <x:c r="C53" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Product Initial Stock View Interface</x:t>
+          <x:t xml:space="preserve">Inventory Transfer Create Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D53" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Item / Warehouse (Dropdown)</x:t>
+          <x:t xml:space="preserve">Item (Dropdown)</x:t>
         </x:is>
       </x:c>
       <x:c r="E53" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Filter batches containing the MD item or warehouse.</x:t>
+          <x:t xml:space="preserve">Select an active company item per line.</x:t>
         </x:is>
       </x:c>
       <x:c r="F53" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Narrow results.</x:t>
+          <x:t xml:space="preserve">Identify stock.</x:t>
         </x:is>
       </x:c>
       <x:c r="G53" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">ID</x:t>
+          <x:t xml:space="preserve">MD ID</x:t>
         </x:is>
       </x:c>
       <x:c r="H53" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Current company</x:t>
+          <x:t xml:space="preserve">Active item</x:t>
         </x:is>
       </x:c>
       <x:c r="I53" s="2" t="inlineStr">
@@ -17138,47 +17138,47 @@
     <x:row r="54">
       <x:c r="A54" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.8.3</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.15.3</x:t>
         </x:is>
       </x:c>
       <x:c r="B54" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.8</x:t>
+          <x:t xml:space="preserve">4.4.1.5.15</x:t>
         </x:is>
       </x:c>
       <x:c r="C54" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Product Initial Stock View Interface</x:t>
+          <x:t xml:space="preserve">Inventory Transfer Create Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D54" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Keyword (Textbox)</x:t>
+          <x:t xml:space="preserve">Source Warehouse / Location (Dropdown)</x:t>
         </x:is>
       </x:c>
       <x:c r="E54" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Match remark or request key.</x:t>
+          <x:t xml:space="preserve">Select the issuing warehouse and optional bin.</x:t>
         </x:is>
       </x:c>
       <x:c r="F54" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Find a batch.</x:t>
+          <x:t xml:space="preserve">Set source balance key.</x:t>
         </x:is>
       </x:c>
       <x:c r="G54" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Text</x:t>
+          <x:t xml:space="preserve">MD IDs</x:t>
         </x:is>
       </x:c>
       <x:c r="H54" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Partial match</x:t>
+          <x:t xml:space="preserve">Current company, active</x:t>
         </x:is>
       </x:c>
       <x:c r="I54" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">None</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.15.2</x:t>
         </x:is>
       </x:c>
       <x:c r="J54" s="2" t="inlineStr">
@@ -17195,47 +17195,47 @@
     <x:row r="55">
       <x:c r="A55" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.8.4</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.15.4</x:t>
         </x:is>
       </x:c>
       <x:c r="B55" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.8</x:t>
+          <x:t xml:space="preserve">4.4.1.5.15</x:t>
         </x:is>
       </x:c>
       <x:c r="C55" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Product Initial Stock View Interface</x:t>
+          <x:t xml:space="preserve">Inventory Transfer Create Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D55" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Batch List (Table)</x:t>
+          <x:t xml:space="preserve">Destination Warehouse / Location (Dropdown)</x:t>
         </x:is>
       </x:c>
       <x:c r="E55" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Paged batches with lines, quantity, amount, remark and posted time.</x:t>
+          <x:t xml:space="preserve">Select a different receiving balance key.</x:t>
         </x:is>
       </x:c>
       <x:c r="F55" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Review opening stock.</x:t>
+          <x:t xml:space="preserve">Set destination.</x:t>
         </x:is>
       </x:c>
       <x:c r="G55" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Table</x:t>
+          <x:t xml:space="preserve">MD IDs</x:t>
         </x:is>
       </x:c>
       <x:c r="H55" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Authorized company</x:t>
+          <x:t xml:space="preserve">Different key, active</x:t>
         </x:is>
       </x:c>
       <x:c r="I55" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.8.1</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.15.3</x:t>
         </x:is>
       </x:c>
       <x:c r="J55" s="2" t="inlineStr">
@@ -17252,47 +17252,47 @@
     <x:row r="56">
       <x:c r="A56" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.8.5</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.15.5</x:t>
         </x:is>
       </x:c>
       <x:c r="B56" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.8</x:t>
+          <x:t xml:space="preserve">4.4.1.5.15</x:t>
         </x:is>
       </x:c>
       <x:c r="C56" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Product Initial Stock View Interface</x:t>
+          <x:t xml:space="preserve">Inventory Transfer Create Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D56" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Batch Detail (Panel)</x:t>
+          <x:t xml:space="preserve">Quantity / Tracking (Input)</x:t>
         </x:is>
       </x:c>
       <x:c r="E56" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Lines by line number with MD names, quantity, unit cost and amount.</x:t>
+          <x:t xml:space="preserve">Enter six-decimal base quantity and source lot or serial numbers.</x:t>
         </x:is>
       </x:c>
       <x:c r="F56" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Inspect a batch.</x:t>
+          <x:t xml:space="preserve">Transfer exact tracked units.</x:t>
         </x:is>
       </x:c>
       <x:c r="G56" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Table</x:t>
+          <x:t xml:space="preserve">Decimal(19,6) / text</x:t>
         </x:is>
       </x:c>
       <x:c r="H56" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Authorized company</x:t>
+          <x:t xml:space="preserve">Positive; tracking total equals quantity</x:t>
         </x:is>
       </x:c>
       <x:c r="I56" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.8.4</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.15.2</x:t>
         </x:is>
       </x:c>
       <x:c r="J56" s="2" t="inlineStr">
@@ -17309,32 +17309,32 @@
     <x:row r="57">
       <x:c r="A57" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.8.6</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.15.6</x:t>
         </x:is>
       </x:c>
       <x:c r="B57" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.8</x:t>
+          <x:t xml:space="preserve">4.4.1.5.15</x:t>
         </x:is>
       </x:c>
       <x:c r="C57" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Product Initial Stock View Interface</x:t>
+          <x:t xml:space="preserve">Inventory Transfer Create Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D57" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Print / Export (Button)</x:t>
+          <x:t xml:space="preserve">Save Draft (Button)</x:t>
         </x:is>
       </x:c>
       <x:c r="E57" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Print one batch; export filtered batches as formula-safe UTF-8 CSV.</x:t>
+          <x:t xml:space="preserve">Validate and save without changing stock.</x:t>
         </x:is>
       </x:c>
       <x:c r="F57" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Keep records.</x:t>
+          <x:t xml:space="preserve">Prepare approval.</x:t>
         </x:is>
       </x:c>
       <x:c r="G57" s="2" t="inlineStr">
@@ -17344,12 +17344,12 @@
       </x:c>
       <x:c r="H57" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Authorized</x:t>
+          <x:t xml:space="preserve">CREATE</x:t>
         </x:is>
       </x:c>
       <x:c r="I57" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.8.4</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.15.1</x:t>
         </x:is>
       </x:c>
       <x:c r="J57" s="2" t="inlineStr">
@@ -17366,42 +17366,42 @@
     <x:row r="58">
       <x:c r="A58" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.9.1</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.16.1</x:t>
         </x:is>
       </x:c>
       <x:c r="B58" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.9</x:t>
+          <x:t xml:space="preserve">4.4.1.5.16</x:t>
         </x:is>
       </x:c>
       <x:c r="C58" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Product Initial Stock Create Interface</x:t>
+          <x:t xml:space="preserve">Inventory Transfer View Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D58" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Opening Date (Date Picker)</x:t>
+          <x:t xml:space="preserve">Filters (Input)</x:t>
         </x:is>
       </x:c>
       <x:c r="E58" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Date the opening balance takes effect.</x:t>
+          <x:t xml:space="preserve">Filter by document number, date and status.</x:t>
         </x:is>
       </x:c>
       <x:c r="F58" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Set start of stock history.</x:t>
+          <x:t xml:space="preserve">Find transfers.</x:t>
         </x:is>
       </x:c>
       <x:c r="G58" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Date</x:t>
+          <x:t xml:space="preserve">Text / date / status</x:t>
         </x:is>
       </x:c>
       <x:c r="H58" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">≤ today; ≤ earliest movement</x:t>
+          <x:t xml:space="preserve">From ≤ To</x:t>
         </x:is>
       </x:c>
       <x:c r="I58" s="2" t="inlineStr">
@@ -17423,47 +17423,47 @@
     <x:row r="59">
       <x:c r="A59" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.9.2</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.16.2</x:t>
         </x:is>
       </x:c>
       <x:c r="B59" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.9</x:t>
+          <x:t xml:space="preserve">4.4.1.5.16</x:t>
         </x:is>
       </x:c>
       <x:c r="C59" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Product Initial Stock Create Interface</x:t>
+          <x:t xml:space="preserve">Inventory Transfer View Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D59" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Item / Warehouse / Location (Dropdown)</x:t>
+          <x:t xml:space="preserve">Transfer List (Table)</x:t>
         </x:is>
       </x:c>
       <x:c r="E59" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Active MD references per line; location limited to the warehouse.</x:t>
+          <x:t xml:space="preserve">Show paged company transfers, quantity and approval state.</x:t>
         </x:is>
       </x:c>
       <x:c r="F59" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Identify balance key.</x:t>
+          <x:t xml:space="preserve">Review records.</x:t>
         </x:is>
       </x:c>
       <x:c r="G59" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">ID</x:t>
+          <x:t xml:space="preserve">Table</x:t>
         </x:is>
       </x:c>
       <x:c r="H59" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Active, current company</x:t>
+          <x:t xml:space="preserve">VIEW</x:t>
         </x:is>
       </x:c>
       <x:c r="I59" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.9.1</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.16.1</x:t>
         </x:is>
       </x:c>
       <x:c r="J59" s="2" t="inlineStr">
@@ -17480,47 +17480,47 @@
     <x:row r="60">
       <x:c r="A60" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.9.3</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.16.3</x:t>
         </x:is>
       </x:c>
       <x:c r="B60" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.9</x:t>
+          <x:t xml:space="preserve">4.4.1.5.16</x:t>
         </x:is>
       </x:c>
       <x:c r="C60" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Product Initial Stock Create Interface</x:t>
+          <x:t xml:space="preserve">Inventory Transfer View Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D60" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Quantity / Unit Cost (Textbox)</x:t>
+          <x:t xml:space="preserve">Detail (Panel)</x:t>
         </x:is>
       </x:c>
       <x:c r="E60" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Base-unit quantity and unit cost.</x:t>
+          <x:t xml:space="preserve">Show stored lines, both locations, tracking and approval.</x:t>
         </x:is>
       </x:c>
       <x:c r="F60" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Value opening stock.</x:t>
+          <x:t xml:space="preserve">Inspect movement pair.</x:t>
         </x:is>
       </x:c>
       <x:c r="G60" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Decimal(6)</x:t>
+          <x:t xml:space="preserve">Panel</x:t>
         </x:is>
       </x:c>
       <x:c r="H60" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Quantity &gt; 0; cost ≥ 0</x:t>
+          <x:t xml:space="preserve">VIEW</x:t>
         </x:is>
       </x:c>
       <x:c r="I60" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.9.2</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.16.2</x:t>
         </x:is>
       </x:c>
       <x:c r="J60" s="2" t="inlineStr">
@@ -17537,32 +17537,32 @@
     <x:row r="61">
       <x:c r="A61" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.9.4</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.16.4</x:t>
         </x:is>
       </x:c>
       <x:c r="B61" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.9</x:t>
+          <x:t xml:space="preserve">4.4.1.5.16</x:t>
         </x:is>
       </x:c>
       <x:c r="C61" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Product Initial Stock Create Interface</x:t>
+          <x:t xml:space="preserve">Inventory Transfer View Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D61" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Preview (Button)</x:t>
+          <x:t xml:space="preserve">Submit / Delete (Button)</x:t>
         </x:is>
       </x:c>
       <x:c r="E61" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Validate without saving; show per-line trilingual errors and totals.</x:t>
+          <x:t xml:space="preserve">Submit a draft or delete a draft with confirmation.</x:t>
         </x:is>
       </x:c>
       <x:c r="F61" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Catch errors before posting.</x:t>
+          <x:t xml:space="preserve">Control lifecycle.</x:t>
         </x:is>
       </x:c>
       <x:c r="G61" s="2" t="inlineStr">
@@ -17572,12 +17572,12 @@
       </x:c>
       <x:c r="H61" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">CREATE</x:t>
+          <x:t xml:space="preserve">SUBMIT / DELETE</x:t>
         </x:is>
       </x:c>
       <x:c r="I61" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.9.1</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.16.2</x:t>
         </x:is>
       </x:c>
       <x:c r="J61" s="2" t="inlineStr">
@@ -17594,32 +17594,32 @@
     <x:row r="62">
       <x:c r="A62" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.9.5</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.16.5</x:t>
         </x:is>
       </x:c>
       <x:c r="B62" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.9</x:t>
+          <x:t xml:space="preserve">4.4.1.5.16</x:t>
         </x:is>
       </x:c>
       <x:c r="C62" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Product Initial Stock Create Interface</x:t>
+          <x:t xml:space="preserve">Inventory Transfer View Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D62" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Submit (Button)</x:t>
+          <x:t xml:space="preserve">Print / Export (Button)</x:t>
         </x:is>
       </x:c>
       <x:c r="E62" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Post a clean, unchanged preview once; retry reuses the batch request key.</x:t>
+          <x:t xml:space="preserve">Print detail or export filtered records to safe UTF-8 CSV.</x:t>
         </x:is>
       </x:c>
       <x:c r="F62" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Post opening stock idempotently.</x:t>
+          <x:t xml:space="preserve">Keep transfer records.</x:t>
         </x:is>
       </x:c>
       <x:c r="G62" s="2" t="inlineStr">
@@ -17629,12 +17629,12 @@
       </x:c>
       <x:c r="H62" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Clean preview</x:t>
+          <x:t xml:space="preserve">VIEW</x:t>
         </x:is>
       </x:c>
       <x:c r="I62" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.9.4</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.16.2</x:t>
         </x:is>
       </x:c>
       <x:c r="J62" s="2" t="inlineStr">
@@ -17651,42 +17651,42 @@
     <x:row r="63">
       <x:c r="A63" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.9.6</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.17.1</x:t>
         </x:is>
       </x:c>
       <x:c r="B63" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.9</x:t>
+          <x:t xml:space="preserve">4.4.1.5.17</x:t>
         </x:is>
       </x:c>
       <x:c r="C63" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Product Initial Stock Create Interface</x:t>
+          <x:t xml:space="preserve">Inventory Transfer Edit Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D63" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Lot or Serial (Input)</x:t>
+          <x:t xml:space="preserve">Business Date / Remark (Input)</x:t>
         </x:is>
       </x:c>
       <x:c r="E63" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Capture opening stock tracking entries.</x:t>
+          <x:t xml:space="preserve">Revise a draft or rejected transfer.</x:t>
         </x:is>
       </x:c>
       <x:c r="F63" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Establish tracked opening stock.</x:t>
+          <x:t xml:space="preserve">Correct header.</x:t>
         </x:is>
       </x:c>
       <x:c r="G63" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Lot rows or serial lines</x:t>
+          <x:t xml:space="preserve">Date / text</x:t>
         </x:is>
       </x:c>
       <x:c r="H63" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Sum equals line quantity</x:t>
+          <x:t xml:space="preserve">Editable status</x:t>
         </x:is>
       </x:c>
       <x:c r="I63" s="2" t="inlineStr">
@@ -17708,47 +17708,47 @@
     <x:row r="64">
       <x:c r="A64" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.10.1</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.17.2</x:t>
         </x:is>
       </x:c>
       <x:c r="B64" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.10</x:t>
+          <x:t xml:space="preserve">4.4.1.5.17</x:t>
         </x:is>
       </x:c>
       <x:c r="C64" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Lot and Serial Trace Interface</x:t>
+          <x:t xml:space="preserve">Inventory Transfer Edit Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D64" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Tracking Type (Button)</x:t>
+          <x:t xml:space="preserve">Source / Destination (Dropdown)</x:t>
         </x:is>
       </x:c>
       <x:c r="E64" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Switch between lot and serial lists.</x:t>
+          <x:t xml:space="preserve">Revise both balance keys per line.</x:t>
         </x:is>
       </x:c>
       <x:c r="F64" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Select tracking type.</x:t>
+          <x:t xml:space="preserve">Correct route.</x:t>
         </x:is>
       </x:c>
       <x:c r="G64" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Button</x:t>
+          <x:t xml:space="preserve">MD IDs</x:t>
         </x:is>
       </x:c>
       <x:c r="H64" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Lot / Serial</x:t>
+          <x:t xml:space="preserve">Different active keys</x:t>
         </x:is>
       </x:c>
       <x:c r="I64" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">None</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.17.1</x:t>
         </x:is>
       </x:c>
       <x:c r="J64" s="2" t="inlineStr">
@@ -17765,47 +17765,47 @@
     <x:row r="65">
       <x:c r="A65" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.10.2</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.17.3</x:t>
         </x:is>
       </x:c>
       <x:c r="B65" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.10</x:t>
+          <x:t xml:space="preserve">4.4.1.5.17</x:t>
         </x:is>
       </x:c>
       <x:c r="C65" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Lot and Serial Trace Interface</x:t>
+          <x:t xml:space="preserve">Inventory Transfer Edit Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D65" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Item (Dropdown)</x:t>
+          <x:t xml:space="preserve">Quantity / Tracking (Input)</x:t>
         </x:is>
       </x:c>
       <x:c r="E65" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Filter by company item.</x:t>
+          <x:t xml:space="preserve">Revise quantity and matching lot or serial list.</x:t>
         </x:is>
       </x:c>
       <x:c r="F65" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Narrow trace results.</x:t>
+          <x:t xml:space="preserve">Correct moved units.</x:t>
         </x:is>
       </x:c>
       <x:c r="G65" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">ID</x:t>
+          <x:t xml:space="preserve">Decimal(19,6) / text</x:t>
         </x:is>
       </x:c>
       <x:c r="H65" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Current company</x:t>
+          <x:t xml:space="preserve">Tracking total equals quantity at submit</x:t>
         </x:is>
       </x:c>
       <x:c r="I65" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">None</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.17.2</x:t>
         </x:is>
       </x:c>
       <x:c r="J65" s="2" t="inlineStr">
@@ -17822,47 +17822,47 @@
     <x:row r="66">
       <x:c r="A66" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.10.3</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.17.4</x:t>
         </x:is>
       </x:c>
       <x:c r="B66" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.10</x:t>
+          <x:t xml:space="preserve">4.4.1.5.17</x:t>
         </x:is>
       </x:c>
       <x:c r="C66" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Lot and Serial Trace Interface</x:t>
+          <x:t xml:space="preserve">Inventory Transfer Edit Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D66" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Number Search (Input)</x:t>
+          <x:t xml:space="preserve">Save Revision (Button)</x:t>
         </x:is>
       </x:c>
       <x:c r="E66" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Filter lot or serial number.</x:t>
+          <x:t xml:space="preserve">Replace draft lines with version check.</x:t>
         </x:is>
       </x:c>
       <x:c r="F66" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Find tracking number.</x:t>
+          <x:t xml:space="preserve">Persist correction.</x:t>
         </x:is>
       </x:c>
       <x:c r="G66" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Text</x:t>
+          <x:t xml:space="preserve">Button</x:t>
         </x:is>
       </x:c>
       <x:c r="H66" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Up to 100 characters</x:t>
+          <x:t xml:space="preserve">EDIT</x:t>
         </x:is>
       </x:c>
       <x:c r="I66" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">None</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.17.1</x:t>
         </x:is>
       </x:c>
       <x:c r="J66" s="2" t="inlineStr">
@@ -17879,42 +17879,42 @@
     <x:row r="67">
       <x:c r="A67" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.10.4</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.18.1</x:t>
         </x:is>
       </x:c>
       <x:c r="B67" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.10</x:t>
+          <x:t xml:space="preserve">4.4.1.5.18</x:t>
         </x:is>
       </x:c>
       <x:c r="C67" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Lot and Serial Trace Interface</x:t>
+          <x:t xml:space="preserve">Stocktake Create Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D67" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">In Stock Only (Checkbox)</x:t>
+          <x:t xml:space="preserve">Warehouse (Select)</x:t>
         </x:is>
       </x:c>
       <x:c r="E67" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Exclude fully issued numbers.</x:t>
+          <x:t xml:space="preserve">Select labelled "Select Warehouse".</x:t>
         </x:is>
       </x:c>
       <x:c r="F67" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Show current stock.</x:t>
+          <x:t xml:space="preserve">Choose one or more warehouses to count.</x:t>
         </x:is>
       </x:c>
       <x:c r="G67" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Boolean</x:t>
+          <x:t xml:space="preserve">MD IDs</x:t>
         </x:is>
       </x:c>
       <x:c r="H67" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">True / false</x:t>
+          <x:t xml:space="preserve">1–20 active company warehouses</x:t>
         </x:is>
       </x:c>
       <x:c r="I67" s="2" t="inlineStr">
@@ -17936,47 +17936,47 @@
     <x:row r="68">
       <x:c r="A68" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.10.5</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.18.2</x:t>
         </x:is>
       </x:c>
       <x:c r="B68" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.10</x:t>
+          <x:t xml:space="preserve">4.4.1.5.18</x:t>
         </x:is>
       </x:c>
       <x:c r="C68" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Lot and Serial Trace Interface</x:t>
+          <x:t xml:space="preserve">Stocktake Create Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D68" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Tracking Results (Table)</x:t>
+          <x:t xml:space="preserve">Category (Select)</x:t>
         </x:is>
       </x:c>
       <x:c r="E68" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Show paged lot or serial records.</x:t>
+          <x:t xml:space="preserve">Select labelled "Category".</x:t>
         </x:is>
       </x:c>
       <x:c r="F68" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Inspect on-hand status.</x:t>
+          <x:t xml:space="preserve">Limit the count to item categories and their children.</x:t>
         </x:is>
       </x:c>
       <x:c r="G68" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Table</x:t>
+          <x:t xml:space="preserve">MD IDs</x:t>
         </x:is>
       </x:c>
       <x:c r="H68" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Current company</x:t>
+          <x:t xml:space="preserve">0–50 categories</x:t>
         </x:is>
       </x:c>
       <x:c r="I68" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.10.1</x:t>
+          <x:t xml:space="preserve">None</x:t>
         </x:is>
       </x:c>
       <x:c r="J68" s="2" t="inlineStr">
@@ -17993,47 +17993,47 @@
     <x:row r="69">
       <x:c r="A69" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.10.6</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.18.3</x:t>
         </x:is>
       </x:c>
       <x:c r="B69" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.10</x:t>
+          <x:t xml:space="preserve">4.4.1.5.18</x:t>
         </x:is>
       </x:c>
       <x:c r="C69" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Lot and Serial Trace Interface</x:t>
+          <x:t xml:space="preserve">Stocktake Create Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D69" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Trace Detail (Table)</x:t>
+          <x:t xml:space="preserve">Item (Select)</x:t>
         </x:is>
       </x:c>
       <x:c r="E69" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Show current locations and movement history with truncation warning.</x:t>
+          <x:t xml:space="preserve">Scrollable multi-select checklist labelled "Items".</x:t>
         </x:is>
       </x:c>
       <x:c r="F69" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Trace provenance.</x:t>
+          <x:t xml:space="preserve">Limit the count to selected items.</x:t>
         </x:is>
       </x:c>
       <x:c r="G69" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Table</x:t>
+          <x:t xml:space="preserve">MD IDs</x:t>
         </x:is>
       </x:c>
       <x:c r="H69" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Most recent 1000 movements</x:t>
+          <x:t xml:space="preserve">0–500 items</x:t>
         </x:is>
       </x:c>
       <x:c r="I69" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.10.5</x:t>
+          <x:t xml:space="preserve">None</x:t>
         </x:is>
       </x:c>
       <x:c r="J69" s="2" t="inlineStr">
@@ -18050,47 +18050,47 @@
     <x:row r="70">
       <x:c r="A70" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.15.1</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.18.4</x:t>
         </x:is>
       </x:c>
       <x:c r="B70" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.15</x:t>
+          <x:t xml:space="preserve">4.4.1.5.18</x:t>
         </x:is>
       </x:c>
       <x:c r="C70" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Inventory Transfer Create Interface</x:t>
+          <x:t xml:space="preserve">Stocktake Create Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D70" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Business Date (Date Picker)</x:t>
+          <x:t xml:space="preserve">Search (Button)</x:t>
         </x:is>
       </x:c>
       <x:c r="E70" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Set transfer business date.</x:t>
+          <x:t xml:space="preserve">Button labeled "Search".</x:t>
         </x:is>
       </x:c>
       <x:c r="F70" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Date both movements.</x:t>
+          <x:t xml:space="preserve">Create the stocktake draft and snapshot of book quantities.</x:t>
         </x:is>
       </x:c>
       <x:c r="G70" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Date</x:t>
+          <x:t xml:space="preserve">Button</x:t>
         </x:is>
       </x:c>
       <x:c r="H70" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Valid business date</x:t>
+          <x:t xml:space="preserve">CREATE; up to 5,000 lines</x:t>
         </x:is>
       </x:c>
       <x:c r="I70" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">None</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.18.1</x:t>
         </x:is>
       </x:c>
       <x:c r="J70" s="2" t="inlineStr">
@@ -18107,47 +18107,47 @@
     <x:row r="71">
       <x:c r="A71" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.15.2</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.18.5</x:t>
         </x:is>
       </x:c>
       <x:c r="B71" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.15</x:t>
+          <x:t xml:space="preserve">4.4.1.5.18</x:t>
         </x:is>
       </x:c>
       <x:c r="C71" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Inventory Transfer Create Interface</x:t>
+          <x:t xml:space="preserve">Stocktake Create Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D71" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Item (Dropdown)</x:t>
+          <x:t xml:space="preserve">Stocktaking Inventory (Input)</x:t>
         </x:is>
       </x:c>
       <x:c r="E71" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Select an active company item per line.</x:t>
+          <x:t xml:space="preserve">Input with header "Stock Taking Inventory" in the stocktake table.</x:t>
         </x:is>
       </x:c>
       <x:c r="F71" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Identify stock.</x:t>
+          <x:t xml:space="preserve">Enter the counted quantity of each line, lot or serial.</x:t>
         </x:is>
       </x:c>
       <x:c r="G71" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MD ID</x:t>
+          <x:t xml:space="preserve">Decimal(19,6)</x:t>
         </x:is>
       </x:c>
       <x:c r="H71" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Active item</x:t>
+          <x:t xml:space="preserve">≥ 0; serial 0 or 1</x:t>
         </x:is>
       </x:c>
       <x:c r="I71" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">None</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.18.4</x:t>
         </x:is>
       </x:c>
       <x:c r="J71" s="2" t="inlineStr">
@@ -18164,47 +18164,47 @@
     <x:row r="72">
       <x:c r="A72" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.15.3</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.18.6</x:t>
         </x:is>
       </x:c>
       <x:c r="B72" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.15</x:t>
+          <x:t xml:space="preserve">4.4.1.5.18</x:t>
         </x:is>
       </x:c>
       <x:c r="C72" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Inventory Transfer Create Interface</x:t>
+          <x:t xml:space="preserve">Stocktake Create Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D72" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Source Warehouse / Location (Dropdown)</x:t>
+          <x:t xml:space="preserve">Remarks (Input)</x:t>
         </x:is>
       </x:c>
       <x:c r="E72" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Select the issuing warehouse and optional bin.</x:t>
+          <x:t xml:space="preserve">Input labelled "Remarks" in the stocktake header.</x:t>
         </x:is>
       </x:c>
       <x:c r="F72" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Set source balance key.</x:t>
+          <x:t xml:space="preserve">Enter remarks of the stocktake.</x:t>
         </x:is>
       </x:c>
       <x:c r="G72" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MD IDs</x:t>
+          <x:t xml:space="preserve">Text</x:t>
         </x:is>
       </x:c>
       <x:c r="H72" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Current company, active</x:t>
+          <x:t xml:space="preserve">0–1000 characters</x:t>
         </x:is>
       </x:c>
       <x:c r="I72" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.15.2</x:t>
+          <x:t xml:space="preserve">None</x:t>
         </x:is>
       </x:c>
       <x:c r="J72" s="2" t="inlineStr">
@@ -18221,47 +18221,47 @@
     <x:row r="73">
       <x:c r="A73" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.15.4</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.18.7</x:t>
         </x:is>
       </x:c>
       <x:c r="B73" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.15</x:t>
+          <x:t xml:space="preserve">4.4.1.5.18</x:t>
         </x:is>
       </x:c>
       <x:c r="C73" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Inventory Transfer Create Interface</x:t>
+          <x:t xml:space="preserve">Stocktake Create Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D73" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Destination Warehouse / Location (Dropdown)</x:t>
+          <x:t xml:space="preserve">Generate Inventory Gain and Loss Document (Button)</x:t>
         </x:is>
       </x:c>
       <x:c r="E73" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Select a different receiving balance key.</x:t>
+          <x:t xml:space="preserve">Save counts and submit the stocktake for approval.</x:t>
         </x:is>
       </x:c>
       <x:c r="F73" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Set destination.</x:t>
+          <x:t xml:space="preserve">Post gains and losses after final approval.</x:t>
         </x:is>
       </x:c>
       <x:c r="G73" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MD IDs</x:t>
+          <x:t xml:space="preserve">Button</x:t>
         </x:is>
       </x:c>
       <x:c r="H73" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Different key, active</x:t>
+          <x:t xml:space="preserve">SUBMIT; all lines counted</x:t>
         </x:is>
       </x:c>
       <x:c r="I73" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.15.3</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.18.5</x:t>
         </x:is>
       </x:c>
       <x:c r="J73" s="2" t="inlineStr">
@@ -18278,47 +18278,47 @@
     <x:row r="74">
       <x:c r="A74" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.15.5</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.18.8</x:t>
         </x:is>
       </x:c>
       <x:c r="B74" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.15</x:t>
+          <x:t xml:space="preserve">4.4.1.5.18</x:t>
         </x:is>
       </x:c>
       <x:c r="C74" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Inventory Transfer Create Interface</x:t>
+          <x:t xml:space="preserve">Stocktake Create Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D74" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Quantity / Tracking (Input)</x:t>
+          <x:t xml:space="preserve">Business Date (Date Picker)</x:t>
         </x:is>
       </x:c>
       <x:c r="E74" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Enter six-decimal base quantity and source lot or serial numbers.</x:t>
+          <x:t xml:space="preserve">Set the stocktake business date.</x:t>
         </x:is>
       </x:c>
       <x:c r="F74" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Transfer exact tracked units.</x:t>
+          <x:t xml:space="preserve">Date the gain and loss movements.</x:t>
         </x:is>
       </x:c>
       <x:c r="G74" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Decimal(19,6) / text</x:t>
+          <x:t xml:space="preserve">Date</x:t>
         </x:is>
       </x:c>
       <x:c r="H74" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Positive; tracking total equals quantity</x:t>
+          <x:t xml:space="preserve">Not later than today</x:t>
         </x:is>
       </x:c>
       <x:c r="I74" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.15.2</x:t>
+          <x:t xml:space="preserve">None</x:t>
         </x:is>
       </x:c>
       <x:c r="J74" s="2" t="inlineStr">
@@ -18335,47 +18335,47 @@
     <x:row r="75">
       <x:c r="A75" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.15.6</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.18.9</x:t>
         </x:is>
       </x:c>
       <x:c r="B75" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.15</x:t>
+          <x:t xml:space="preserve">4.4.1.5.18</x:t>
         </x:is>
       </x:c>
       <x:c r="C75" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Inventory Transfer Create Interface</x:t>
+          <x:t xml:space="preserve">Stocktake Create Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D75" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Save Draft (Button)</x:t>
+          <x:t xml:space="preserve">Add Found Line (Button)</x:t>
         </x:is>
       </x:c>
       <x:c r="E75" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Validate and save without changing stock.</x:t>
+          <x:t xml:space="preserve">Add an item, warehouse and location found on site with zero book quantity.</x:t>
         </x:is>
       </x:c>
       <x:c r="F75" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Prepare approval.</x:t>
+          <x:t xml:space="preserve">Record unbooked stock.</x:t>
         </x:is>
       </x:c>
       <x:c r="G75" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Button</x:t>
+          <x:t xml:space="preserve">Button / MD IDs</x:t>
         </x:is>
       </x:c>
       <x:c r="H75" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">CREATE</x:t>
+          <x:t xml:space="preserve">Warehouse in scope, active item</x:t>
         </x:is>
       </x:c>
       <x:c r="I75" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.15.1</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.18.5</x:t>
         </x:is>
       </x:c>
       <x:c r="J75" s="2" t="inlineStr">
@@ -18392,47 +18392,47 @@
     <x:row r="76">
       <x:c r="A76" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.16.1</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.18.10</x:t>
         </x:is>
       </x:c>
       <x:c r="B76" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.16</x:t>
+          <x:t xml:space="preserve">4.4.1.5.18</x:t>
         </x:is>
       </x:c>
       <x:c r="C76" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Inventory Transfer View Interface</x:t>
+          <x:t xml:space="preserve">Stocktake Create Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D76" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Filters (Input)</x:t>
+          <x:t xml:space="preserve">Save Counts / Fill Uncounted (Button)</x:t>
         </x:is>
       </x:c>
       <x:c r="E76" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Filter by document number, date and status.</x:t>
+          <x:t xml:space="preserve">Save counts with version, or fill uncounted lines with book quantity.</x:t>
         </x:is>
       </x:c>
       <x:c r="F76" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Find transfers.</x:t>
+          <x:t xml:space="preserve">Keep counting progress.</x:t>
         </x:is>
       </x:c>
       <x:c r="G76" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Text / date / status</x:t>
+          <x:t xml:space="preserve">Button</x:t>
         </x:is>
       </x:c>
       <x:c r="H76" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">From ≤ To</x:t>
+          <x:t xml:space="preserve">EDIT</x:t>
         </x:is>
       </x:c>
       <x:c r="I76" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">None</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.18.5</x:t>
         </x:is>
       </x:c>
       <x:c r="J76" s="2" t="inlineStr">
@@ -18449,47 +18449,47 @@
     <x:row r="77">
       <x:c r="A77" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.16.2</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.18.11</x:t>
         </x:is>
       </x:c>
       <x:c r="B77" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.16</x:t>
+          <x:t xml:space="preserve">4.4.1.5.18</x:t>
         </x:is>
       </x:c>
       <x:c r="C77" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Inventory Transfer View Interface</x:t>
+          <x:t xml:space="preserve">Stocktake Create Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D77" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Transfer List (Table)</x:t>
+          <x:t xml:space="preserve">Refresh Snapshot (Button)</x:t>
         </x:is>
       </x:c>
       <x:c r="E77" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Show paged company transfers, quantity and approval state.</x:t>
+          <x:t xml:space="preserve">Re-read book quantities, keep counts and flag changed lines.</x:t>
         </x:is>
       </x:c>
       <x:c r="F77" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Review records.</x:t>
+          <x:t xml:space="preserve">Resolve a stale snapshot.</x:t>
         </x:is>
       </x:c>
       <x:c r="G77" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Table</x:t>
+          <x:t xml:space="preserve">Button</x:t>
         </x:is>
       </x:c>
       <x:c r="H77" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">VIEW</x:t>
+          <x:t xml:space="preserve">EDIT; draft only</x:t>
         </x:is>
       </x:c>
       <x:c r="I77" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.16.1</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.18.4</x:t>
         </x:is>
       </x:c>
       <x:c r="J77" s="2" t="inlineStr">
@@ -18506,47 +18506,47 @@
     <x:row r="78">
       <x:c r="A78" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.16.3</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.21.1</x:t>
         </x:is>
       </x:c>
       <x:c r="B78" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.16</x:t>
+          <x:t xml:space="preserve">4.4.1.5.21</x:t>
         </x:is>
       </x:c>
       <x:c r="C78" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Inventory Transfer View Interface</x:t>
+          <x:t xml:space="preserve">Product Initial Stock View Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D78" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Detail (Panel)</x:t>
+          <x:t xml:space="preserve">Opening Date Range (Date Picker)</x:t>
         </x:is>
       </x:c>
       <x:c r="E78" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Show stored lines, both locations, tracking and approval.</x:t>
+          <x:t xml:space="preserve">Filter batches by opening date inclusively.</x:t>
         </x:is>
       </x:c>
       <x:c r="F78" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Inspect movement pair.</x:t>
+          <x:t xml:space="preserve">Narrow results.</x:t>
         </x:is>
       </x:c>
       <x:c r="G78" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Panel</x:t>
+          <x:t xml:space="preserve">Date</x:t>
         </x:is>
       </x:c>
       <x:c r="H78" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">VIEW</x:t>
+          <x:t xml:space="preserve">From ≤ To</x:t>
         </x:is>
       </x:c>
       <x:c r="I78" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.16.2</x:t>
+          <x:t xml:space="preserve">None</x:t>
         </x:is>
       </x:c>
       <x:c r="J78" s="2" t="inlineStr">
@@ -18563,47 +18563,47 @@
     <x:row r="79">
       <x:c r="A79" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.16.4</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.21.2</x:t>
         </x:is>
       </x:c>
       <x:c r="B79" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.16</x:t>
+          <x:t xml:space="preserve">4.4.1.5.21</x:t>
         </x:is>
       </x:c>
       <x:c r="C79" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Inventory Transfer View Interface</x:t>
+          <x:t xml:space="preserve">Product Initial Stock View Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D79" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Submit / Delete (Button)</x:t>
+          <x:t xml:space="preserve">Item / Warehouse (Dropdown)</x:t>
         </x:is>
       </x:c>
       <x:c r="E79" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Submit a draft or delete a draft with confirmation.</x:t>
+          <x:t xml:space="preserve">Filter batches containing the MD item or warehouse.</x:t>
         </x:is>
       </x:c>
       <x:c r="F79" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Control lifecycle.</x:t>
+          <x:t xml:space="preserve">Narrow results.</x:t>
         </x:is>
       </x:c>
       <x:c r="G79" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Button</x:t>
+          <x:t xml:space="preserve">ID</x:t>
         </x:is>
       </x:c>
       <x:c r="H79" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SUBMIT / DELETE</x:t>
+          <x:t xml:space="preserve">Current company</x:t>
         </x:is>
       </x:c>
       <x:c r="I79" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.16.2</x:t>
+          <x:t xml:space="preserve">None</x:t>
         </x:is>
       </x:c>
       <x:c r="J79" s="2" t="inlineStr">
@@ -18620,47 +18620,47 @@
     <x:row r="80">
       <x:c r="A80" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.16.5</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.21.3</x:t>
         </x:is>
       </x:c>
       <x:c r="B80" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.16</x:t>
+          <x:t xml:space="preserve">4.4.1.5.21</x:t>
         </x:is>
       </x:c>
       <x:c r="C80" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Inventory Transfer View Interface</x:t>
+          <x:t xml:space="preserve">Product Initial Stock View Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D80" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Print / Export (Button)</x:t>
+          <x:t xml:space="preserve">Keyword (Textbox)</x:t>
         </x:is>
       </x:c>
       <x:c r="E80" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Print detail or export filtered records to safe UTF-8 CSV.</x:t>
+          <x:t xml:space="preserve">Match remark or request key.</x:t>
         </x:is>
       </x:c>
       <x:c r="F80" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Keep transfer records.</x:t>
+          <x:t xml:space="preserve">Find a batch.</x:t>
         </x:is>
       </x:c>
       <x:c r="G80" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Button</x:t>
+          <x:t xml:space="preserve">Text</x:t>
         </x:is>
       </x:c>
       <x:c r="H80" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">VIEW</x:t>
+          <x:t xml:space="preserve">Partial match</x:t>
         </x:is>
       </x:c>
       <x:c r="I80" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.16.2</x:t>
+          <x:t xml:space="preserve">None</x:t>
         </x:is>
       </x:c>
       <x:c r="J80" s="2" t="inlineStr">
@@ -18677,47 +18677,47 @@
     <x:row r="81">
       <x:c r="A81" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.17.1</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.21.4</x:t>
         </x:is>
       </x:c>
       <x:c r="B81" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.17</x:t>
+          <x:t xml:space="preserve">4.4.1.5.21</x:t>
         </x:is>
       </x:c>
       <x:c r="C81" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Inventory Transfer Edit Interface</x:t>
+          <x:t xml:space="preserve">Product Initial Stock View Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D81" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Business Date / Remark (Input)</x:t>
+          <x:t xml:space="preserve">Batch List (Table)</x:t>
         </x:is>
       </x:c>
       <x:c r="E81" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Revise a draft or rejected transfer.</x:t>
+          <x:t xml:space="preserve">Paged batches with lines, quantity, amount, remark and posted time.</x:t>
         </x:is>
       </x:c>
       <x:c r="F81" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Correct header.</x:t>
+          <x:t xml:space="preserve">Review opening stock.</x:t>
         </x:is>
       </x:c>
       <x:c r="G81" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Date / text</x:t>
+          <x:t xml:space="preserve">Table</x:t>
         </x:is>
       </x:c>
       <x:c r="H81" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Editable status</x:t>
+          <x:t xml:space="preserve">Authorized company</x:t>
         </x:is>
       </x:c>
       <x:c r="I81" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">None</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.21.1</x:t>
         </x:is>
       </x:c>
       <x:c r="J81" s="2" t="inlineStr">
@@ -18734,47 +18734,47 @@
     <x:row r="82">
       <x:c r="A82" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.17.2</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.21.5</x:t>
         </x:is>
       </x:c>
       <x:c r="B82" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.17</x:t>
+          <x:t xml:space="preserve">4.4.1.5.21</x:t>
         </x:is>
       </x:c>
       <x:c r="C82" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Inventory Transfer Edit Interface</x:t>
+          <x:t xml:space="preserve">Product Initial Stock View Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D82" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Source / Destination (Dropdown)</x:t>
+          <x:t xml:space="preserve">Batch Detail (Panel)</x:t>
         </x:is>
       </x:c>
       <x:c r="E82" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Revise both balance keys per line.</x:t>
+          <x:t xml:space="preserve">Lines by line number with MD names, quantity, unit cost and amount.</x:t>
         </x:is>
       </x:c>
       <x:c r="F82" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Correct route.</x:t>
+          <x:t xml:space="preserve">Inspect a batch.</x:t>
         </x:is>
       </x:c>
       <x:c r="G82" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MD IDs</x:t>
+          <x:t xml:space="preserve">Table</x:t>
         </x:is>
       </x:c>
       <x:c r="H82" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Different active keys</x:t>
+          <x:t xml:space="preserve">Authorized company</x:t>
         </x:is>
       </x:c>
       <x:c r="I82" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.17.1</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.21.4</x:t>
         </x:is>
       </x:c>
       <x:c r="J82" s="2" t="inlineStr">
@@ -18791,47 +18791,47 @@
     <x:row r="83">
       <x:c r="A83" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.17.3</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.21.6</x:t>
         </x:is>
       </x:c>
       <x:c r="B83" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.17</x:t>
+          <x:t xml:space="preserve">4.4.1.5.21</x:t>
         </x:is>
       </x:c>
       <x:c r="C83" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Inventory Transfer Edit Interface</x:t>
+          <x:t xml:space="preserve">Product Initial Stock View Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D83" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Quantity / Tracking (Input)</x:t>
+          <x:t xml:space="preserve">Print / Export (Button)</x:t>
         </x:is>
       </x:c>
       <x:c r="E83" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Revise quantity and matching lot or serial list.</x:t>
+          <x:t xml:space="preserve">Print one batch; export filtered batches as formula-safe UTF-8 CSV.</x:t>
         </x:is>
       </x:c>
       <x:c r="F83" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Correct moved units.</x:t>
+          <x:t xml:space="preserve">Keep records.</x:t>
         </x:is>
       </x:c>
       <x:c r="G83" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Decimal(19,6) / text</x:t>
+          <x:t xml:space="preserve">Button</x:t>
         </x:is>
       </x:c>
       <x:c r="H83" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Tracking total equals quantity at submit</x:t>
+          <x:t xml:space="preserve">Authorized</x:t>
         </x:is>
       </x:c>
       <x:c r="I83" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.17.2</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.21.4</x:t>
         </x:is>
       </x:c>
       <x:c r="J83" s="2" t="inlineStr">
@@ -18848,47 +18848,47 @@
     <x:row r="84">
       <x:c r="A84" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.17.4</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.22.1</x:t>
         </x:is>
       </x:c>
       <x:c r="B84" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.17</x:t>
+          <x:t xml:space="preserve">4.4.1.5.22</x:t>
         </x:is>
       </x:c>
       <x:c r="C84" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Inventory Transfer Edit Interface</x:t>
+          <x:t xml:space="preserve">Product Initial Stock Create Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D84" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Save Revision (Button)</x:t>
+          <x:t xml:space="preserve">Opening Date (Date Picker)</x:t>
         </x:is>
       </x:c>
       <x:c r="E84" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Replace draft lines with version check.</x:t>
+          <x:t xml:space="preserve">Date the opening balance takes effect.</x:t>
         </x:is>
       </x:c>
       <x:c r="F84" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Persist correction.</x:t>
+          <x:t xml:space="preserve">Set start of stock history.</x:t>
         </x:is>
       </x:c>
       <x:c r="G84" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Button</x:t>
+          <x:t xml:space="preserve">Date</x:t>
         </x:is>
       </x:c>
       <x:c r="H84" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">EDIT</x:t>
+          <x:t xml:space="preserve">≤ today; ≤ earliest movement</x:t>
         </x:is>
       </x:c>
       <x:c r="I84" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.17.1</x:t>
+          <x:t xml:space="preserve">None</x:t>
         </x:is>
       </x:c>
       <x:c r="J84" s="2" t="inlineStr">
@@ -18905,47 +18905,47 @@
     <x:row r="85">
       <x:c r="A85" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.18.1</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.22.2</x:t>
         </x:is>
       </x:c>
       <x:c r="B85" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.18</x:t>
+          <x:t xml:space="preserve">4.4.1.5.22</x:t>
         </x:is>
       </x:c>
       <x:c r="C85" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Stocktake Create Interface</x:t>
+          <x:t xml:space="preserve">Product Initial Stock Create Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D85" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Warehouse (Select)</x:t>
+          <x:t xml:space="preserve">Item / Warehouse / Location (Dropdown)</x:t>
         </x:is>
       </x:c>
       <x:c r="E85" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Select labelled "Select Warehouse".</x:t>
+          <x:t xml:space="preserve">Active MD references per line; location limited to the warehouse.</x:t>
         </x:is>
       </x:c>
       <x:c r="F85" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Choose one or more warehouses to count.</x:t>
+          <x:t xml:space="preserve">Identify balance key.</x:t>
         </x:is>
       </x:c>
       <x:c r="G85" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MD IDs</x:t>
+          <x:t xml:space="preserve">ID</x:t>
         </x:is>
       </x:c>
       <x:c r="H85" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">1–20 active company warehouses</x:t>
+          <x:t xml:space="preserve">Active, current company</x:t>
         </x:is>
       </x:c>
       <x:c r="I85" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">None</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.22.1</x:t>
         </x:is>
       </x:c>
       <x:c r="J85" s="2" t="inlineStr">
@@ -18962,47 +18962,47 @@
     <x:row r="86">
       <x:c r="A86" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.18.2</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.22.3</x:t>
         </x:is>
       </x:c>
       <x:c r="B86" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.18</x:t>
+          <x:t xml:space="preserve">4.4.1.5.22</x:t>
         </x:is>
       </x:c>
       <x:c r="C86" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Stocktake Create Interface</x:t>
+          <x:t xml:space="preserve">Product Initial Stock Create Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D86" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Category (Select)</x:t>
+          <x:t xml:space="preserve">Quantity / Unit Cost (Textbox)</x:t>
         </x:is>
       </x:c>
       <x:c r="E86" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Select labelled "Category".</x:t>
+          <x:t xml:space="preserve">Base-unit quantity and unit cost.</x:t>
         </x:is>
       </x:c>
       <x:c r="F86" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Limit the count to item categories and their children.</x:t>
+          <x:t xml:space="preserve">Value opening stock.</x:t>
         </x:is>
       </x:c>
       <x:c r="G86" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MD IDs</x:t>
+          <x:t xml:space="preserve">Decimal(6)</x:t>
         </x:is>
       </x:c>
       <x:c r="H86" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">0–50 categories</x:t>
+          <x:t xml:space="preserve">Quantity &gt; 0; cost ≥ 0</x:t>
         </x:is>
       </x:c>
       <x:c r="I86" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">None</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.22.2</x:t>
         </x:is>
       </x:c>
       <x:c r="J86" s="2" t="inlineStr">
@@ -19019,47 +19019,47 @@
     <x:row r="87">
       <x:c r="A87" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.18.3</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.22.4</x:t>
         </x:is>
       </x:c>
       <x:c r="B87" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.18</x:t>
+          <x:t xml:space="preserve">4.4.1.5.22</x:t>
         </x:is>
       </x:c>
       <x:c r="C87" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Stocktake Create Interface</x:t>
+          <x:t xml:space="preserve">Product Initial Stock Create Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D87" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Item (Select)</x:t>
+          <x:t xml:space="preserve">Preview (Button)</x:t>
         </x:is>
       </x:c>
       <x:c r="E87" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Scrollable multi-select checklist labelled "Items".</x:t>
+          <x:t xml:space="preserve">Validate without saving; show per-line trilingual errors and totals.</x:t>
         </x:is>
       </x:c>
       <x:c r="F87" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Limit the count to selected items.</x:t>
+          <x:t xml:space="preserve">Catch errors before posting.</x:t>
         </x:is>
       </x:c>
       <x:c r="G87" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">MD IDs</x:t>
+          <x:t xml:space="preserve">Button</x:t>
         </x:is>
       </x:c>
       <x:c r="H87" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">0–500 items</x:t>
+          <x:t xml:space="preserve">CREATE</x:t>
         </x:is>
       </x:c>
       <x:c r="I87" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">None</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.22.1</x:t>
         </x:is>
       </x:c>
       <x:c r="J87" s="2" t="inlineStr">
@@ -19076,32 +19076,32 @@
     <x:row r="88">
       <x:c r="A88" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.18.4</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.22.5</x:t>
         </x:is>
       </x:c>
       <x:c r="B88" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.18</x:t>
+          <x:t xml:space="preserve">4.4.1.5.22</x:t>
         </x:is>
       </x:c>
       <x:c r="C88" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Stocktake Create Interface</x:t>
+          <x:t xml:space="preserve">Product Initial Stock Create Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D88" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Search (Button)</x:t>
+          <x:t xml:space="preserve">Submit (Button)</x:t>
         </x:is>
       </x:c>
       <x:c r="E88" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Button labeled "Search".</x:t>
+          <x:t xml:space="preserve">Post a clean, unchanged preview once; retry reuses the batch request key.</x:t>
         </x:is>
       </x:c>
       <x:c r="F88" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Create the stocktake draft and snapshot of book quantities.</x:t>
+          <x:t xml:space="preserve">Post opening stock idempotently.</x:t>
         </x:is>
       </x:c>
       <x:c r="G88" s="2" t="inlineStr">
@@ -19111,12 +19111,12 @@
       </x:c>
       <x:c r="H88" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">CREATE; up to 5,000 lines</x:t>
+          <x:t xml:space="preserve">Clean preview</x:t>
         </x:is>
       </x:c>
       <x:c r="I88" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.18.1</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.22.4</x:t>
         </x:is>
       </x:c>
       <x:c r="J88" s="2" t="inlineStr">
@@ -19133,47 +19133,47 @@
     <x:row r="89">
       <x:c r="A89" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.18.5</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.22.6</x:t>
         </x:is>
       </x:c>
       <x:c r="B89" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.18</x:t>
+          <x:t xml:space="preserve">4.4.1.5.22</x:t>
         </x:is>
       </x:c>
       <x:c r="C89" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Stocktake Create Interface</x:t>
+          <x:t xml:space="preserve">Product Initial Stock Create Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D89" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Stocktaking Inventory (Input)</x:t>
+          <x:t xml:space="preserve">Lot or Serial (Input)</x:t>
         </x:is>
       </x:c>
       <x:c r="E89" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Input with header "Stock Taking Inventory" in the stocktake table.</x:t>
+          <x:t xml:space="preserve">Capture opening stock tracking entries.</x:t>
         </x:is>
       </x:c>
       <x:c r="F89" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Enter the counted quantity of each line, lot or serial.</x:t>
+          <x:t xml:space="preserve">Establish tracked opening stock.</x:t>
         </x:is>
       </x:c>
       <x:c r="G89" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Decimal(19,6)</x:t>
+          <x:t xml:space="preserve">Lot rows or serial lines</x:t>
         </x:is>
       </x:c>
       <x:c r="H89" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">≥ 0; serial 0 or 1</x:t>
+          <x:t xml:space="preserve">Sum equals line quantity</x:t>
         </x:is>
       </x:c>
       <x:c r="I89" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.18.4</x:t>
+          <x:t xml:space="preserve">None</x:t>
         </x:is>
       </x:c>
       <x:c r="J89" s="2" t="inlineStr">
@@ -19190,42 +19190,42 @@
     <x:row r="90">
       <x:c r="A90" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.18.6</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.23.1</x:t>
         </x:is>
       </x:c>
       <x:c r="B90" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.18</x:t>
+          <x:t xml:space="preserve">4.4.1.5.23</x:t>
         </x:is>
       </x:c>
       <x:c r="C90" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Stocktake Create Interface</x:t>
+          <x:t xml:space="preserve">Lot and Serial Trace Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D90" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Remarks (Input)</x:t>
+          <x:t xml:space="preserve">Tracking Type (Button)</x:t>
         </x:is>
       </x:c>
       <x:c r="E90" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Input labelled "Remarks" in the stocktake header.</x:t>
+          <x:t xml:space="preserve">Switch between lot and serial lists.</x:t>
         </x:is>
       </x:c>
       <x:c r="F90" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Enter remarks of the stocktake.</x:t>
+          <x:t xml:space="preserve">Select tracking type.</x:t>
         </x:is>
       </x:c>
       <x:c r="G90" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Text</x:t>
+          <x:t xml:space="preserve">Button</x:t>
         </x:is>
       </x:c>
       <x:c r="H90" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">0–1000 characters</x:t>
+          <x:t xml:space="preserve">Lot / Serial</x:t>
         </x:is>
       </x:c>
       <x:c r="I90" s="2" t="inlineStr">
@@ -19247,47 +19247,47 @@
     <x:row r="91">
       <x:c r="A91" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.18.7</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.23.2</x:t>
         </x:is>
       </x:c>
       <x:c r="B91" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.18</x:t>
+          <x:t xml:space="preserve">4.4.1.5.23</x:t>
         </x:is>
       </x:c>
       <x:c r="C91" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Stocktake Create Interface</x:t>
+          <x:t xml:space="preserve">Lot and Serial Trace Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D91" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Generate Inventory Gain and Loss Document (Button)</x:t>
+          <x:t xml:space="preserve">Item (Dropdown)</x:t>
         </x:is>
       </x:c>
       <x:c r="E91" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Save counts and submit the stocktake for approval.</x:t>
+          <x:t xml:space="preserve">Filter by company item.</x:t>
         </x:is>
       </x:c>
       <x:c r="F91" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Post gains and losses after final approval.</x:t>
+          <x:t xml:space="preserve">Narrow trace results.</x:t>
         </x:is>
       </x:c>
       <x:c r="G91" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Button</x:t>
+          <x:t xml:space="preserve">ID</x:t>
         </x:is>
       </x:c>
       <x:c r="H91" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">SUBMIT; all lines counted</x:t>
+          <x:t xml:space="preserve">Current company</x:t>
         </x:is>
       </x:c>
       <x:c r="I91" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.18.5</x:t>
+          <x:t xml:space="preserve">None</x:t>
         </x:is>
       </x:c>
       <x:c r="J91" s="2" t="inlineStr">
@@ -19304,42 +19304,42 @@
     <x:row r="92">
       <x:c r="A92" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.18.8</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.23.3</x:t>
         </x:is>
       </x:c>
       <x:c r="B92" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.18</x:t>
+          <x:t xml:space="preserve">4.4.1.5.23</x:t>
         </x:is>
       </x:c>
       <x:c r="C92" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Stocktake Create Interface</x:t>
+          <x:t xml:space="preserve">Lot and Serial Trace Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D92" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Business Date (Date Picker)</x:t>
+          <x:t xml:space="preserve">Number Search (Input)</x:t>
         </x:is>
       </x:c>
       <x:c r="E92" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Set the stocktake business date.</x:t>
+          <x:t xml:space="preserve">Filter lot or serial number.</x:t>
         </x:is>
       </x:c>
       <x:c r="F92" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Date the gain and loss movements.</x:t>
+          <x:t xml:space="preserve">Find tracking number.</x:t>
         </x:is>
       </x:c>
       <x:c r="G92" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Date</x:t>
+          <x:t xml:space="preserve">Text</x:t>
         </x:is>
       </x:c>
       <x:c r="H92" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Not later than today</x:t>
+          <x:t xml:space="preserve">Up to 100 characters</x:t>
         </x:is>
       </x:c>
       <x:c r="I92" s="2" t="inlineStr">
@@ -19361,47 +19361,47 @@
     <x:row r="93">
       <x:c r="A93" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.18.9</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.23.4</x:t>
         </x:is>
       </x:c>
       <x:c r="B93" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.18</x:t>
+          <x:t xml:space="preserve">4.4.1.5.23</x:t>
         </x:is>
       </x:c>
       <x:c r="C93" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Stocktake Create Interface</x:t>
+          <x:t xml:space="preserve">Lot and Serial Trace Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D93" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Add Found Line (Button)</x:t>
+          <x:t xml:space="preserve">In Stock Only (Checkbox)</x:t>
         </x:is>
       </x:c>
       <x:c r="E93" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Add an item, warehouse and location found on site with zero book quantity.</x:t>
+          <x:t xml:space="preserve">Exclude fully issued numbers.</x:t>
         </x:is>
       </x:c>
       <x:c r="F93" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Record unbooked stock.</x:t>
+          <x:t xml:space="preserve">Show current stock.</x:t>
         </x:is>
       </x:c>
       <x:c r="G93" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Button / MD IDs</x:t>
+          <x:t xml:space="preserve">Boolean</x:t>
         </x:is>
       </x:c>
       <x:c r="H93" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Warehouse in scope, active item</x:t>
+          <x:t xml:space="preserve">True / false</x:t>
         </x:is>
       </x:c>
       <x:c r="I93" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.18.5</x:t>
+          <x:t xml:space="preserve">None</x:t>
         </x:is>
       </x:c>
       <x:c r="J93" s="2" t="inlineStr">
@@ -19418,47 +19418,47 @@
     <x:row r="94">
       <x:c r="A94" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.18.10</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.23.5</x:t>
         </x:is>
       </x:c>
       <x:c r="B94" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.18</x:t>
+          <x:t xml:space="preserve">4.4.1.5.23</x:t>
         </x:is>
       </x:c>
       <x:c r="C94" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Stocktake Create Interface</x:t>
+          <x:t xml:space="preserve">Lot and Serial Trace Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D94" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Save Counts / Fill Uncounted (Button)</x:t>
+          <x:t xml:space="preserve">Tracking Results (Table)</x:t>
         </x:is>
       </x:c>
       <x:c r="E94" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Save counts with version, or fill uncounted lines with book quantity.</x:t>
+          <x:t xml:space="preserve">Show paged lot or serial records.</x:t>
         </x:is>
       </x:c>
       <x:c r="F94" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Keep counting progress.</x:t>
+          <x:t xml:space="preserve">Inspect on-hand status.</x:t>
         </x:is>
       </x:c>
       <x:c r="G94" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Button</x:t>
+          <x:t xml:space="preserve">Table</x:t>
         </x:is>
       </x:c>
       <x:c r="H94" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">EDIT</x:t>
+          <x:t xml:space="preserve">Current company</x:t>
         </x:is>
       </x:c>
       <x:c r="I94" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.18.5</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.23.1</x:t>
         </x:is>
       </x:c>
       <x:c r="J94" s="2" t="inlineStr">
@@ -19475,47 +19475,47 @@
     <x:row r="95">
       <x:c r="A95" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.18.11</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.23.6</x:t>
         </x:is>
       </x:c>
       <x:c r="B95" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.18</x:t>
+          <x:t xml:space="preserve">4.4.1.5.23</x:t>
         </x:is>
       </x:c>
       <x:c r="C95" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Stocktake Create Interface</x:t>
+          <x:t xml:space="preserve">Lot and Serial Trace Interface</x:t>
         </x:is>
       </x:c>
       <x:c r="D95" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Refresh Snapshot (Button)</x:t>
+          <x:t xml:space="preserve">Trace Detail (Table)</x:t>
         </x:is>
       </x:c>
       <x:c r="E95" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Re-read book quantities, keep counts and flag changed lines.</x:t>
+          <x:t xml:space="preserve">Show current locations and movement history with truncation warning.</x:t>
         </x:is>
       </x:c>
       <x:c r="F95" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Resolve a stale snapshot.</x:t>
+          <x:t xml:space="preserve">Trace provenance.</x:t>
         </x:is>
       </x:c>
       <x:c r="G95" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Button</x:t>
+          <x:t xml:space="preserve">Table</x:t>
         </x:is>
       </x:c>
       <x:c r="H95" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">EDIT; draft only</x:t>
+          <x:t xml:space="preserve">Most recent 1000 movements</x:t>
         </x:is>
       </x:c>
       <x:c r="I95" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.18.4</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.23.5</x:t>
         </x:is>
       </x:c>
       <x:c r="J95" s="2" t="inlineStr">
@@ -38089,17 +38089,17 @@
       </x:c>
       <x:c r="D38" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.8</x:t>
+          <x:t xml:space="preserve">4.4.1.5.21</x:t>
         </x:is>
       </x:c>
       <x:c r="E38" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.8.1, REQ_IO_A5.8.2, REQ_IO_A5.8.3, REQ_IO_A5.8.4, REQ_IO_A5.8.5, REQ_IO_A5.8.6</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.21.1, REQ_IO_A5.21.2, REQ_IO_A5.21.3, REQ_IO_A5.21.4, REQ_IO_A5.21.5, REQ_IO_A5.21.6</x:t>
         </x:is>
       </x:c>
       <x:c r="F38" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">INV-OPN-005, INV-OPN-006, INV-OPN-007</x:t>
+          <x:t xml:space="preserve">INV-DOC-001, INV-DOC-002, INV-OPN-005, INV-OPN-006, INV-OPN-007</x:t>
         </x:is>
       </x:c>
       <x:c r="G38" s="2" t="inlineStr">
@@ -38126,17 +38126,17 @@
       </x:c>
       <x:c r="D39" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.9</x:t>
+          <x:t xml:space="preserve">4.4.1.5.22</x:t>
         </x:is>
       </x:c>
       <x:c r="E39" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.9.1, REQ_IO_A5.9.4</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.22.1, REQ_IO_A5.22.4</x:t>
         </x:is>
       </x:c>
       <x:c r="F39" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">INV-OPN-001, INV-OPN-004, INV-OPN-006, INV-OPN-007</x:t>
+          <x:t xml:space="preserve">INV-DOC-001, INV-OPN-001, INV-OPN-004, INV-OPN-006, INV-OPN-007</x:t>
         </x:is>
       </x:c>
       <x:c r="G39" s="2" t="inlineStr">
@@ -38163,12 +38163,12 @@
       </x:c>
       <x:c r="D40" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.9</x:t>
+          <x:t xml:space="preserve">4.4.1.5.22</x:t>
         </x:is>
       </x:c>
       <x:c r="E40" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.9.1, REQ_IO_A5.9.2, REQ_IO_A5.9.3, REQ_IO_A5.9.5</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.22.1, REQ_IO_A5.22.2, REQ_IO_A5.22.3, REQ_IO_A5.22.5</x:t>
         </x:is>
       </x:c>
       <x:c r="F40" s="2" t="inlineStr">
@@ -38200,12 +38200,12 @@
       </x:c>
       <x:c r="D41" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.9</x:t>
+          <x:t xml:space="preserve">4.4.1.5.22</x:t>
         </x:is>
       </x:c>
       <x:c r="E41" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.9.5</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.22.5</x:t>
         </x:is>
       </x:c>
       <x:c r="F41" s="2" t="inlineStr">
@@ -38242,7 +38242,7 @@
       </x:c>
       <x:c r="E42" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.2.8, REQ_IO_A5.9.6</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.2.8, REQ_IO_A5.22.6</x:t>
         </x:is>
       </x:c>
       <x:c r="F42" s="2" t="inlineStr">
@@ -38279,7 +38279,7 @@
       </x:c>
       <x:c r="E43" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.2.8, REQ_IO_A5.9.6</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.2.8, REQ_IO_A5.22.6</x:t>
         </x:is>
       </x:c>
       <x:c r="F43" s="2" t="inlineStr">
@@ -38353,7 +38353,7 @@
       </x:c>
       <x:c r="E45" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.2.8, REQ_IO_A5.5.8, REQ_IO_A5.9.6</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.2.8, REQ_IO_A5.5.8, REQ_IO_A5.22.6</x:t>
         </x:is>
       </x:c>
       <x:c r="F45" s="2" t="inlineStr">
@@ -38385,17 +38385,17 @@
       </x:c>
       <x:c r="D46" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.10</x:t>
+          <x:t xml:space="preserve">4.4.1.5.23</x:t>
         </x:is>
       </x:c>
       <x:c r="E46" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.10.1, REQ_IO_A5.10.2, REQ_IO_A5.10.3, REQ_IO_A5.10.4, REQ_IO_A5.10.5</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.23.1, REQ_IO_A5.23.2, REQ_IO_A5.23.3, REQ_IO_A5.23.4, REQ_IO_A5.23.5</x:t>
         </x:is>
       </x:c>
       <x:c r="F46" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">INV-LOT-012, INV-LOT-015, INV-LOT-UI-002, INV-LOT-UI-003</x:t>
+          <x:t xml:space="preserve">INV-DOC-001, INV-DOC-002, INV-LOT-012, INV-LOT-015, INV-LOT-UI-002, INV-LOT-UI-003</x:t>
         </x:is>
       </x:c>
       <x:c r="G46" s="2" t="inlineStr">
@@ -38422,12 +38422,12 @@
       </x:c>
       <x:c r="D47" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">4.4.1.5.10</x:t>
+          <x:t xml:space="preserve">4.4.1.5.23</x:t>
         </x:is>
       </x:c>
       <x:c r="E47" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.10.6</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.23.6</x:t>
         </x:is>
       </x:c>
       <x:c r="F47" s="2" t="inlineStr">
@@ -56723,7 +56723,7 @@
       </x:c>
       <x:c r="F327" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">完成（WU-INV-007a API 經 OPENING_STOCK 寫庫存異動帳；007b 三語介面 5.8／5.9）</x:t>
+          <x:t xml:space="preserve">完成（WU-INV-007a API 經 OPENING_STOCK 寫庫存異動帳；007b 三語介面 5.21／5.22）</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
feat(inv): add moving-average valuation query
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Reb2920f6d92747bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R90a09d39f3414d2c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Rff6a783495e24149"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R8cde225529094d08"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Rb3ebdfce8b024fab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R3c68a30677cf400b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R1ac482338b3349d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R31d9d3d798a14ae5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R85b6f5fa94074ab5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R3bc0c3eed13649cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Rda581103852f486c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Rb6cffca351414115"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R3ea7f4acc60e42fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Rc772b8fdbeb6486b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R4420359d852d4f13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Rf2114d32264c4a32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="Re7c92dd1a70e4e86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Re10f010f282a4a1e"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
feat(inv): add authorized provisional valuation view
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R3bc0c3eed13649cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Rda581103852f486c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Rb6cffca351414115"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R3ea7f4acc60e42fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Rc772b8fdbeb6486b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R4420359d852d4f13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Rf2114d32264c4a32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="Re7c92dd1a70e4e86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Re10f010f282a4a1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Rce1af9674dca40fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R9c246fa62b4548c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R8368e283a8744c9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Raf8acda3062a493d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R0fb880efbd9e4fab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="Rd2f38be0e3a146ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R9a4734edb2714884"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R00a15be1d1ea4d63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R69a9c4f3294d40f8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19963,7 +19963,7 @@
       </x:c>
       <x:c r="E101" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Select a company item through the MD lookup.</x:t>
+          <x:t xml:space="preserve">Select a company item through the INV valuation options backed by the MD read-only contract; only valuation permission is required.</x:t>
         </x:is>
       </x:c>
       <x:c r="F101" s="2" t="inlineStr">
@@ -20072,12 +20072,12 @@
       </x:c>
       <x:c r="D103" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Valuation Result (Table)</x:t>
+          <x:t xml:space="preserve">Valuation Result (Panel)</x:t>
         </x:is>
       </x:c>
       <x:c r="E103" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Show six-place quantity, four-place value, average cost and provisional status.</x:t>
+          <x:t xml:space="preserve">Show six-place quantity, four-place value, average cost, movement count, cutoff and provisional status.</x:t>
         </x:is>
       </x:c>
       <x:c r="F103" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat(inv): add external purchase and sales posting contract
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R770a69a5abb24bee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R26f32808bcc3441c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R8e9f1bbcbfa94d5f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Rd44b6a62c0cb48d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R2f6f0af939ec455b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R2ca3067b6a304c88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Ref2832d7fed94de1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R028379a3758b4a6a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R4bea62b666c44fab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Rb32d3541eed14d23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Rca34d9d31c654fb1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R8c0f8642024b4ed4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Rbc6e425b28744633"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Re1ed608ecf0742cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R16b0fe4811284fa9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R1f5861ddef1047d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R21c79b3376a1475b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rb1d441173ad04f4a"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
feat(inv): use authorized selectors in transfer and opening forms
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R0d0f3817624c469e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Re0f225ac3acc474c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R75dc716a956548c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R05e0dc859f8d4820"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Refc5c18399a14d86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R40eab5f69e874db5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Rd048392e1e3e478a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R934ebe4ed7bc42ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rd0d2a83ddd634e5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R470f6fd200164056"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R3610c82448034df2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R3c7e9e5f94284a44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Re8839f0894624a76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Ra17a4441f41a4312"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R44f0487635cf4d3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R06283767106d475f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R8d59aab31344441e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Radb0175af7344897"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
feat(inv): complete stocktake selection dialogs
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R470f6fd200164056"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R3610c82448034df2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R3c7e9e5f94284a44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Re8839f0894624a76"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Ra17a4441f41a4312"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R44f0487635cf4d3d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R06283767106d475f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R8d59aab31344441e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Radb0175af7344897"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R9f3a0e7f52d8485b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Rb9bea040dbfb437d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R0e7bb2d13a1e4d1a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R77d91017f71a40f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R6c1f8864fbd14860"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R501ab0289b3a46f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R84b79f73be40496e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R5c168c446a154c13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R15b85fdae8db43ba"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18235,7 +18235,7 @@
       </x:c>
       <x:c r="E67" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Select labelled "Select Warehouse".</x:t>
+          <x:t xml:space="preserve">Open the paged Select Data Interface for multiple warehouses and show confirmed choices.</x:t>
         </x:is>
       </x:c>
       <x:c r="F67" s="2" t="inlineStr">
@@ -18255,7 +18255,7 @@
       </x:c>
       <x:c r="I67" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">None</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.20.1</x:t>
         </x:is>
       </x:c>
       <x:c r="J67" s="2" t="inlineStr">
@@ -18349,7 +18349,7 @@
       </x:c>
       <x:c r="E69" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Scrollable multi-select checklist labelled "Items".</x:t>
+          <x:t xml:space="preserve">Open the paged Select Data Interface for multiple items and show confirmed choices.</x:t>
         </x:is>
       </x:c>
       <x:c r="F69" s="2" t="inlineStr">
@@ -18369,7 +18369,7 @@
       </x:c>
       <x:c r="I69" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">None</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.20.1</x:t>
         </x:is>
       </x:c>
       <x:c r="J69" s="2" t="inlineStr">
@@ -38778,7 +38778,7 @@
       </x:c>
       <x:c r="E32" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.20.1, REQ_IO_A5.20.2, REQ_IO_A5.20.3</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.20.1, REQ_IO_A5.20.2, REQ_IO_A5.20.3, REQ_IO_A5.18.3</x:t>
         </x:is>
       </x:c>
       <x:c r="F32" s="2" t="inlineStr">
@@ -38815,7 +38815,7 @@
       </x:c>
       <x:c r="E33" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">REQ_IO_A5.20.1, REQ_IO_A5.20.2, REQ_IO_A5.20.3, REQ_IO_A5.20.5</x:t>
+          <x:t xml:space="preserve">REQ_IO_A5.20.1, REQ_IO_A5.20.2, REQ_IO_A5.20.3, REQ_IO_A5.20.5, REQ_IO_A5.18.1</x:t>
         </x:is>
       </x:c>
       <x:c r="F33" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat(inv): add assembly draft documents and API
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Rdebf270c21a0499d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R7f2e97ad8e184ff7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R60fc5dea06d241e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R7d384b7f472b4a0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R25e15a9138f049c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="Rfb081bc19c8a4dea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Rfab82c7aed3b4af3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R24b00a24bb5c4436"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R64fa51673fcf409b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R12b68336667546dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Rb3b2aafa8e8b41b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R113bbdb0b98e44af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R57df170469c643ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R11a4bf4e0f7544df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R0fd52164ef124f03"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R855e4fc886fd4d22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R8750870858a94bbd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R2e5a60bcb04d4e39"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14682,6 +14682,102 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="71">
+      <x:c r="A71" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.154</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B71" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C71" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">inv_assembly</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D71" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">This table stores company-scoped assembly headers, draft state, approval state and posting time.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E71" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F71" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4115.4.1, REQ_F4115.4.2, REQ_F4115.4.3, REQ_F4115.4.4, REQ_F4115.4.5, REQ_F4115.4.6</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.155</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B72" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C72" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">inv_assembly_line</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D72" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">This table stores one finished item or component per assembly line and its posted unit cost.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E72" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F72" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4115.4.1, REQ_F4115.4.2, REQ_F4115.4.3, REQ_F4115.4.4</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.156</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B73" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C73" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">inv_assembly_line_tracking</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D73" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">This table stores the lot or serial quantities selected for each assembly line.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E73" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F73" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4115.4.1, REQ_F4115.4.2, REQ_F4115.4.3, REQ_F4115.4.4</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
   </x:sheetData>
 </x:worksheet>
 </file>
@@ -39337,7 +39433,7 @@
       </x:c>
       <x:c r="C19" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">REQ_DS43.154, REQ_DS43.155, REQ_DS43.156</x:t>
         </x:is>
       </x:c>
       <x:c r="D19" s="2" t="inlineStr">
@@ -39357,7 +39453,7 @@
       </x:c>
       <x:c r="G19" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Partial</x:t>
+          <x:t xml:space="preserve">Covered</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -39374,7 +39470,7 @@
       </x:c>
       <x:c r="C20" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">REQ_DS43.154, REQ_DS43.155, REQ_DS43.156</x:t>
         </x:is>
       </x:c>
       <x:c r="D20" s="2" t="inlineStr">
@@ -39394,7 +39490,7 @@
       </x:c>
       <x:c r="G20" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Partial</x:t>
+          <x:t xml:space="preserve">Covered</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -39411,7 +39507,7 @@
       </x:c>
       <x:c r="C21" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">REQ_DS43.154, REQ_DS43.155, REQ_DS43.156</x:t>
         </x:is>
       </x:c>
       <x:c r="D21" s="2" t="inlineStr">
@@ -39431,7 +39527,7 @@
       </x:c>
       <x:c r="G21" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Partial</x:t>
+          <x:t xml:space="preserve">Covered</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -39448,7 +39544,7 @@
       </x:c>
       <x:c r="C22" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">REQ_DS43.154, REQ_DS43.155, REQ_DS43.156</x:t>
         </x:is>
       </x:c>
       <x:c r="D22" s="2" t="inlineStr">
@@ -39468,7 +39564,7 @@
       </x:c>
       <x:c r="G22" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Partial</x:t>
+          <x:t xml:space="preserve">Covered</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -39485,19 +39581,19 @@
       </x:c>
       <x:c r="C23" s="2" t="inlineStr">
         <x:is>
+          <x:t xml:space="preserve">REQ_DS43.154</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D23" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">4.4.1.5.9</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E23" s="2" t="inlineStr">
+        <x:is>
           <x:t xml:space="preserve"/>
         </x:is>
       </x:c>
-      <x:c r="D23" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">4.4.1.5.9</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E23" s="2" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve"/>
-        </x:is>
-      </x:c>
       <x:c r="F23" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">INV-ASM-008</x:t>
@@ -39505,7 +39601,7 @@
       </x:c>
       <x:c r="G23" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Partial</x:t>
+          <x:t xml:space="preserve">Covered</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -39522,7 +39618,7 @@
       </x:c>
       <x:c r="C24" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">REQ_DS43.154</x:t>
         </x:is>
       </x:c>
       <x:c r="D24" s="2" t="inlineStr">
@@ -39542,7 +39638,7 @@
       </x:c>
       <x:c r="G24" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Partial</x:t>
+          <x:t xml:space="preserve">Covered</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
feat(inv): serialize assembly valuation with stock posting
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R12b68336667546dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Rb3b2aafa8e8b41b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R113bbdb0b98e44af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R57df170469c643ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R11a4bf4e0f7544df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R0fd52164ef124f03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R855e4fc886fd4d22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R8750870858a94bbd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R2e5a60bcb04d4e39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Rbe3d4972d69544df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R4d0ac98a735c4610"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R19098a1e0d104ea0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R38a77dc23e20429e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R2d37137544934bce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="Rb7c6ce612b024fd9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Rfe2c39ffa250454f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R51c9d14833fc421e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R1704c7ddb7c643dd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -39559,7 +39559,7 @@
       </x:c>
       <x:c r="F22" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">INV-ASM-001, INV-ASM-003, INV-ASM-004, INV-ASM-005, INV-ASM-006, INV-ASM-007, INV-ASM-012, INV-ASM-013, INV-ASM-015, INV-ASM-016</x:t>
+          <x:t xml:space="preserve">INV-ASM-001, INV-ASM-003, INV-ASM-004, INV-ASM-005, INV-ASM-006, INV-ASM-017, INV-ASM-007, INV-ASM-012, INV-ASM-013, INV-ASM-015, INV-ASM-016</x:t>
         </x:is>
       </x:c>
       <x:c r="G22" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat(inv): post assemblies atomically after approval
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Rbe3d4972d69544df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R4d0ac98a735c4610"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R19098a1e0d104ea0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R38a77dc23e20429e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R2d37137544934bce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="Rb7c6ce612b024fd9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Rfe2c39ffa250454f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R51c9d14833fc421e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R1704c7ddb7c643dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R3d75fc026841433b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R3f2bd73e10b04d39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R74880963439a4a1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R09189d5276794795"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R0fd5349ece7344c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="Rb16304d5e8a84325"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Rd44a6ed9fbd84040"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R80a9d386a4204154"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rea10288d40bb4d95"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
feat(inv): advance assembly UI and QA coverage
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R3d75fc026841433b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R3f2bd73e10b04d39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R74880963439a4a1f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R09189d5276794795"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R0fd5349ece7344c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="Rb16304d5e8a84325"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Rd44a6ed9fbd84040"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R80a9d386a4204154"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rea10288d40bb4d95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R0c8e0f782c5644c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R9d503446a13c4315"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Rc3652a4d2ef14ab2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R43eee392248d47e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R08573ee750d74fbe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R66549fae62dc47d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R4d59ce39a96743cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R081c817a3910415d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Re1bf9eab388c4565"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
feat(inv): page safety stock code sorting in bounded batches
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R3fb72c74c4394de6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R2e3d9858d7ae49c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R53ff6673d2b6481d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R61f3da086a814794"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Rff09919c71ac48b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R8952ece21eee4e5b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R8a2a7cf0c287428c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="Ra3187ece1cb147c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R0925741ec9984246"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R3b4ba09842a84e44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R4e66de647c3b4b4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R20f1311650294af5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Rcd121fc935274d33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Re95be6e089ec4aad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R2ef0549087294a7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R41da3b9d1417488d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="Rfec77de12bad41d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R929fefe7931e465b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -41690,7 +41690,7 @@
       </x:c>
       <x:c r="F63" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">INV-SAF-001, INV-SAF-002, INV-SAF-006, INV-SAF-008, INV-SAF-009, INV-SAF-011, INV-SAF-012</x:t>
+          <x:t xml:space="preserve">INV-SAF-001, INV-SAF-002, INV-SAF-006, INV-SAF-008, INV-SAF-009, INV-SAF-011, INV-SAF-012, INV-SAF-015</x:t>
         </x:is>
       </x:c>
       <x:c r="G63" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat(inv): complete safety stock page and QA
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R3b4ba09842a84e44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R4e66de647c3b4b4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R20f1311650294af5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Rcd121fc935274d33"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Re95be6e089ec4aad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R2ef0549087294a7d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R41da3b9d1417488d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="Rfec77de12bad41d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R929fefe7931e465b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R21136dc9428946b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R1cc7967100cb47da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Rc8defcaf88264959"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R989be564daff403e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R4340b3e1bacf42cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="Redf7a5538dc149d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R1dab84dbfdba41a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R4c42f5f85ea241fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R38ce451c81e94d42"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
feat(inv): add snapshot stock flow report API
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R98a18376ca7e4659"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Ra70306de3b11466b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R968c93af517d4820"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R29b14d1597c6431a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R3de28c0429cd4dab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="Rf3a99bed962e4cac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Rffc39fb663e54038"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R12957892f8534ec5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rc4e2b99d72244377"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Rc778a295002a46f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R47e35ece6d654e85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Rb69b42f0cf784c5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Re59ce848723c4cb0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R4e50d60c9c3249e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R02ae3484d8f840b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Rfc186e4f0b14400c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R048e0c2c635a4ad7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R6a1269fcf8284ce7"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
feat(inv): add stock flow report CSV export and page
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Rc778a295002a46f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R47e35ece6d654e85"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Rb69b42f0cf784c5c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Re59ce848723c4cb0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R4e50d60c9c3249e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R02ae3484d8f840b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Rfc186e4f0b14400c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R048e0c2c635a4ad7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R6a1269fcf8284ce7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R4705940fbfe54b33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Rb0d92c4e1fe54a3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R7fb2d57680c54e84"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R78a8997f99f34918"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Rd7573894d3d845ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="Rc106489ba2c14d1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R3ff230fb89854c70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="Rb570f6d929b94b2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R16b1f54f242244c9"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
feat(inv): export complete lot and serial histories
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R4705940fbfe54b33"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Rb0d92c4e1fe54a3f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R7fb2d57680c54e84"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R78a8997f99f34918"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Rd7573894d3d845ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="Rc106489ba2c14d1f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R3ff230fb89854c70"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="Rb570f6d929b94b2e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R16b1f54f242244c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Re18b323a72e74190"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R0bf26ee14b5f4671"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R27b5cdbaf97641b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Rbef1a337efc7437c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Rde149036efca4c16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="Rd43a962b6f3a4ec8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Ra922681e75304613"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R0b263ea61084457c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rd4ae52cd93a7446e"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
feat(inv): add disassembly draft backend
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R72821c31ef844549"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R77cfef1156ab4e94"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R79f8e2408e48427a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R816d7bc0824042c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R03a1ea5be0074f9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R8831b3d029b44255"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Rfbb6c4054dfb41a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R649ae005d68446cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R4e0c8745bdd14e98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R7e26d6f3b45c4fbd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R6222dbb9a09348f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R15d1c2d4d156497c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R762f900f901a4aec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Rd14cc08c16fc4d06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R72ec69f1a5824da2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R81a1d55e86be4272"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="Racd4443d4ae34820"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rf9abf10701924e17"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15314,6 +15314,102 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="75">
+      <x:c r="A75" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.158</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B75" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C75" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">inv_disassembly</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D75" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">This table stores company-scoped disassembly headers, document status and posting time.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E75" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F75" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4115.5.1, REQ_F4115.5.2, REQ_F4115.5.3, REQ_F4115.5.4, REQ_F4115.5.5, REQ_F4115.5.6</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="76">
+      <x:c r="A76" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.159</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B76" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C76" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">inv_disassembly_line</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D76" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">This table stores the finished source and component destinations with allocation weight and posted unit cost.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E76" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F76" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4115.5.1, REQ_F4115.5.2, REQ_F4115.5.3, REQ_F4115.5.4</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.160</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B77" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C77" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">inv_disassembly_line_tracking</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D77" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">This table stores selected lot or serial quantities for each disassembly line.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E77" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F77" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4115.5.1, REQ_F4115.5.2, REQ_F4115.5.3, REQ_F4115.5.4</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
   </x:sheetData>
 </x:worksheet>
 </file>
@@ -41844,7 +41940,7 @@
       </x:c>
       <x:c r="C25" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">REQ_DS43.158, REQ_DS43.159, REQ_DS43.160</x:t>
         </x:is>
       </x:c>
       <x:c r="D25" s="2" t="inlineStr">
@@ -41864,7 +41960,7 @@
       </x:c>
       <x:c r="G25" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Partial</x:t>
+          <x:t xml:space="preserve">Covered</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -41881,7 +41977,7 @@
       </x:c>
       <x:c r="C26" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">REQ_DS43.158, REQ_DS43.159, REQ_DS43.160</x:t>
         </x:is>
       </x:c>
       <x:c r="D26" s="2" t="inlineStr">
@@ -41901,7 +41997,7 @@
       </x:c>
       <x:c r="G26" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Partial</x:t>
+          <x:t xml:space="preserve">Covered</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -41918,7 +42014,7 @@
       </x:c>
       <x:c r="C27" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">REQ_DS43.158, REQ_DS43.159, REQ_DS43.160</x:t>
         </x:is>
       </x:c>
       <x:c r="D27" s="2" t="inlineStr">
@@ -41938,7 +42034,7 @@
       </x:c>
       <x:c r="G27" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Partial</x:t>
+          <x:t xml:space="preserve">Covered</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -41955,7 +42051,7 @@
       </x:c>
       <x:c r="C28" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">REQ_DS43.158, REQ_DS43.159, REQ_DS43.160</x:t>
         </x:is>
       </x:c>
       <x:c r="D28" s="2" t="inlineStr">
@@ -41975,7 +42071,7 @@
       </x:c>
       <x:c r="G28" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Partial</x:t>
+          <x:t xml:space="preserve">Covered</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -41992,7 +42088,7 @@
       </x:c>
       <x:c r="C29" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">REQ_DS43.158</x:t>
         </x:is>
       </x:c>
       <x:c r="D29" s="2" t="inlineStr">
@@ -42012,7 +42108,7 @@
       </x:c>
       <x:c r="G29" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Partial</x:t>
+          <x:t xml:space="preserve">Covered</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -42029,7 +42125,7 @@
       </x:c>
       <x:c r="C30" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">REQ_DS43.158</x:t>
         </x:is>
       </x:c>
       <x:c r="D30" s="2" t="inlineStr">
@@ -42049,7 +42145,7 @@
       </x:c>
       <x:c r="G30" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Partial</x:t>
+          <x:t xml:space="preserve">Covered</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
feat(inv): post disassemblies through approval workflow
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R7e26d6f3b45c4fbd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R6222dbb9a09348f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R15d1c2d4d156497c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R762f900f901a4aec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Rd14cc08c16fc4d06"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R72ec69f1a5824da2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R81a1d55e86be4272"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="Racd4443d4ae34820"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rf9abf10701924e17"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Rae56d276857a4316"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Rd926ed535f1042d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Ra5bf0e16927a4494"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R937c79b9c38749fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R2eefbe2ced7741e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R4c1bde69b3ca4724"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R503f8142eedf4627"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R862907b4fde94645"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rb4fd645a68e94a5d"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
feat(inv): complete disassembly frontend and QA
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Rae56d276857a4316"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Rd926ed535f1042d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Ra5bf0e16927a4494"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R937c79b9c38749fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R2eefbe2ced7741e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R4c1bde69b3ca4724"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R503f8142eedf4627"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R862907b4fde94645"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rb4fd645a68e94a5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Ra65c4cd333654126"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Rfe168a9c7a454748"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R28b0faebc65a450b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R4451f78453a1439f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R635e68635f1d4145"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R3df9ff83123a46e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Rba6781003b9346c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="Ra15846770e404fba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R8f529573e4bb4b71"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
test(inv): cover disassembly boundary and reference states
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Ra65c4cd333654126"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Rfe168a9c7a454748"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R28b0faebc65a450b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R4451f78453a1439f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R635e68635f1d4145"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R3df9ff83123a46e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Rba6781003b9346c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="Ra15846770e404fba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R8f529573e4bb4b71"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Rd3393dd5f49648be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R8345de0a651b4d43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R3ee2a7d5f8d346cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R92263cdb2faf47e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Rb5efab9b3df54a4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R90472f1cd0194365"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R4c5a593ff7444d6e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R68ed3af71c724606"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Re8376b46c9df42ba"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
test(inv): verify disassembly approval rollback and cost locking
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Rd3393dd5f49648be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R8345de0a651b4d43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R3ee2a7d5f8d346cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R92263cdb2faf47e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Rb5efab9b3df54a4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R90472f1cd0194365"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R4c5a593ff7444d6e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R68ed3af71c724606"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Re8376b46c9df42ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R28169ba497de45ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Re39d1bdd980a47c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R20c9bef2a5864707"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Rca1bf6ff682c40df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R2802605cbf724c6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R0ccf0f735c7b4ca5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R6a6766f17c7c4cee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="Rb27c3c79820d4a04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rc69e616964ba49f5"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
feat(pur): add requisition draft schema
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Re23effd8522346bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R1106ae4445474d23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R8247573efcf84753"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R031041a7a6ac4442"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R03cfc23a25044786"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R911ae3c63db04029"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R1d71b3a8c39442dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R84968d81f8ab4ab1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R7a04469c0c284a32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R7f799eefc0be4f96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R0ffd33c22aed4771"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Rb73272d8fdea4df3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R129397effb2e4ae2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R52b4f39cb83b4e1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R6a5577dffbaf4470"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R0ff618c786d34941"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R73af4a21910a40ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rf196e8286c5a4c5c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -277,7 +277,7 @@
       </x:c>
       <x:c r="H5" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/02-modules/PUR/requirements.md:13</x:t>
+          <x:t xml:space="preserve">docs/02-modules/PUR/requirements.md:15</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -319,7 +319,7 @@
       </x:c>
       <x:c r="H6" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/02-modules/PUR/requirements.md:14</x:t>
+          <x:t xml:space="preserve">docs/02-modules/PUR/requirements.md:16</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -361,7 +361,7 @@
       </x:c>
       <x:c r="H7" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/02-modules/PUR/requirements.md:15</x:t>
+          <x:t xml:space="preserve">docs/02-modules/PUR/requirements.md:17</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -403,7 +403,7 @@
       </x:c>
       <x:c r="H8" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/02-modules/PUR/requirements.md:16</x:t>
+          <x:t xml:space="preserve">docs/02-modules/PUR/requirements.md:18</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -445,7 +445,7 @@
       </x:c>
       <x:c r="H9" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/02-modules/PUR/requirements.md:17</x:t>
+          <x:t xml:space="preserve">docs/02-modules/PUR/requirements.md:19</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -487,7 +487,7 @@
       </x:c>
       <x:c r="H10" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">docs/02-modules/PUR/requirements.md:18</x:t>
+          <x:t xml:space="preserve">docs/02-modules/PUR/requirements.md:20</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -15659,6 +15659,70 @@
       <x:c r="F77" s="2" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">REQ_F4115.5.1, REQ_F4115.5.2, REQ_F4115.5.3, REQ_F4115.5.4</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="78">
+      <x:c r="A78" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.161</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B78" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C78" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">pur_requisition</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D78" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">This table stores company-scoped purchase requisition headers, document numbers and approval state.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E78" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F78" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4114.3.1, REQ_F4114.3.2, REQ_F4114.3.3, REQ_F4114.3.4, REQ_F4114.3.5, REQ_F4114.3.6</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="79">
+      <x:c r="A79" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_DS43.162</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B79" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">1.0</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C79" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">pur_requisition_line</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D79" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">This table stores ordered item demand, required dates, quantities and downstream order consumption.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E79" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Developer</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F79" s="2" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">REQ_F4114.3.1, REQ_F4114.3.2, REQ_F4114.3.3, REQ_F4114.3.4</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -41965,7 +42029,7 @@
       </x:c>
       <x:c r="C5" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">REQ_DS43.161, REQ_DS43.162</x:t>
         </x:is>
       </x:c>
       <x:c r="D5" s="2" t="inlineStr">
@@ -41985,7 +42049,7 @@
       </x:c>
       <x:c r="G5" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Partial</x:t>
+          <x:t xml:space="preserve">Covered</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -42002,7 +42066,7 @@
       </x:c>
       <x:c r="C6" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">REQ_DS43.161, REQ_DS43.162</x:t>
         </x:is>
       </x:c>
       <x:c r="D6" s="2" t="inlineStr">
@@ -42022,7 +42086,7 @@
       </x:c>
       <x:c r="G6" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Partial</x:t>
+          <x:t xml:space="preserve">Covered</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -42039,7 +42103,7 @@
       </x:c>
       <x:c r="C7" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">REQ_DS43.161, REQ_DS43.162</x:t>
         </x:is>
       </x:c>
       <x:c r="D7" s="2" t="inlineStr">
@@ -42059,7 +42123,7 @@
       </x:c>
       <x:c r="G7" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Partial</x:t>
+          <x:t xml:space="preserve">Covered</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -42076,7 +42140,7 @@
       </x:c>
       <x:c r="C8" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">REQ_DS43.161, REQ_DS43.162</x:t>
         </x:is>
       </x:c>
       <x:c r="D8" s="2" t="inlineStr">
@@ -42096,7 +42160,7 @@
       </x:c>
       <x:c r="G8" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Partial</x:t>
+          <x:t xml:space="preserve">Covered</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -42113,7 +42177,7 @@
       </x:c>
       <x:c r="C9" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">REQ_DS43.161</x:t>
         </x:is>
       </x:c>
       <x:c r="D9" s="2" t="inlineStr">
@@ -42133,7 +42197,7 @@
       </x:c>
       <x:c r="G9" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Partial</x:t>
+          <x:t xml:space="preserve">Covered</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -42150,7 +42214,7 @@
       </x:c>
       <x:c r="C10" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve"/>
+          <x:t xml:space="preserve">REQ_DS43.161</x:t>
         </x:is>
       </x:c>
       <x:c r="D10" s="2" t="inlineStr">
@@ -42170,7 +42234,7 @@
       </x:c>
       <x:c r="G10" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Partial</x:t>
+          <x:t xml:space="preserve">Covered</x:t>
         </x:is>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
feat(pur): enforce requisition read data scope
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R7f799eefc0be4f96"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R0ffd33c22aed4771"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Rb73272d8fdea4df3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R129397effb2e4ae2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R52b4f39cb83b4e1f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R6a5577dffbaf4470"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R0ff618c786d34941"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R73af4a21910a40ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rf196e8286c5a4c5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Re01b347a8d564baf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R89e17f0207994e2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R2fa111ebb8c240a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Rc1d1e60297fe4495"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R34ed93c531be47a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R7691071d209c4901"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R192c9a9b19504c8e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R3612c22ed0c14609"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rb9148229952c4b80"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -257,7 +257,7 @@
       </x:c>
       <x:c r="D5" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">1.0</x:t>
+          <x:t xml:space="preserve">1.1</x:t>
         </x:is>
       </x:c>
       <x:c r="E5" s="2" t="inlineStr">
@@ -272,7 +272,7 @@
       </x:c>
       <x:c r="G5" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">PUR.REQUISITION.VIEW 僅列目前公司；依單號、業務日期、狀態、請購人穩定分頁；詳情呈現保存行、版本、SYS 審批歷史與可轉採購餘量；他公司 ID 回 404。</x:t>
+          <x:t xml:space="preserve">PUR.REQUISITION.VIEW 僅列目前公司及 SYS 授權的本人／部門／分店／全公司範圍；依單號、業務日期、狀態、請購人穩定分頁；詳情呈現保存行、版本、SYS 審批歷史與可轉採購餘量；範圍外及他公司 ID 回 404。</x:t>
         </x:is>
       </x:c>
       <x:c r="H5" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat(pur): create requisition drafts with authorized ownership
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Re01b347a8d564baf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R89e17f0207994e2e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R2fa111ebb8c240a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Rc1d1e60297fe4495"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R34ed93c531be47a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R7691071d209c4901"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R192c9a9b19504c8e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R3612c22ed0c14609"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rb9148229952c4b80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Rce02c398dfdf4330"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Rfc0b032ae9c74b6d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R916a57e08d1743c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R3a80c78023ff45cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R8ae76c3dead94184"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R610db36f2fae4bf7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R6c6a733dae9e48b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R1432d8c903a0464b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R4ed4599b74484bb4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -299,7 +299,7 @@
       </x:c>
       <x:c r="D6" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">1.0</x:t>
+          <x:t xml:space="preserve">1.1</x:t>
         </x:is>
       </x:c>
       <x:c r="E6" s="2" t="inlineStr">
@@ -314,7 +314,7 @@
       </x:c>
       <x:c r="G6" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">PUR.REQUISITION.CREATE 建立草稿並取 SYS 公司單號；1–1000 行、物料與基本單位正數六位數量、需求日期不得早於單據日；只驗本公司有效 MD 引用，不寫 INV 異動或預留庫存。</x:t>
+          <x:t xml:space="preserve">PUR.REQUISITION.CREATE 建立草稿並取 SYS 公司單號；1–1000 行、物料與基本單位正數六位數量、需求日期不得早於單據日；只驗本公司有效 MD 引用，不寫 INV 異動或預留庫存。請購人、分店、部門從 SYS 目前授權取得。</x:t>
         </x:is>
       </x:c>
       <x:c r="H6" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat(pur): add scoped requisition update and soft delete
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Rce02c398dfdf4330"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Rfc0b032ae9c74b6d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R916a57e08d1743c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R3a80c78023ff45cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R8ae76c3dead94184"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R610db36f2fae4bf7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R6c6a733dae9e48b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R1432d8c903a0464b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R4ed4599b74484bb4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Rba77f3aaa2c3403d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R990f0004cef84cfc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R652ffc32ca0946c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R668949a5f7d0409b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R9f930c8039334e94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R13b6ee487c144d7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R68242b436bc64a96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R77eae648116e4c01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R64f0f4a7bdbe416f"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
feat(pur): add requisition submission workflow
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="Rba77f3aaa2c3403d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R990f0004cef84cfc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R652ffc32ca0946c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R668949a5f7d0409b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R9f930c8039334e94"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R13b6ee487c144d7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R68242b436bc64a96"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R77eae648116e4c01"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R64f0f4a7bdbe416f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R2a1f29a6c8d64b8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Rdbfd46686d9f4c8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R44c1ad9b40834bc5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R981fd17347794e06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Rf81e28ff27ea40c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R3d94c49b7df64368"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Ra13109290a3845d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="Rb70d150dc54449de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R7477e9f6687f42cd"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
test(pur): verify requisition approval boundaries and races
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R2a1f29a6c8d64b8c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="Rdbfd46686d9f4c8c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R44c1ad9b40834bc5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R981fd17347794e06"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="Rf81e28ff27ea40c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R3d94c49b7df64368"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Ra13109290a3845d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="Rb70d150dc54449de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R7477e9f6687f42cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R05c0f3a338464dcd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R4df07870c93e4755"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Ra5669a630af04ea9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Raac83d475c1843cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R28210ec154ca4316"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R4d7a5bea701c4775"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Ra6b38cb9cc49429d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R7cd13962a64e422a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R78b698ff0b2448ae"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
feat(pur): add requisition frontend API contract
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R05c0f3a338464dcd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R4df07870c93e4755"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Ra5669a630af04ea9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Raac83d475c1843cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R28210ec154ca4316"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R4d7a5bea701c4775"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="Ra6b38cb9cc49429d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="R7cd13962a64e422a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="R78b698ff0b2448ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R7aea68c605fd4992"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R889ad6f4e1544d5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R6b4fccdc257943d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Re269636073594b51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R547052d73b854f64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R4a30574fb6904242"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R8036465108784d9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="Rb2c8871af64f4341"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rd42aeadd76fc43dd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -16582,7 +16582,7 @@
       </x:c>
       <x:c r="H15" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Valid date; remark ≤ 1000</x:t>
+          <x:t xml:space="preserve">Valid date; remark ≤ 500</x:t>
         </x:is>
       </x:c>
       <x:c r="I15" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat(pur): complete requisition create and edit forms
</commit_message>
<xml_diff>
--- a/docs/99-output/MyERP_Requirements.xlsx
+++ b/docs/99-output/MyERP_Requirements.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R7aea68c605fd4992"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R889ad6f4e1544d5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="R6b4fccdc257943d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="Re269636073594b51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R547052d73b854f64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R4a30574fb6904242"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R8036465108784d9b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="Rb2c8871af64f4341"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rd42aeadd76fc43dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Functional" sheetId="1" r:id="R7130e062753e404a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-Functional" sheetId="2" r:id="R6f0f5137f6ab469d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Structure" sheetId="3" r:id="Rb2d503bddd554375"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interface" sheetId="4" r:id="R7659504e0fc140e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Traceability Matrix" sheetId="5" r:id="R4011322bcf424aea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BlueWhale Parity" sheetId="6" r:id="R38afa47206954184"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="7" r:id="R66b9880b16684acf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human Resources" sheetId="8" r:id="Rb0ed87d9f94441ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="9" r:id="Rdaedc159a0e248a4"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>